<commit_message>
Pedidos sin enviar: usar el envío estándar en lugar de 0 €
El export del almacén trae el coste de envío a 0 hasta que el pedido sale, y eso
inflaba el beneficio proyectado de los días recientes (07/10: 32 € en vez de 13 €).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFjE4yx23BY3D6kaMQowKe
</commit_message>
<xml_diff>
--- a/contabilidad/CeraLux_Contabilidad.xlsx
+++ b/contabilidad/CeraLux_Contabilidad.xlsx
@@ -1835,16 +1835,16 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>56.5721652892561</c:v>
+                  <c:v>62.6280826446281</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>21.5064132231405</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>-28.9578016528926</c:v>
+                  <c:v>12.9661652892562</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0</c:v>
+                  <c:v>-2.73</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1852,8 +1852,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="54532552"/>
-        <c:axId val="6895685"/>
+        <c:axId val="12703388"/>
+        <c:axId val="77698927"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2007,7 +2007,7 @@
                   <c:v>47.41</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0</c:v>
+                  <c:v>2.73</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2022,11 +2022,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="54532552"/>
-        <c:axId val="6895685"/>
+        <c:axId val="12703388"/>
+        <c:axId val="77698927"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="54532552"/>
+        <c:axId val="12703388"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2058,7 +2058,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6895685"/>
+        <c:crossAx val="77698927"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2066,7 +2066,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="6895685"/>
+        <c:axId val="77698927"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2108,7 +2108,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="54532552"/>
+        <c:crossAx val="12703388"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2307,7 +2307,7 @@
                 <c:formatCode>#,##0" €";[RED]\-#,##0" €";\-</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>49.1207768595041</c:v>
+                  <c:v>94.3706611570248</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -2348,8 +2348,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="84115311"/>
-        <c:axId val="62576645"/>
+        <c:axId val="9173522"/>
+        <c:axId val="77168686"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2446,11 +2446,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="84115311"/>
-        <c:axId val="62576645"/>
+        <c:axId val="9173522"/>
+        <c:axId val="77168686"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="84115311"/>
+        <c:axId val="9173522"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2482,7 +2482,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="62576645"/>
+        <c:crossAx val="77168686"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2490,7 +2490,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="62576645"/>
+        <c:axId val="77168686"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2532,7 +2532,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="84115311"/>
+        <c:crossAx val="9173522"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2926,32 +2926,32 @@
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="10" t="n">
         <f aca="false">F25</f>
-        <v>49.1207768595042</v>
+        <v>94.3706611570248</v>
       </c>
       <c r="C7" s="10"/>
       <c r="D7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$T$6:$T$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>126.2547</v>
+        <v>154.5789</v>
       </c>
       <c r="E7" s="10"/>
       <c r="F7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$U$6:$U$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+F24</f>
-        <v>-107.09479338843</v>
+        <v>-91.4052066115703</v>
       </c>
       <c r="G7" s="10"/>
       <c r="H7" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$M$6:$M$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="I7" s="11"/>
       <c r="J7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$O$6:$O$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>619.81</v>
+        <v>749.77</v>
       </c>
       <c r="K7" s="10"/>
       <c r="L7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$K$6:$K$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>185.26</v>
+        <v>187.99</v>
       </c>
       <c r="M7" s="10"/>
     </row>
@@ -2984,32 +2984,32 @@
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="10" t="n">
         <f aca="false">IF(H7&gt;0,L7/H7,"")</f>
-        <v>9.75052631578947</v>
+        <v>8.17347826086957</v>
       </c>
       <c r="C10" s="10"/>
       <c r="D10" s="10" t="n">
         <f aca="false">CPA_BE</f>
-        <v>10.8139860809047</v>
+        <v>10.7560740208408</v>
       </c>
       <c r="E10" s="10"/>
       <c r="F10" s="12" t="n">
         <f aca="false">IF(L7&gt;0,J7/L7,"")</f>
-        <v>3.3456223685631</v>
+        <v>3.98835044417256</v>
       </c>
       <c r="G10" s="12"/>
       <c r="H10" s="12" t="n">
         <f aca="false">ROAS_BE</f>
-        <v>3.01661003660541</v>
+        <v>3.0307243692272</v>
       </c>
       <c r="I10" s="12"/>
       <c r="J10" s="10" t="n">
         <f aca="false">IF(H7&gt;0,J7/H7,"")</f>
-        <v>32.6215789473684</v>
+        <v>32.5986956521739</v>
       </c>
       <c r="K10" s="10"/>
       <c r="L10" s="13" t="n">
         <f aca="false">IF(H7&gt;0,SUMIFS(Diario!$C$6:$C$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)/H7,"")</f>
-        <v>0.263157894736842</v>
+        <v>0.260869565217391</v>
       </c>
       <c r="M10" s="13"/>
     </row>
@@ -3042,12 +3042,12 @@
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$D$6:$D$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C13" s="11"/>
       <c r="D13" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E13" s="11"/>
       <c r="F13" s="11" t="n">
@@ -3099,7 +3099,7 @@
       </c>
       <c r="F16" s="17" t="n">
         <f aca="false">SUMIFS(Diario!$AC$6:$AC$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>533.836</v>
+        <v>645.802</v>
       </c>
       <c r="H16" s="15" t="s">
         <v>29</v>
@@ -3121,11 +3121,11 @@
       <c r="D17" s="15"/>
       <c r="E17" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F17/$F$16,"")</f>
-        <v>-0.0929175626971579</v>
+        <v>-0.0932135546189079</v>
       </c>
       <c r="F17" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AD$6:$AD$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-49.60274</v>
+        <v>-60.1975</v>
       </c>
       <c r="H17" s="15" t="s">
         <v>31</v>
@@ -3135,7 +3135,7 @@
       <c r="K17" s="15"/>
       <c r="L17" s="20" t="n">
         <f aca="false">F25/I3</f>
-        <v>6.14009710743802</v>
+        <v>11.7963326446281</v>
       </c>
       <c r="M17" s="20"/>
     </row>
@@ -3147,11 +3147,11 @@
       <c r="D18" s="15"/>
       <c r="E18" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F18/$F$16,"")</f>
-        <v>-0.237537371027806</v>
+        <v>-0.238413631422634</v>
       </c>
       <c r="F18" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AE$6:$AE$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-126.806</v>
+        <v>-153.968</v>
       </c>
       <c r="H18" s="15" t="s">
         <v>33</v>
@@ -3161,7 +3161,7 @@
       <c r="K18" s="15"/>
       <c r="L18" s="18" t="n">
         <f aca="false">L17*30</f>
-        <v>184.202913223141</v>
+        <v>353.889979338843</v>
       </c>
       <c r="M18" s="18"/>
     </row>
@@ -3173,11 +3173,11 @@
       <c r="D19" s="15"/>
       <c r="E19" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F19/$F$16,"")</f>
-        <v>-0.0392555016896575</v>
+        <v>-0.0399379376341355</v>
       </c>
       <c r="F19" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AF$6:$AF$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-20.956</v>
+        <v>-25.792</v>
       </c>
       <c r="H19" s="21" t="s">
         <v>35</v>
@@ -3187,7 +3187,7 @@
       <c r="K19" s="21"/>
       <c r="L19" s="22" t="n">
         <f aca="false">IF(L16&gt;0,L18/L16,"")</f>
-        <v>0.0184202913223141</v>
+        <v>0.0353889979338843</v>
       </c>
       <c r="M19" s="22"/>
     </row>
@@ -3199,11 +3199,11 @@
       <c r="D20" s="15"/>
       <c r="E20" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F20/$F$16,"")</f>
-        <v>-0.0338118823009314</v>
+        <v>-0.0338338995543526</v>
       </c>
       <c r="F20" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AJ$6:$AJ$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-18.05</v>
+        <v>-21.85</v>
       </c>
       <c r="H20" s="15" t="s">
         <v>37</v>
@@ -3213,7 +3213,7 @@
       <c r="K20" s="15"/>
       <c r="L20" s="20" t="n">
         <f aca="false">BEN_PEDIDO</f>
-        <v>10.8139860809047</v>
+        <v>10.7560740208408</v>
       </c>
       <c r="M20" s="20"/>
     </row>
@@ -3225,11 +3225,11 @@
       <c r="D21" s="15"/>
       <c r="E21" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F21/$F$16,"")</f>
-        <v>-0.157427530440989</v>
+        <v>-0.157376159942173</v>
       </c>
       <c r="F21" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AG$6:$AG$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-84.0404831404959</v>
+        <v>-101.633838842975</v>
       </c>
       <c r="H21" s="15" t="s">
         <v>39</v>
@@ -3239,7 +3239,7 @@
       <c r="K21" s="15"/>
       <c r="L21" s="20" t="n">
         <f aca="false">B10</f>
-        <v>9.75052631578947</v>
+        <v>8.17347826086957</v>
       </c>
       <c r="M21" s="20"/>
     </row>
@@ -3251,11 +3251,11 @@
       <c r="D22" s="15"/>
       <c r="E22" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F22/$F$16,"")</f>
-        <v>-0.347035419117482</v>
+        <v>-0.291095413145206</v>
       </c>
       <c r="F22" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AH$6:$AH$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-185.26</v>
+        <v>-187.99</v>
       </c>
       <c r="H22" s="15" t="s">
         <v>41</v>
@@ -3265,7 +3265,7 @@
       <c r="K22" s="15"/>
       <c r="L22" s="20" t="n">
         <f aca="false">IF(ISNUMBER(L21),L20-L21*(1+RECARGO_ADS),"")</f>
-        <v>1.06345976511527</v>
+        <v>2.58259575997125</v>
       </c>
       <c r="M22" s="20"/>
     </row>
@@ -3277,11 +3277,11 @@
       <c r="D23" s="23"/>
       <c r="E23" s="24" t="n">
         <f aca="false">IF($F$16&gt;0,F23/$F$16,"")</f>
-        <v>0.0920147327259761</v>
+        <v>0.146129403682591</v>
       </c>
       <c r="F23" s="25" t="n">
         <f aca="false">SUM(F16:F22)</f>
-        <v>49.1207768595042</v>
+        <v>94.3706611570248</v>
       </c>
       <c r="H23" s="21" t="s">
         <v>43</v>
@@ -3291,7 +3291,7 @@
       <c r="K23" s="21"/>
       <c r="L23" s="26" t="n">
         <f aca="false">IF(NOT(ISNUMBER(L22)),"",IF(L22&lt;=0,"Baja el CPA",ROUNDUP((L16-F24/I3*30)/30/L22,0)))</f>
-        <v>314</v>
+        <v>130</v>
       </c>
       <c r="M23" s="26"/>
     </row>
@@ -3317,7 +3317,7 @@
       <c r="K24" s="15"/>
       <c r="L24" s="18" t="n">
         <f aca="false">IF(ISNUMBER(L23),L23*L21,"")</f>
-        <v>3061.66526315789</v>
+        <v>1062.55217391304</v>
       </c>
       <c r="M24" s="18"/>
     </row>
@@ -3329,11 +3329,11 @@
       <c r="D25" s="23"/>
       <c r="E25" s="24" t="n">
         <f aca="false">IF($F$16&gt;0,F25/$F$16,"")</f>
-        <v>0.0920147327259761</v>
+        <v>0.146129403682591</v>
       </c>
       <c r="F25" s="25" t="n">
         <f aca="false">F23+F24</f>
-        <v>49.1207768595042</v>
+        <v>94.3706611570248</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3344,7 +3344,7 @@
       <c r="D26" s="27"/>
       <c r="F26" s="28" t="n">
         <f aca="false">IF(F16&gt;0,F25/F16,"")</f>
-        <v>0.0920147327259761</v>
+        <v>0.146129403682591</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3656,7 +3656,7 @@
       </c>
       <c r="F39" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$V$6:$V$370,Diario!$A$6:$A$370,$B39)</f>
-        <v>56.5721652892561</v>
+        <v>62.6280826446281</v>
       </c>
       <c r="G39" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$D$6:$D$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B39))&gt;0,(SUMIFS(Diario!$D$6:$D$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B39))/(SUMIFS(Diario!$D$6:$D$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B39)),"")</f>
@@ -3696,7 +3696,7 @@
       </c>
       <c r="C41" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$M$6:$M$370,Diario!$A$6:$A$370,$B41)</f>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D41" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$K$6:$K$370,Diario!$A$6:$A$370,$B41)</f>
@@ -3704,11 +3704,11 @@
       </c>
       <c r="E41" s="32" t="n">
         <f aca="false">IF(C41&gt;0,D41/C41,"")</f>
-        <v>23.705</v>
+        <v>7.90166666666667</v>
       </c>
       <c r="F41" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$V$6:$V$370,Diario!$A$6:$A$370,$B41)</f>
-        <v>-28.9578016528926</v>
+        <v>12.9661652892562</v>
       </c>
       <c r="G41" s="34" t="str">
         <f aca="false">IF((SUMIFS(Diario!$D$6:$D$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B41))&gt;0,(SUMIFS(Diario!$D$6:$D$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B41))/(SUMIFS(Diario!$D$6:$D$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B41)),"")</f>
@@ -3726,7 +3726,7 @@
       </c>
       <c r="D42" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$K$6:$K$370,Diario!$A$6:$A$370,$B42)</f>
-        <v>0</v>
+        <v>2.73</v>
       </c>
       <c r="E42" s="32" t="str">
         <f aca="false">IF(C42&gt;0,D42/C42,"")</f>
@@ -3734,7 +3734,7 @@
       </c>
       <c r="F42" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$V$6:$V$370,Diario!$A$6:$A$370,$B42)</f>
-        <v>0</v>
+        <v>-2.73</v>
       </c>
       <c r="G42" s="34" t="str">
         <f aca="false">IF((SUMIFS(Diario!$D$6:$D$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B42))&gt;0,(SUMIFS(Diario!$D$6:$D$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B42))/(SUMIFS(Diario!$D$6:$D$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B42)),"")</f>
@@ -3805,23 +3805,23 @@
       </c>
       <c r="C47" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$M$6:$M$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D47" s="37" t="n">
         <f aca="false">SUMIFS(Diario!$K$6:$K$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>185.26</v>
+        <v>187.99</v>
       </c>
       <c r="E47" s="32" t="n">
         <f aca="false">IF(C47&gt;0,D47/C47,"")</f>
-        <v>9.75052631578947</v>
+        <v>8.17347826086957</v>
       </c>
       <c r="F47" s="37" t="n">
         <f aca="false">SUMIFS(Diario!$O$6:$O$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>619.81</v>
+        <v>749.77</v>
       </c>
       <c r="G47" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$D$6:$D$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))+SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H47" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
@@ -3833,7 +3833,7 @@
       </c>
       <c r="J47" s="37" t="n">
         <f aca="false">SUMIFS(Diario!$V$6:$V$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>49.1207768595041</v>
+        <v>94.3706611570248</v>
       </c>
       <c r="K47" s="37" t="n">
         <f aca="false">-SUMIFS(Gastos!$D$5:$D$304,Gastos!$A$5:$A$304,"&gt;="&amp;$B47,Gastos!$A$5:$A$304,"&lt;="&amp;EOMONTH($B47,0))</f>
@@ -3841,11 +3841,11 @@
       </c>
       <c r="L47" s="38" t="n">
         <f aca="false">J47+K47</f>
-        <v>49.1207768595041</v>
+        <v>94.3706611570248</v>
       </c>
       <c r="M47" s="34" t="n">
         <f aca="false">IF(OBJETIVO_MES&gt;0,L47/OBJETIVO_MES,"")</f>
-        <v>0.00491207768595041</v>
+        <v>0.00943706611570248</v>
       </c>
       <c r="O47" s="39" t="n">
         <f aca="false">OBJETIVO_MES</f>
@@ -4452,23 +4452,23 @@
       </c>
       <c r="C59" s="41" t="n">
         <f aca="false">SUM(C47:C58)</f>
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D59" s="42" t="n">
         <f aca="false">SUM(D47:D58)</f>
-        <v>185.26</v>
+        <v>187.99</v>
       </c>
       <c r="E59" s="43" t="n">
         <f aca="false">IF(C59&gt;0,D59/C59,"")</f>
-        <v>9.75052631578947</v>
+        <v>8.17347826086957</v>
       </c>
       <c r="F59" s="42" t="n">
         <f aca="false">SUM(F47:F58)</f>
-        <v>619.81</v>
+        <v>749.77</v>
       </c>
       <c r="G59" s="41" t="n">
         <f aca="false">SUM(G47:G58)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H59" s="41" t="n">
         <f aca="false">SUM(H47:H58)</f>
@@ -4480,7 +4480,7 @@
       </c>
       <c r="J59" s="42" t="n">
         <f aca="false">SUM(J47:J58)</f>
-        <v>49.1207768595041</v>
+        <v>94.3706611570248</v>
       </c>
       <c r="K59" s="42" t="n">
         <f aca="false">SUM(K47:K58)</f>
@@ -4488,7 +4488,7 @@
       </c>
       <c r="L59" s="42" t="n">
         <f aca="false">SUM(L47:L58)</f>
-        <v>49.1207768595041</v>
+        <v>94.3706611570248</v>
       </c>
       <c r="M59" s="45"/>
     </row>
@@ -4675,11 +4675,11 @@
       </c>
       <c r="B4" s="47" t="n">
         <f aca="false">SUM(B6:B370)</f>
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C4" s="47" t="n">
         <f aca="false">SUM(C6:C370)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D4" s="47" t="n">
         <f aca="false">SUM(D6:D370)</f>
@@ -4687,7 +4687,7 @@
       </c>
       <c r="E4" s="47" t="n">
         <f aca="false">SUM(E6:E370)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4" s="47" t="n">
         <f aca="false">SUM(F6:F370)</f>
@@ -4703,39 +4703,39 @@
       </c>
       <c r="I4" s="48" t="n">
         <f aca="false">SUM(I6:I370)</f>
-        <v>46.83</v>
+        <v>53.68</v>
       </c>
       <c r="J4" s="48" t="n">
         <f aca="false">SUM(J6:J370)</f>
-        <v>99.97</v>
+        <v>125.36</v>
       </c>
       <c r="K4" s="48" t="n">
         <f aca="false">SUM(K6:K370)</f>
-        <v>185.26</v>
+        <v>187.99</v>
       </c>
       <c r="M4" s="47" t="n">
         <f aca="false">SUM(M6:M370)</f>
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="N4" s="47" t="n">
         <f aca="false">SUM(N6:N370)</f>
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="O4" s="48" t="n">
         <f aca="false">SUM(O6:O370)</f>
-        <v>619.81</v>
+        <v>749.77</v>
       </c>
       <c r="P4" s="48" t="n">
         <f aca="false">IF(M4&gt;0,O4/M4,"")</f>
-        <v>32.6215789473684</v>
+        <v>32.5986956521739</v>
       </c>
       <c r="Q4" s="48" t="n">
         <f aca="false">IF(M4&gt;0,K4/M4,"")</f>
-        <v>9.75052631578947</v>
+        <v>8.17347826086957</v>
       </c>
       <c r="R4" s="49" t="n">
         <f aca="false">IF(K4&gt;0,O4/K4,"")</f>
-        <v>3.3456223685631</v>
+        <v>3.98835044417256</v>
       </c>
       <c r="S4" s="50" t="n">
         <f aca="false">IF(D4+E4+F4+G4&gt;0,(D4+E4)/(D4+E4+F4+G4),"")</f>
@@ -4743,19 +4743,19 @@
       </c>
       <c r="T4" s="48" t="n">
         <f aca="false">SUM(T6:T370)</f>
-        <v>126.2547</v>
+        <v>154.5789</v>
       </c>
       <c r="U4" s="48" t="n">
         <f aca="false">SUM(U6:U370)</f>
-        <v>-107.09479338843</v>
+        <v>-91.4052066115703</v>
       </c>
       <c r="V4" s="48" t="n">
         <f aca="false">SUM(V6:V370)</f>
-        <v>49.1207768595041</v>
+        <v>94.3706611570248</v>
       </c>
       <c r="X4" s="47" t="n">
         <f aca="false">SUM(X6:X370)</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="Y4" s="47" t="n">
         <f aca="false">SUM(Y6:Y370)</f>
@@ -4763,47 +4763,47 @@
       </c>
       <c r="Z4" s="51" t="n">
         <f aca="false">SUM(Z6:Z370)</f>
-        <v>12.2</v>
+        <v>14.6</v>
       </c>
       <c r="AA4" s="51" t="n">
         <f aca="false">SUM(AA6:AA370)</f>
-        <v>4.2</v>
+        <v>5.2</v>
       </c>
       <c r="AB4" s="51" t="n">
         <f aca="false">SUM(AB6:AB370)</f>
-        <v>2.6</v>
+        <v>3.2</v>
       </c>
       <c r="AC4" s="48" t="n">
         <f aca="false">SUM(AC6:AC370)</f>
-        <v>533.836</v>
+        <v>645.802</v>
       </c>
       <c r="AD4" s="48" t="n">
         <f aca="false">SUM(AD6:AD370)</f>
-        <v>49.60274</v>
+        <v>60.1975</v>
       </c>
       <c r="AE4" s="48" t="n">
         <f aca="false">SUM(AE6:AE370)</f>
-        <v>126.806</v>
+        <v>153.968</v>
       </c>
       <c r="AF4" s="48" t="n">
         <f aca="false">SUM(AF6:AF370)</f>
-        <v>20.956</v>
+        <v>25.792</v>
       </c>
       <c r="AG4" s="48" t="n">
         <f aca="false">SUM(AG6:AG370)</f>
-        <v>84.0404831404959</v>
+        <v>101.633838842975</v>
       </c>
       <c r="AH4" s="48" t="n">
         <f aca="false">SUM(AH6:AH370)</f>
-        <v>185.26</v>
+        <v>187.99</v>
       </c>
       <c r="AI4" s="47" t="n">
         <f aca="false">SUM(AI6:AI370)</f>
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="AJ4" s="48" t="n">
         <f aca="false">SUM(AJ6:AJ370)</f>
-        <v>18.05</v>
+        <v>21.85</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4927,7 +4927,7 @@
         <v>3</v>
       </c>
       <c r="E6" s="54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6" s="54"/>
       <c r="G6" s="54"/>
@@ -4935,10 +4935,10 @@
         <v>3</v>
       </c>
       <c r="I6" s="55" t="n">
-        <v>31.57</v>
+        <v>38.42</v>
       </c>
       <c r="J6" s="55" t="n">
-        <v>39.09</v>
+        <v>32.24</v>
       </c>
       <c r="K6" s="55" t="n">
         <v>67.67</v>
@@ -4952,7 +4952,7 @@
       </c>
       <c r="N6" s="31" t="n">
         <f aca="false">X6+Y6</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O6" s="32" t="n">
         <f aca="false">B6*P1_PVP+C6*P2_PVP</f>
@@ -4976,15 +4976,15 @@
       </c>
       <c r="T6" s="33" t="n">
         <f aca="false">D6*(P1_PVP-P1_CPROD)+E6*(P2_PVP-P2_CPROD)-IF(ISNUMBER(I6),I6,D6*P1_LOG+E6*P2_LOG)</f>
-        <v>86.3505</v>
+        <v>114.6747</v>
       </c>
       <c r="U6" s="33" t="n">
         <f aca="false">T6-(D6*P1_IVAN+E6*P2_IVAN)-(F6+G6)*(COSTE_DEV-IVA_DEV)-AH6-AJ6</f>
-        <v>-10.3350413223141</v>
+        <v>11.8845454545454</v>
       </c>
       <c r="V6" s="33" t="n">
         <f aca="false">AC6-AD6-AE6-AF6-AG6-AH6-AJ6</f>
-        <v>56.5721652892561</v>
+        <v>62.6280826446281</v>
       </c>
       <c r="X6" s="58" t="n">
         <f aca="false">MAX(0,B6-D6-F6)</f>
@@ -4992,7 +4992,7 @@
       </c>
       <c r="Y6" s="58" t="n">
         <f aca="false">MAX(0,C6-E6-G6)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Z6" s="59" t="n">
         <f aca="false">D6+X6*TASA_USADA</f>
@@ -5000,31 +5000,31 @@
       </c>
       <c r="AA6" s="59" t="n">
         <f aca="false">E6+Y6*TASA_USADA</f>
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="AB6" s="59" t="n">
         <f aca="false">F6+G6+(X6+Y6)*(1-TASA_USADA)</f>
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="AC6" s="60" t="n">
         <f aca="false">Z6*P1_PVP+AA6*P2_PVP</f>
-        <v>273.92</v>
+        <v>281.918</v>
       </c>
       <c r="AD6" s="60" t="n">
         <f aca="false">Z6*P1_CPROD+AA6*P2_CPROD</f>
-        <v>27.45006</v>
+        <v>28.41322</v>
       </c>
       <c r="AE6" s="60" t="n">
         <f aca="false">IF(ISNUMBER(I6),I6,D6*P1_LOG+E6*P2_LOG)+IF(ISNUMBER(J6),J6,X6*P1_LOG+Y6*P2_LOG)*TASA_USADA</f>
-        <v>62.842</v>
+        <v>64.212</v>
       </c>
       <c r="AF6" s="60" t="n">
         <f aca="false">AB6*COSTE_DEV</f>
-        <v>8.06</v>
+        <v>6.448</v>
       </c>
       <c r="AG6" s="60" t="n">
         <f aca="false">Z6*P1_IVAN+AA6*P2_IVAN-AB6*IVA_DEV</f>
-        <v>42.7757747107438</v>
+        <v>43.9966973553719</v>
       </c>
       <c r="AH6" s="60" t="n">
         <f aca="false">K6*(1+RECARGO_ADS)</f>
@@ -5164,10 +5164,10 @@
         <v>46302</v>
       </c>
       <c r="B8" s="54" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C8" s="54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" s="54"/>
       <c r="E8" s="54"/>
@@ -5178,7 +5178,7 @@
         <v>0</v>
       </c>
       <c r="J8" s="55" t="n">
-        <v>16.12</v>
+        <v>48.36</v>
       </c>
       <c r="K8" s="55" t="n">
         <v>47.41</v>
@@ -5186,27 +5186,27 @@
       <c r="L8" s="56"/>
       <c r="M8" s="31" t="n">
         <f aca="false">B8+C8</f>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N8" s="31" t="n">
         <f aca="false">X8+Y8</f>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="O8" s="32" t="n">
         <f aca="false">B8*P1_PVP+C8*P2_PVP</f>
-        <v>59.98</v>
+        <v>189.94</v>
       </c>
       <c r="P8" s="32" t="n">
         <f aca="false">IF(M8&gt;0,O8/M8,"")</f>
-        <v>29.99</v>
+        <v>31.6566666666667</v>
       </c>
       <c r="Q8" s="32" t="n">
         <f aca="false">IF(M8&gt;0,K8/M8,"")</f>
-        <v>23.705</v>
+        <v>7.90166666666667</v>
       </c>
       <c r="R8" s="57" t="n">
         <f aca="false">IF(K8&gt;0,O8/K8,"")</f>
-        <v>1.26513393798777</v>
+        <v>4.00632777894959</v>
       </c>
       <c r="S8" s="34" t="str">
         <f aca="false">IF(D8+E8+F8+G8&gt;0,(D8+E8)/(D8+E8+F8+G8),"")</f>
@@ -5218,51 +5218,51 @@
       </c>
       <c r="U8" s="33" t="n">
         <f aca="false">T8-(D8*P1_IVAN+E8*P2_IVAN)-(F8+G8)*(COSTE_DEV-IVA_DEV)-AH8-AJ8</f>
-        <v>-49.31</v>
+        <v>-53.11</v>
       </c>
       <c r="V8" s="33" t="n">
         <f aca="false">AC8-AD8-AE8-AF8-AG8-AH8-AJ8</f>
-        <v>-28.9578016528926</v>
+        <v>12.9661652892562</v>
       </c>
       <c r="X8" s="58" t="n">
         <f aca="false">MAX(0,B8-D8-F8)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Y8" s="58" t="n">
         <f aca="false">MAX(0,C8-E8-G8)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z8" s="59" t="n">
         <f aca="false">D8+X8*TASA_USADA</f>
-        <v>1.6</v>
+        <v>4</v>
       </c>
       <c r="AA8" s="59" t="n">
         <f aca="false">E8+Y8*TASA_USADA</f>
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="AB8" s="59" t="n">
         <f aca="false">F8+G8+(X8+Y8)*(1-TASA_USADA)</f>
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="AC8" s="60" t="n">
         <f aca="false">Z8*P1_PVP+AA8*P2_PVP</f>
-        <v>47.984</v>
+        <v>151.952</v>
       </c>
       <c r="AD8" s="60" t="n">
         <f aca="false">Z8*P1_CPROD+AA8*P2_CPROD</f>
-        <v>3.85264</v>
+        <v>13.48424</v>
       </c>
       <c r="AE8" s="60" t="n">
         <f aca="false">IF(ISNUMBER(I8),I8,D8*P1_LOG+E8*P2_LOG)+IF(ISNUMBER(J8),J8,X8*P1_LOG+Y8*P2_LOG)*TASA_USADA</f>
-        <v>12.896</v>
+        <v>38.688</v>
       </c>
       <c r="AF8" s="60" t="n">
         <f aca="false">AB8*COSTE_DEV</f>
-        <v>3.224</v>
+        <v>9.672</v>
       </c>
       <c r="AG8" s="60" t="n">
         <f aca="false">Z8*P1_IVAN+AA8*P2_IVAN-AB8*IVA_DEV</f>
-        <v>7.65916165289256</v>
+        <v>24.0315947107438</v>
       </c>
       <c r="AH8" s="60" t="n">
         <f aca="false">K8*(1+RECARGO_ADS)</f>
@@ -5270,27 +5270,37 @@
       </c>
       <c r="AI8" s="58" t="n">
         <f aca="false">IF(ISNUMBER(I8),D8+E8+X8+Y8,0)</f>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AJ8" s="60" t="n">
         <f aca="false">M8*COMISION</f>
-        <v>1.9</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="53" t="n">
         <v>46303</v>
       </c>
-      <c r="B9" s="54"/>
-      <c r="C9" s="54"/>
+      <c r="B9" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="54" t="n">
+        <v>0</v>
+      </c>
       <c r="D9" s="54"/>
       <c r="E9" s="54"/>
       <c r="F9" s="54"/>
       <c r="G9" s="54"/>
       <c r="H9" s="54"/>
-      <c r="I9" s="55"/>
-      <c r="J9" s="55"/>
-      <c r="K9" s="55"/>
+      <c r="I9" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="55" t="n">
+        <v>2.73</v>
+      </c>
       <c r="L9" s="56"/>
       <c r="M9" s="31" t="n">
         <f aca="false">B9+C9</f>
@@ -5312,9 +5322,9 @@
         <f aca="false">IF(M9&gt;0,K9/M9,"")</f>
         <v/>
       </c>
-      <c r="R9" s="57" t="str">
+      <c r="R9" s="57" t="n">
         <f aca="false">IF(K9&gt;0,O9/K9,"")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S9" s="34" t="str">
         <f aca="false">IF(D9+E9+F9+G9&gt;0,(D9+E9)/(D9+E9+F9+G9),"")</f>
@@ -5326,11 +5336,11 @@
       </c>
       <c r="U9" s="33" t="n">
         <f aca="false">T9-(D9*P1_IVAN+E9*P2_IVAN)-(F9+G9)*(COSTE_DEV-IVA_DEV)-AH9-AJ9</f>
-        <v>0</v>
+        <v>-2.73</v>
       </c>
       <c r="V9" s="33" t="n">
         <f aca="false">AC9-AD9-AE9-AF9-AG9-AH9-AJ9</f>
-        <v>0</v>
+        <v>-2.73</v>
       </c>
       <c r="X9" s="58" t="n">
         <f aca="false">MAX(0,B9-D9-F9)</f>
@@ -5374,7 +5384,7 @@
       </c>
       <c r="AH9" s="60" t="n">
         <f aca="false">K9*(1+RECARGO_ADS)</f>
-        <v>0</v>
+        <v>2.73</v>
       </c>
       <c r="AI9" s="58" t="n">
         <f aca="false">IF(ISNUMBER(I9),D9+E9+X9+Y9,0)</f>
@@ -46999,7 +47009,7 @@
       </c>
       <c r="C37" s="31" t="n">
         <f aca="false">(SUM(Diario!$D$6:$D$370)+SUM(Diario!$E$6:$E$370))+(SUM(Diario!$F$6:$F$370)+SUM(Diario!$G$6:$G$370))</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E37" s="67" t="s">
         <v>176</v>
@@ -47035,7 +47045,7 @@
       </c>
       <c r="C40" s="34" t="n">
         <f aca="false">IF(SUM(Diario!$M$6:$M$370)&gt;0,SUM(Diario!$C$6:$C$370)/SUM(Diario!$M$6:$M$370),"")</f>
-        <v>0.263157894736842</v>
+        <v>0.260869565217391</v>
       </c>
       <c r="E40" s="67" t="s">
         <v>182</v>
@@ -47047,7 +47057,7 @@
       </c>
       <c r="C41" s="34" t="n">
         <f aca="false">IF(C40="",C26,C40)</f>
-        <v>0.263157894736842</v>
+        <v>0.260869565217391</v>
       </c>
       <c r="E41" s="67"/>
     </row>
@@ -47057,7 +47067,7 @@
       </c>
       <c r="C42" s="32" t="n">
         <f aca="false">IF(SUM(Diario!$AI$6:$AI$370)&gt;0,(SUM(Diario!$I$6:$I$370)+SUM(Diario!$J$6:$J$370))/SUM(Diario!$AI$6:$AI$370),"")</f>
-        <v>7.72631578947369</v>
+        <v>7.78434782608696</v>
       </c>
       <c r="E42" s="67" t="s">
         <v>185</v>
@@ -47069,7 +47079,7 @@
       </c>
       <c r="C43" s="32" t="n">
         <f aca="false">(1-C41)*C5+C41*D5</f>
-        <v>32.6215789473684</v>
+        <v>32.5986956521739</v>
       </c>
       <c r="E43" s="67"/>
     </row>
@@ -47079,7 +47089,7 @@
       </c>
       <c r="C44" s="32" t="n">
         <f aca="false">(1-C41)*(C5-C9-IF(C42="",C8,C42)-C14)+C41*(D5-D9-IF(C42="",D8,C42)-D14)</f>
-        <v>16.7199826011309</v>
+        <v>16.647592526051</v>
       </c>
       <c r="E44" s="67" t="s">
         <v>188</v>
@@ -47091,7 +47101,7 @@
       </c>
       <c r="C45" s="32" t="n">
         <f aca="false">C39*C44-(1-C39)*C36-COMISION</f>
-        <v>10.8139860809047</v>
+        <v>10.7560740208408</v>
       </c>
       <c r="E45" s="67" t="s">
         <v>190</v>
@@ -47103,7 +47113,7 @@
       </c>
       <c r="C46" s="33" t="n">
         <f aca="false">C45/(1+RECARGO_ADS)</f>
-        <v>10.8139860809047</v>
+        <v>10.7560740208408</v>
       </c>
       <c r="E46" s="67" t="s">
         <v>192</v>
@@ -47115,7 +47125,7 @@
       </c>
       <c r="C47" s="72" t="n">
         <f aca="false">IF(C46&gt;0,C43/C46,"")</f>
-        <v>3.01661003660541</v>
+        <v>3.0307243692272</v>
       </c>
       <c r="E47" s="67" t="s">
         <v>194</v>

</xml_diff>

<commit_message>
Devoluciones: coste de 8,06 € confirmado con Dropi (el envío incluye la vuelta)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFjE4yx23BY3D6kaMQowKe
</commit_message>
<xml_diff>
--- a/contabilidad/CeraLux_Contabilidad.xlsx
+++ b/contabilidad/CeraLux_Contabilidad.xlsx
@@ -625,7 +625,7 @@
     <t xml:space="preserve">Coste por pedido devuelto</t>
   </si>
   <si>
-    <t xml:space="preserve">SUPUESTO: pierdes el envío (8,06 €) y el producto vuelve al stock. Confírmalo con tu almacén.</t>
+    <t xml:space="preserve">Confirmado con Dropi: el envío de ida ya incluye la vuelta, así que pierdes el envío (8,06 €) y el producto vuelve.</t>
   </si>
   <si>
     <t xml:space="preserve">Recargo sobre el gasto en Ads</t>
@@ -1852,8 +1852,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="12703388"/>
-        <c:axId val="77698927"/>
+        <c:axId val="80276800"/>
+        <c:axId val="39529553"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2022,11 +2022,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="12703388"/>
-        <c:axId val="77698927"/>
+        <c:axId val="80276800"/>
+        <c:axId val="39529553"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="12703388"/>
+        <c:axId val="80276800"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2058,7 +2058,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="77698927"/>
+        <c:crossAx val="39529553"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2066,7 +2066,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="77698927"/>
+        <c:axId val="39529553"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2108,7 +2108,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="12703388"/>
+        <c:crossAx val="80276800"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2348,8 +2348,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="9173522"/>
-        <c:axId val="77168686"/>
+        <c:axId val="88888392"/>
+        <c:axId val="17330329"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2446,11 +2446,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="9173522"/>
-        <c:axId val="77168686"/>
+        <c:axId val="88888392"/>
+        <c:axId val="17330329"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="9173522"/>
+        <c:axId val="88888392"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2482,7 +2482,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="77168686"/>
+        <c:crossAx val="17330329"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2490,7 +2490,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="77168686"/>
+        <c:axId val="17330329"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2532,7 +2532,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9173522"/>
+        <c:crossAx val="88888392"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -46841,7 +46841,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="63" t="s">
         <v>148</v>
       </c>

</xml_diff>

<commit_message>
Almacén al 09/10: Rehusado cuenta como devuelto, estados nuevos
- Importador Python y página comparan estados por prefijo: "Rehusado - en
  tránsito" = devolución; "Pedido nuevo", "Enviado", "Confirmado - Pendiente
  de preparación" = pendiente.
- La fuente del panel recoge la versión en vivo (pestañas Embudo y Horas).
- Excel de contabilidad regenerado con el export del 09/10 (44 pedidos,
  9 entregados, 2 devueltos; liquidación 202,43 € vs 202,40 € del almacén).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFjE4yx23BY3D6kaMQowKe
</commit_message>
<xml_diff>
--- a/contabilidad/CeraLux_Contabilidad.xlsx
+++ b/contabilidad/CeraLux_Contabilidad.xlsx
@@ -180,7 +180,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="231">
   <si>
     <t xml:space="preserve">CeraLux · Dashboard de rentabilidad</t>
   </si>
@@ -501,6 +501,9 @@
   </si>
   <si>
     <t xml:space="preserve">Arranca campaña CeraLux ES - Test 3 ángulos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Primer rehusado: #1184 (pack 2, 39,99 €) rechazado en la puerta</t>
   </si>
   <si>
     <t xml:space="preserve">Todo lo que no es producto, envío ni Ads: Shopify, apps, dominio, muestras, gestoría...</t>
@@ -1776,46 +1779,46 @@
               <c:strCache>
                 <c:ptCount val="14"/>
                 <c:pt idx="0">
-                  <c:v>Fri 25/09</c:v>
+                  <c:v>Sat 26/09</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Sat 26/09</c:v>
+                  <c:v>Sun 27/09</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Sun 27/09</c:v>
+                  <c:v>Mon 28/09</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Mon 28/09</c:v>
+                  <c:v>Tue 29/09</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Tue 29/09</c:v>
+                  <c:v>Wed 30/09</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Wed 30/09</c:v>
+                  <c:v>Thu 01/10</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Thu 01/10</c:v>
+                  <c:v>Fri 02/10</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>Fri 02/10</c:v>
+                  <c:v>Sat 03/10</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Sat 03/10</c:v>
+                  <c:v>Sun 04/10</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Sun 04/10</c:v>
+                  <c:v>Mon 05/10</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Mon 05/10</c:v>
+                  <c:v>Tue 06/10</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>Tue 06/10</c:v>
+                  <c:v>Wed 07/10</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>Wed 07/10</c:v>
+                  <c:v>Thu 08/10</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>Thu 08/10</c:v>
+                  <c:v>Fri 09/10</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1854,19 +1857,19 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>62.6280826446281</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>62.6280826446281</c:v>
+                  <c:v>8.63823140495868</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>27.5623305785124</c:v>
+                  <c:v>28.2932892561984</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>28.2932892561984</c:v>
+                  <c:v>122.108479338843</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>73.8827438016529</c:v>
+                  <c:v>30.8135371900827</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1874,8 +1877,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="44160966"/>
-        <c:axId val="60711204"/>
+        <c:axId val="52780188"/>
+        <c:axId val="78457029"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -1939,46 +1942,46 @@
               <c:strCache>
                 <c:ptCount val="14"/>
                 <c:pt idx="0">
-                  <c:v>Fri 25/09</c:v>
+                  <c:v>Sat 26/09</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Sat 26/09</c:v>
+                  <c:v>Sun 27/09</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Sun 27/09</c:v>
+                  <c:v>Mon 28/09</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Mon 28/09</c:v>
+                  <c:v>Tue 29/09</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Tue 29/09</c:v>
+                  <c:v>Wed 30/09</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Wed 30/09</c:v>
+                  <c:v>Thu 01/10</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Thu 01/10</c:v>
+                  <c:v>Fri 02/10</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>Fri 02/10</c:v>
+                  <c:v>Sat 03/10</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Sat 03/10</c:v>
+                  <c:v>Sun 04/10</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Sun 04/10</c:v>
+                  <c:v>Mon 05/10</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Mon 05/10</c:v>
+                  <c:v>Tue 06/10</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>Tue 06/10</c:v>
+                  <c:v>Wed 07/10</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>Wed 07/10</c:v>
+                  <c:v>Thu 08/10</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>Thu 08/10</c:v>
+                  <c:v>Fri 09/10</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2017,19 +2020,19 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>67.67</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>67.67</c:v>
+                  <c:v>70.18</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>70.18</c:v>
+                  <c:v>47.78</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>47.78</c:v>
+                  <c:v>50.41</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>38.25</c:v>
+                  <c:v>16.13</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2044,11 +2047,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="44160966"/>
-        <c:axId val="60711204"/>
+        <c:axId val="52780188"/>
+        <c:axId val="78457029"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="44160966"/>
+        <c:axId val="52780188"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2080,7 +2083,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60711204"/>
+        <c:crossAx val="78457029"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2088,7 +2091,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="60711204"/>
+        <c:axId val="78457029"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2130,7 +2133,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44160966"/>
+        <c:crossAx val="52780188"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2329,7 +2332,7 @@
                 <c:formatCode>#,##0" €";[RED]\-#,##0" €";\-</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>192.366446280992</c:v>
+                  <c:v>252.481619834711</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -2370,8 +2373,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="16974961"/>
-        <c:axId val="15853717"/>
+        <c:axId val="83250474"/>
+        <c:axId val="45140102"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2468,11 +2471,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="16974961"/>
-        <c:axId val="15853717"/>
+        <c:axId val="83250474"/>
+        <c:axId val="45140102"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="16974961"/>
+        <c:axId val="83250474"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2504,7 +2507,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="15853717"/>
+        <c:crossAx val="45140102"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2512,7 +2515,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="15853717"/>
+        <c:axId val="45140102"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2554,7 +2557,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="16974961"/>
+        <c:crossAx val="83250474"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2884,7 +2887,7 @@
       </c>
       <c r="F3" s="4" t="n">
         <f aca="true">TODAY()</f>
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="G3" s="4"/>
       <c r="H3" s="3" t="s">
@@ -2892,7 +2895,7 @@
       </c>
       <c r="I3" s="5" t="n">
         <f aca="false">MAX(1,$F$3-$C$3+1)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J3" s="6" t="s">
         <v>5</v>
@@ -2948,7 +2951,7 @@
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="10" t="n">
         <f aca="false">F25</f>
-        <v>192.366446280992</v>
+        <v>252.481619834711</v>
       </c>
       <c r="C7" s="10"/>
       <c r="D7" s="10" t="n">
@@ -2958,22 +2961,22 @@
       <c r="E7" s="10"/>
       <c r="F7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$X$6:$X$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+F24</f>
-        <v>-99.8404958677686</v>
+        <v>-154.700495867769</v>
       </c>
       <c r="G7" s="10"/>
       <c r="H7" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="I7" s="11"/>
       <c r="J7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$R$6:$R$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>1099.67</v>
+        <v>1479.56</v>
       </c>
       <c r="K7" s="10"/>
       <c r="L7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>223.88</v>
+        <v>252.17</v>
       </c>
       <c r="M7" s="10"/>
     </row>
@@ -3006,32 +3009,32 @@
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="10" t="n">
         <f aca="false">IF(H7&gt;0,L7/H7,"")</f>
-        <v>6.78424242424242</v>
+        <v>5.73113636363636</v>
       </c>
       <c r="C10" s="10"/>
       <c r="D10" s="10" t="n">
         <f aca="false">CPA_BE</f>
-        <v>11.2321377410468</v>
+        <v>11.3917783979106</v>
       </c>
       <c r="E10" s="10"/>
       <c r="F10" s="12" t="n">
         <f aca="false">IF(L7&gt;0,J7/L7,"")</f>
-        <v>4.91187243165982</v>
+        <v>5.8673117341476</v>
       </c>
       <c r="G10" s="12"/>
       <c r="H10" s="12" t="n">
         <f aca="false">ROAS_BE</f>
-        <v>2.96678460517415</v>
+        <v>2.95180984582101</v>
       </c>
       <c r="I10" s="12"/>
       <c r="J10" s="10" t="n">
         <f aca="false">IF(H7&gt;0,J7/H7,"")</f>
-        <v>33.3233333333333</v>
+        <v>33.6263636363636</v>
       </c>
       <c r="K10" s="10"/>
       <c r="L10" s="13" t="n">
         <f aca="false">IF(H7&gt;0,(SUMIFS(Diario!$C$6:$C$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+SUMIFS(Diario!$D$6:$D$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3))/H7,"")</f>
-        <v>0.333333333333333</v>
+        <v>0.340909090909091</v>
       </c>
       <c r="M10" s="13"/>
     </row>
@@ -3069,22 +3072,22 @@
       <c r="C13" s="11"/>
       <c r="D13" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$Q$6:$Q$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="E13" s="11"/>
       <c r="F13" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$K$6:$K$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G13" s="11"/>
       <c r="H13" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I13" s="11"/>
       <c r="J13" s="13" t="n">
         <f aca="false">IF(B13+H13&gt;0,B13/(B13+H13),"")</f>
-        <v>1</v>
+        <v>0.818181818181818</v>
       </c>
       <c r="K13" s="13"/>
       <c r="L13" s="14" t="str">
@@ -3121,7 +3124,7 @@
       </c>
       <c r="F16" s="17" t="n">
         <f aca="false">SUMIFS(Diario!$AH$6:$AH$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>939.718</v>
+        <v>1187.646</v>
       </c>
       <c r="H16" s="15" t="s">
         <v>29</v>
@@ -3143,11 +3146,11 @@
       <c r="D17" s="15"/>
       <c r="E17" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F17/$F$16,"")</f>
-        <v>-0.0963449034710413</v>
+        <v>-0.0973178876533916</v>
       </c>
       <c r="F17" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AI$6:$AI$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-90.53704</v>
+        <v>-115.5792</v>
       </c>
       <c r="H17" s="15" t="s">
         <v>31</v>
@@ -3157,7 +3160,7 @@
       <c r="K17" s="15"/>
       <c r="L17" s="20" t="n">
         <f aca="false">F25/I3</f>
-        <v>24.045805785124</v>
+        <v>28.0535133149679</v>
       </c>
       <c r="M17" s="20"/>
     </row>
@@ -3169,11 +3172,11 @@
       <c r="D18" s="15"/>
       <c r="E18" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F18/$F$16,"")</f>
-        <v>-0.229343271066426</v>
+        <v>-0.227540866554512</v>
       </c>
       <c r="F18" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AJ$6:$AJ$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-215.518</v>
+        <v>-270.238</v>
       </c>
       <c r="H18" s="15" t="s">
         <v>33</v>
@@ -3183,7 +3186,7 @@
       <c r="K18" s="15"/>
       <c r="L18" s="18" t="n">
         <f aca="false">L17*30</f>
-        <v>721.374173553719</v>
+        <v>841.605399449037</v>
       </c>
       <c r="M18" s="18"/>
     </row>
@@ -3195,11 +3198,11 @@
       <c r="D19" s="15"/>
       <c r="E19" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F19/$F$16,"")</f>
-        <v>-0.041169797747835</v>
+        <v>-0.0583641926971505</v>
       </c>
       <c r="F19" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AK$6:$AK$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-38.688</v>
+        <v>-69.316</v>
       </c>
       <c r="H19" s="21" t="s">
         <v>35</v>
@@ -3209,7 +3212,7 @@
       <c r="K19" s="21"/>
       <c r="L19" s="22" t="n">
         <f aca="false">IF(L16&gt;0,L18/L16,"")</f>
-        <v>0.0721374173553719</v>
+        <v>0.0841605399449037</v>
       </c>
       <c r="M19" s="22"/>
     </row>
@@ -3221,11 +3224,11 @@
       <c r="D20" s="15"/>
       <c r="E20" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F20/$F$16,"")</f>
-        <v>-0.0333610721514327</v>
+        <v>-0.0351956727846513</v>
       </c>
       <c r="F20" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AO$6:$AO$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-31.35</v>
+        <v>-41.8</v>
       </c>
       <c r="H20" s="15" t="s">
         <v>37</v>
@@ -3235,7 +3238,7 @@
       <c r="K20" s="15"/>
       <c r="L20" s="20" t="n">
         <f aca="false">BEN_PEDIDO</f>
-        <v>11.2321377410468</v>
+        <v>11.3917783979106</v>
       </c>
       <c r="M20" s="20"/>
     </row>
@@ -3247,11 +3250,11 @@
       <c r="D21" s="15"/>
       <c r="E21" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F21/$F$16,"")</f>
-        <v>-0.156832702703373</v>
+        <v>-0.15666383767999</v>
       </c>
       <c r="F21" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AL$6:$AL$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-147.378513719008</v>
+        <v>-186.061180165289</v>
       </c>
       <c r="H21" s="15" t="s">
         <v>39</v>
@@ -3261,7 +3264,7 @@
       <c r="K21" s="15"/>
       <c r="L21" s="20" t="n">
         <f aca="false">B10</f>
-        <v>6.78424242424242</v>
+        <v>5.73113636363636</v>
       </c>
       <c r="M21" s="20"/>
     </row>
@@ -3273,11 +3276,11 @@
       <c r="D22" s="15"/>
       <c r="E22" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F22/$F$16,"")</f>
-        <v>-0.238241685271539</v>
+        <v>-0.212327579093434</v>
       </c>
       <c r="F22" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AM$6:$AM$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-223.88</v>
+        <v>-252.17</v>
       </c>
       <c r="H22" s="15" t="s">
         <v>41</v>
@@ -3287,7 +3290,7 @@
       <c r="K22" s="15"/>
       <c r="L22" s="20" t="n">
         <f aca="false">IF(ISNUMBER(L21),L20-L21*(1+RECARGO_ADS),"")</f>
-        <v>4.44789531680441</v>
+        <v>5.66064203427427</v>
       </c>
       <c r="M22" s="20"/>
     </row>
@@ -3299,11 +3302,11 @@
       <c r="D23" s="23"/>
       <c r="E23" s="24" t="n">
         <f aca="false">IF($F$16&gt;0,F23/$F$16,"")</f>
-        <v>0.204706567588353</v>
+        <v>0.212589963536871</v>
       </c>
       <c r="F23" s="25" t="n">
         <f aca="false">SUM(F16:F22)</f>
-        <v>192.366446280992</v>
+        <v>252.481619834711</v>
       </c>
       <c r="H23" s="21" t="s">
         <v>43</v>
@@ -3313,7 +3316,7 @@
       <c r="K23" s="21"/>
       <c r="L23" s="26" t="n">
         <f aca="false">IF(NOT(ISNUMBER(L22)),"",IF(L22&lt;=0,"Baja el CPA",ROUNDUP((L16-F24/I3*30)/30/L22,0)))</f>
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="M23" s="26"/>
     </row>
@@ -3339,7 +3342,7 @@
       <c r="K24" s="15"/>
       <c r="L24" s="18" t="n">
         <f aca="false">IF(ISNUMBER(L23),L23*L21,"")</f>
-        <v>508.818181818182</v>
+        <v>338.137045454545</v>
       </c>
       <c r="M24" s="18"/>
     </row>
@@ -3351,11 +3354,11 @@
       <c r="D25" s="23"/>
       <c r="E25" s="24" t="n">
         <f aca="false">IF($F$16&gt;0,F25/$F$16,"")</f>
-        <v>0.204706567588353</v>
+        <v>0.212589963536871</v>
       </c>
       <c r="F25" s="25" t="n">
         <f aca="false">F23+F24</f>
-        <v>192.366446280992</v>
+        <v>252.481619834711</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3366,7 +3369,7 @@
       <c r="D26" s="27"/>
       <c r="F26" s="28" t="n">
         <f aca="false">IF(F16&gt;0,F25/F16,"")</f>
-        <v>0.204706567588353</v>
+        <v>0.212589963536871</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3402,7 +3405,7 @@
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="30" t="n">
         <f aca="false">$F$3-13</f>
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="C29" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B29)</f>
@@ -3428,7 +3431,7 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="30" t="n">
         <f aca="false">$F$3-12</f>
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="C30" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B30)</f>
@@ -3454,7 +3457,7 @@
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="30" t="n">
         <f aca="false">$F$3-11</f>
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="C31" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B31)</f>
@@ -3480,7 +3483,7 @@
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="30" t="n">
         <f aca="false">$F$3-10</f>
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="C32" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B32)</f>
@@ -3506,7 +3509,7 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="30" t="n">
         <f aca="false">$F$3-9</f>
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="C33" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B33)</f>
@@ -3532,7 +3535,7 @@
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="30" t="n">
         <f aca="false">$F$3-8</f>
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="C34" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B34)</f>
@@ -3558,7 +3561,7 @@
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="30" t="n">
         <f aca="false">$F$3-7</f>
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="C35" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B35)</f>
@@ -3584,7 +3587,7 @@
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="30" t="n">
         <f aca="false">$F$3-6</f>
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="C36" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B36)</f>
@@ -3610,7 +3613,7 @@
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="30" t="n">
         <f aca="false">$F$3-5</f>
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="C37" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B37)</f>
@@ -3636,75 +3639,75 @@
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="30" t="n">
         <f aca="false">$F$3-4</f>
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="C38" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B38)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D38" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B38)</f>
-        <v>0</v>
-      </c>
-      <c r="E38" s="32" t="str">
+        <v>67.67</v>
+      </c>
+      <c r="E38" s="32" t="n">
         <f aca="false">IF(C38&gt;0,D38/C38,"")</f>
-        <v/>
+        <v>7.51888888888889</v>
       </c>
       <c r="F38" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B38)</f>
-        <v>0</v>
-      </c>
-      <c r="G38" s="34" t="str">
+        <v>62.6280826446281</v>
+      </c>
+      <c r="G38" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B38))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B38))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B38)),"")</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="30" t="n">
         <f aca="false">$F$3-3</f>
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="C39" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B39)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D39" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B39)</f>
-        <v>67.67</v>
+        <v>70.18</v>
       </c>
       <c r="E39" s="32" t="n">
         <f aca="false">IF(C39&gt;0,D39/C39,"")</f>
-        <v>7.51888888888889</v>
+        <v>8.7725</v>
       </c>
       <c r="F39" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B39)</f>
-        <v>62.6280826446281</v>
+        <v>8.63823140495868</v>
       </c>
       <c r="G39" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B39))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B39))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B39)),"")</f>
-        <v>1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="30" t="n">
         <f aca="false">$F$3-2</f>
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="C40" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B40)</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D40" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B40)</f>
-        <v>70.18</v>
+        <v>47.78</v>
       </c>
       <c r="E40" s="32" t="n">
         <f aca="false">IF(C40&gt;0,D40/C40,"")</f>
-        <v>8.7725</v>
+        <v>6.82571428571429</v>
       </c>
       <c r="F40" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B40)</f>
-        <v>27.5623305785124</v>
+        <v>28.2932892561984</v>
       </c>
       <c r="G40" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B40))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B40))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B40)),"")</f>
@@ -3714,49 +3717,49 @@
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="30" t="n">
         <f aca="false">$F$3-1</f>
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="C41" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B41)</f>
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="D41" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B41)</f>
-        <v>47.78</v>
+        <v>50.41</v>
       </c>
       <c r="E41" s="32" t="n">
         <f aca="false">IF(C41&gt;0,D41/C41,"")</f>
-        <v>6.82571428571429</v>
+        <v>3.150625</v>
       </c>
       <c r="F41" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B41)</f>
-        <v>28.2932892561984</v>
+        <v>122.108479338843</v>
       </c>
       <c r="G41" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B41))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B41))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B41)),"")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="30" t="n">
         <f aca="false">$F$3-0</f>
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="C42" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B42)</f>
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D42" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B42)</f>
-        <v>38.25</v>
+        <v>16.13</v>
       </c>
       <c r="E42" s="32" t="n">
         <f aca="false">IF(C42&gt;0,D42/C42,"")</f>
-        <v>4.25</v>
+        <v>4.0325</v>
       </c>
       <c r="F42" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B42)</f>
-        <v>73.8827438016529</v>
+        <v>30.8135371900827</v>
       </c>
       <c r="G42" s="34" t="str">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B42))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B42))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B42)),"")</f>
@@ -3827,19 +3830,19 @@
       </c>
       <c r="C47" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="D47" s="37" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>223.88</v>
+        <v>252.17</v>
       </c>
       <c r="E47" s="32" t="n">
         <f aca="false">IF(C47&gt;0,D47/C47,"")</f>
-        <v>6.78424242424242</v>
+        <v>5.73113636363636</v>
       </c>
       <c r="F47" s="37" t="n">
         <f aca="false">SUMIFS(Diario!$R$6:$R$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>1099.67</v>
+        <v>1479.56</v>
       </c>
       <c r="G47" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
@@ -3847,15 +3850,15 @@
       </c>
       <c r="H47" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I47" s="34" t="n">
         <f aca="false">IF(G47+H47&gt;0,G47/(G47+H47),"")</f>
-        <v>1</v>
+        <v>0.818181818181818</v>
       </c>
       <c r="J47" s="37" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>192.366446280992</v>
+        <v>252.481619834711</v>
       </c>
       <c r="K47" s="37" t="n">
         <f aca="false">-SUMIFS(Gastos!$D$5:$D$304,Gastos!$A$5:$A$304,"&gt;="&amp;$B47,Gastos!$A$5:$A$304,"&lt;="&amp;EOMONTH($B47,0))</f>
@@ -3863,11 +3866,11 @@
       </c>
       <c r="L47" s="38" t="n">
         <f aca="false">J47+K47</f>
-        <v>192.366446280992</v>
+        <v>252.481619834711</v>
       </c>
       <c r="M47" s="34" t="n">
         <f aca="false">IF(OBJETIVO_MES&gt;0,L47/OBJETIVO_MES,"")</f>
-        <v>0.0192366446280992</v>
+        <v>0.0252481619834711</v>
       </c>
       <c r="O47" s="39" t="n">
         <f aca="false">OBJETIVO_MES</f>
@@ -4474,19 +4477,19 @@
       </c>
       <c r="C59" s="41" t="n">
         <f aca="false">SUM(C47:C58)</f>
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="D59" s="42" t="n">
         <f aca="false">SUM(D47:D58)</f>
-        <v>223.88</v>
+        <v>252.17</v>
       </c>
       <c r="E59" s="43" t="n">
         <f aca="false">IF(C59&gt;0,D59/C59,"")</f>
-        <v>6.78424242424242</v>
+        <v>5.73113636363636</v>
       </c>
       <c r="F59" s="42" t="n">
         <f aca="false">SUM(F47:F58)</f>
-        <v>1099.67</v>
+        <v>1479.56</v>
       </c>
       <c r="G59" s="41" t="n">
         <f aca="false">SUM(G47:G58)</f>
@@ -4494,15 +4497,15 @@
       </c>
       <c r="H59" s="41" t="n">
         <f aca="false">SUM(H47:H58)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I59" s="44" t="n">
         <f aca="false">IF(G59+H59&gt;0,G59/(G59+H59),"")</f>
-        <v>1</v>
+        <v>0.818181818181818</v>
       </c>
       <c r="J59" s="42" t="n">
         <f aca="false">SUM(J47:J58)</f>
-        <v>192.366446280992</v>
+        <v>252.481619834711</v>
       </c>
       <c r="K59" s="42" t="n">
         <f aca="false">SUM(K47:K58)</f>
@@ -4510,7 +4513,7 @@
       </c>
       <c r="L59" s="42" t="n">
         <f aca="false">SUM(L47:L58)</f>
-        <v>192.366446280992</v>
+        <v>252.481619834711</v>
       </c>
       <c r="M59" s="45"/>
     </row>
@@ -4697,15 +4700,15 @@
       </c>
       <c r="B4" s="47" t="n">
         <f aca="false">SUM(B6:B370)</f>
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C4" s="47" t="n">
         <f aca="false">SUM(C6:C370)</f>
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D4" s="47" t="n">
         <f aca="false">SUM(D6:D370)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" s="47" t="n">
         <f aca="false">SUM(E6:E370)</f>
@@ -4721,11 +4724,11 @@
       </c>
       <c r="H4" s="47" t="n">
         <f aca="false">SUM(H6:H370)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" s="47" t="n">
         <f aca="false">SUM(I6:I370)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" s="47" t="n">
         <f aca="false">SUM(J6:J370)</f>
@@ -4733,7 +4736,7 @@
       </c>
       <c r="K4" s="47" t="n">
         <f aca="false">SUM(K6:K370)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L4" s="48" t="n">
         <f aca="false">SUM(L6:L370)</f>
@@ -4741,39 +4744,39 @@
       </c>
       <c r="M4" s="48" t="n">
         <f aca="false">SUM(M6:M370)</f>
-        <v>183.66</v>
+        <v>252.06</v>
       </c>
       <c r="N4" s="48" t="n">
         <f aca="false">SUM(N6:N370)</f>
-        <v>223.88</v>
+        <v>252.17</v>
       </c>
       <c r="P4" s="47" t="n">
         <f aca="false">SUM(P6:P370)</f>
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="Q4" s="47" t="n">
         <f aca="false">SUM(Q6:Q370)</f>
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="R4" s="48" t="n">
         <f aca="false">SUM(R6:R370)</f>
-        <v>1099.67</v>
+        <v>1479.56</v>
       </c>
       <c r="S4" s="48" t="n">
         <f aca="false">IF(P4&gt;0,R4/P4,"")</f>
-        <v>33.3233333333333</v>
+        <v>33.6263636363636</v>
       </c>
       <c r="T4" s="48" t="n">
         <f aca="false">IF(P4&gt;0,N4/P4,"")</f>
-        <v>6.78424242424242</v>
+        <v>5.73113636363636</v>
       </c>
       <c r="U4" s="49" t="n">
         <f aca="false">IF(N4&gt;0,R4/N4,"")</f>
-        <v>4.91187243165982</v>
+        <v>5.8673117341476</v>
       </c>
       <c r="V4" s="50" t="n">
         <f aca="false">IF(E4+F4+G4+H4+I4+J4&gt;0,(E4+F4+G4)/(E4+F4+G4+H4+I4+J4),"")</f>
-        <v>1</v>
+        <v>0.818181818181818</v>
       </c>
       <c r="W4" s="48" t="n">
         <f aca="false">SUM(W6:W370)</f>
@@ -4781,71 +4784,71 @@
       </c>
       <c r="X4" s="48" t="n">
         <f aca="false">SUM(X6:X370)</f>
-        <v>-99.8404958677686</v>
+        <v>-154.700495867769</v>
       </c>
       <c r="Y4" s="48" t="n">
         <f aca="false">SUM(Y6:Y370)</f>
-        <v>192.366446280992</v>
+        <v>252.481619834711</v>
       </c>
       <c r="AA4" s="47" t="n">
         <f aca="false">SUM(AA6:AA370)</f>
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="AB4" s="47" t="n">
         <f aca="false">SUM(AB6:AB370)</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="AC4" s="47" t="n">
         <f aca="false">SUM(AC6:AC370)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD4" s="51" t="n">
         <f aca="false">SUM(AD6:AD370)</f>
-        <v>18.8</v>
+        <v>23.6</v>
       </c>
       <c r="AE4" s="51" t="n">
         <f aca="false">SUM(AE6:AE370)</f>
-        <v>9.4</v>
+        <v>11</v>
       </c>
       <c r="AF4" s="51" t="n">
         <f aca="false">SUM(AF6:AF370)</f>
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="AG4" s="51" t="n">
         <f aca="false">SUM(AG6:AG370)</f>
-        <v>4.8</v>
+        <v>8.6</v>
       </c>
       <c r="AH4" s="48" t="n">
         <f aca="false">SUM(AH6:AH370)</f>
-        <v>939.718</v>
+        <v>1187.646</v>
       </c>
       <c r="AI4" s="48" t="n">
         <f aca="false">SUM(AI6:AI370)</f>
-        <v>90.53704</v>
+        <v>115.5792</v>
       </c>
       <c r="AJ4" s="48" t="n">
         <f aca="false">SUM(AJ6:AJ370)</f>
-        <v>215.518</v>
+        <v>270.238</v>
       </c>
       <c r="AK4" s="48" t="n">
         <f aca="false">SUM(AK6:AK370)</f>
-        <v>38.688</v>
+        <v>69.316</v>
       </c>
       <c r="AL4" s="48" t="n">
         <f aca="false">SUM(AL6:AL370)</f>
-        <v>147.378513719008</v>
+        <v>186.061180165289</v>
       </c>
       <c r="AM4" s="48" t="n">
         <f aca="false">SUM(AM6:AM370)</f>
-        <v>223.88</v>
+        <v>252.17</v>
       </c>
       <c r="AN4" s="47" t="n">
         <f aca="false">SUM(AN6:AN370)</f>
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="AO4" s="48" t="n">
         <f aca="false">SUM(AO6:AO370)</f>
-        <v>31.35</v>
+        <v>41.8</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4980,7 +4983,9 @@
       <c r="C6" s="54" t="n">
         <v>4</v>
       </c>
-      <c r="D6" s="54"/>
+      <c r="D6" s="54" t="n">
+        <v>0</v>
+      </c>
       <c r="E6" s="54" t="n">
         <v>3</v>
       </c>
@@ -5117,7 +5122,9 @@
       <c r="C7" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="54"/>
+      <c r="D7" s="54" t="n">
+        <v>0</v>
+      </c>
       <c r="E7" s="54" t="n">
         <v>2</v>
       </c>
@@ -5125,7 +5132,9 @@
         <v>1</v>
       </c>
       <c r="G7" s="54"/>
-      <c r="H7" s="54"/>
+      <c r="H7" s="54" t="n">
+        <v>1</v>
+      </c>
       <c r="I7" s="54"/>
       <c r="J7" s="54"/>
       <c r="K7" s="54" t="n">
@@ -5135,7 +5144,7 @@
         <v>22.11</v>
       </c>
       <c r="M7" s="55" t="n">
-        <v>37.91</v>
+        <v>30.71</v>
       </c>
       <c r="N7" s="55" t="n">
         <v>70.18</v>
@@ -5147,7 +5156,7 @@
       </c>
       <c r="Q7" s="31" t="n">
         <f aca="false">AA7+AB7+AC7</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R7" s="32" t="n">
         <f aca="false">B7*P1_PVP+C7*P2_PVP+D7*P3_PVP</f>
@@ -5167,7 +5176,7 @@
       </c>
       <c r="V7" s="34" t="n">
         <f aca="false">IF(E7+F7+G7+H7+I7+J7&gt;0,(E7+F7+G7)/(E7+F7+G7+H7+I7+J7),"")</f>
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="W7" s="33" t="n">
         <f aca="false">E7*(P1_PVP-P1_CPROD)+F7*(P2_PVP-P2_CPROD)+G7*(P3_PVP-P3_CPROD)-IF(ISNUMBER(L7),L7,E7*P1_LOG+F7*P2_LOG+G7*P3_LOG)</f>
@@ -5175,15 +5184,15 @@
       </c>
       <c r="X7" s="33" t="n">
         <f aca="false">W7-(E7*P1_IVAN+F7*P2_IVAN+G7*P3_IVAN)-(H7+I7+J7)*(COSTE_DEV-IVA_DEV)-AM7-AO7</f>
-        <v>-25.2301652892562</v>
+        <v>-33.2901652892562</v>
       </c>
       <c r="Y7" s="33" t="n">
         <f aca="false">AH7-AI7-AJ7-AK7-AL7-AM7-AO7</f>
-        <v>27.5623305785124</v>
+        <v>8.63823140495868</v>
       </c>
       <c r="AA7" s="58" t="n">
         <f aca="false">MAX(0,B7-E7-H7)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AB7" s="58" t="n">
         <f aca="false">MAX(0,C7-F7-I7)</f>
@@ -5195,7 +5204,7 @@
       </c>
       <c r="AD7" s="59" t="n">
         <f aca="false">E7+AA7*TASA_USADA</f>
-        <v>6</v>
+        <v>5.2</v>
       </c>
       <c r="AE7" s="59" t="n">
         <f aca="false">F7+AB7*TASA_USADA</f>
@@ -5207,27 +5216,27 @@
       </c>
       <c r="AG7" s="59" t="n">
         <f aca="false">H7+I7+J7+(AA7+AB7+AC7)*(1-TASA_USADA)</f>
-        <v>1</v>
+        <v>1.8</v>
       </c>
       <c r="AH7" s="60" t="n">
         <f aca="false">AD7*P1_PVP+AE7*P2_PVP+AF7*P3_PVP</f>
-        <v>219.93</v>
+        <v>195.938</v>
       </c>
       <c r="AI7" s="60" t="n">
         <f aca="false">AD7*P1_CPROD+AE7*P2_CPROD+AF7*P3_CPROD</f>
-        <v>19.2632</v>
+        <v>17.33688</v>
       </c>
       <c r="AJ7" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L7),L7,E7*P1_LOG+F7*P2_LOG+G7*P3_LOG)+IF(ISNUMBER(M7),M7,AA7*P1_LOG+AB7*P2_LOG+AC7*P3_LOG)*TASA_USADA</f>
-        <v>52.438</v>
+        <v>46.678</v>
       </c>
       <c r="AK7" s="60" t="n">
         <f aca="false">AG7*COSTE_DEV</f>
-        <v>8.06</v>
+        <v>14.508</v>
       </c>
       <c r="AL7" s="60" t="n">
         <f aca="false">AD7*P1_IVAN+AE7*P2_IVAN+AF7*P3_IVAN-AG7*IVA_DEV</f>
-        <v>34.8264694214876</v>
+        <v>30.9968885950413</v>
       </c>
       <c r="AM7" s="60" t="n">
         <f aca="false">N7*(1+RECARGO_ADS)</f>
@@ -5235,7 +5244,7 @@
       </c>
       <c r="AN7" s="58" t="n">
         <f aca="false">IF(ISNUMBER(L7),E7+F7+G7+AA7+AB7+AC7,0)</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AO7" s="60" t="n">
         <f aca="false">P7*COMISION</f>
@@ -5252,7 +5261,9 @@
       <c r="C8" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="54"/>
+      <c r="D8" s="54" t="n">
+        <v>0</v>
+      </c>
       <c r="E8" s="54" t="n">
         <v>1</v>
       </c>
@@ -5378,56 +5389,64 @@
         <v>46303</v>
       </c>
       <c r="B9" s="54" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C9" s="54" t="n">
-        <v>5</v>
-      </c>
-      <c r="D9" s="54"/>
+        <v>6</v>
+      </c>
+      <c r="D9" s="54" t="n">
+        <v>1</v>
+      </c>
       <c r="E9" s="54"/>
       <c r="F9" s="54"/>
       <c r="G9" s="54"/>
       <c r="H9" s="54"/>
-      <c r="I9" s="54"/>
+      <c r="I9" s="54" t="n">
+        <v>1</v>
+      </c>
       <c r="J9" s="54"/>
-      <c r="K9" s="54"/>
+      <c r="K9" s="54" t="n">
+        <v>1</v>
+      </c>
       <c r="L9" s="55" t="n">
         <v>0</v>
       </c>
       <c r="M9" s="55" t="n">
-        <v>67.54</v>
+        <v>110.9</v>
       </c>
       <c r="N9" s="55" t="n">
-        <v>38.25</v>
-      </c>
-      <c r="O9" s="56"/>
+        <v>50.41</v>
+      </c>
+      <c r="O9" s="56" t="s">
+        <v>107</v>
+      </c>
       <c r="P9" s="31" t="n">
         <f aca="false">B9+C9+D9</f>
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="Q9" s="31" t="n">
         <f aca="false">AA9+AB9+AC9</f>
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="R9" s="32" t="n">
         <f aca="false">B9*P1_PVP+C9*P2_PVP+D9*P3_PVP</f>
-        <v>319.91</v>
+        <v>559.84</v>
       </c>
       <c r="S9" s="32" t="n">
         <f aca="false">IF(P9&gt;0,R9/P9,"")</f>
-        <v>35.5455555555556</v>
+        <v>34.99</v>
       </c>
       <c r="T9" s="32" t="n">
         <f aca="false">IF(P9&gt;0,N9/P9,"")</f>
-        <v>4.25</v>
+        <v>3.150625</v>
       </c>
       <c r="U9" s="57" t="n">
         <f aca="false">IF(N9&gt;0,R9/N9,"")</f>
-        <v>8.36366013071896</v>
-      </c>
-      <c r="V9" s="34" t="str">
+        <v>11.1057329894862</v>
+      </c>
+      <c r="V9" s="34" t="n">
         <f aca="false">IF(E9+F9+G9+H9+I9+J9&gt;0,(E9+F9+G9)/(E9+F9+G9+H9+I9+J9),"")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="W9" s="33" t="n">
         <f aca="false">E9*(P1_PVP-P1_CPROD)+F9*(P2_PVP-P2_CPROD)+G9*(P3_PVP-P3_CPROD)-IF(ISNUMBER(L9),L9,E9*P1_LOG+F9*P2_LOG+G9*P3_LOG)</f>
@@ -5435,15 +5454,15 @@
       </c>
       <c r="X9" s="33" t="n">
         <f aca="false">W9-(E9*P1_IVAN+F9*P2_IVAN+G9*P3_IVAN)-(H9+I9+J9)*(COSTE_DEV-IVA_DEV)-AM9-AO9</f>
-        <v>-46.8</v>
+        <v>-73.67</v>
       </c>
       <c r="Y9" s="33" t="n">
         <f aca="false">AH9-AI9-AJ9-AK9-AL9-AM9-AO9</f>
-        <v>73.8827438016529</v>
+        <v>122.108479338843</v>
       </c>
       <c r="AA9" s="58" t="n">
         <f aca="false">MAX(0,B9-E9-H9)</f>
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="AB9" s="58" t="n">
         <f aca="false">MAX(0,C9-F9-I9)</f>
@@ -5451,11 +5470,11 @@
       </c>
       <c r="AC9" s="58" t="n">
         <f aca="false">MAX(0,D9-G9-J9)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD9" s="59" t="n">
         <f aca="false">E9+AA9*TASA_USADA</f>
-        <v>3.2</v>
+        <v>7.2</v>
       </c>
       <c r="AE9" s="59" t="n">
         <f aca="false">F9+AB9*TASA_USADA</f>
@@ -5463,52 +5482,58 @@
       </c>
       <c r="AF9" s="59" t="n">
         <f aca="false">G9+AC9*TASA_USADA</f>
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="AG9" s="59" t="n">
         <f aca="false">H9+I9+J9+(AA9+AB9+AC9)*(1-TASA_USADA)</f>
-        <v>1.8</v>
+        <v>4</v>
       </c>
       <c r="AH9" s="60" t="n">
         <f aca="false">AD9*P1_PVP+AE9*P2_PVP+AF9*P3_PVP</f>
-        <v>255.928</v>
+        <v>415.88</v>
       </c>
       <c r="AI9" s="60" t="n">
         <f aca="false">AD9*P1_CPROD+AE9*P2_CPROD+AF9*P3_CPROD</f>
-        <v>26.96848</v>
+        <v>42.37904</v>
       </c>
       <c r="AJ9" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L9),L9,E9*P1_LOG+F9*P2_LOG+G9*P3_LOG)+IF(ISNUMBER(M9),M9,AA9*P1_LOG+AB9*P2_LOG+AC9*P3_LOG)*TASA_USADA</f>
-        <v>54.032</v>
+        <v>88.72</v>
       </c>
       <c r="AK9" s="60" t="n">
         <f aca="false">AG9*COSTE_DEV</f>
-        <v>14.508</v>
+        <v>32.24</v>
       </c>
       <c r="AL9" s="60" t="n">
         <f aca="false">AD9*P1_IVAN+AE9*P2_IVAN+AF9*P3_IVAN-AG9*IVA_DEV</f>
-        <v>39.7367761983471</v>
+        <v>64.822480661157</v>
       </c>
       <c r="AM9" s="60" t="n">
         <f aca="false">N9*(1+RECARGO_ADS)</f>
-        <v>38.25</v>
+        <v>50.41</v>
       </c>
       <c r="AN9" s="58" t="n">
         <f aca="false">IF(ISNUMBER(L9),E9+F9+G9+AA9+AB9+AC9,0)</f>
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="AO9" s="60" t="n">
         <f aca="false">P9*COMISION</f>
-        <v>8.55</v>
+        <v>15.2</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="53" t="n">
         <v>46304</v>
       </c>
-      <c r="B10" s="54"/>
-      <c r="C10" s="54"/>
-      <c r="D10" s="54"/>
+      <c r="B10" s="54" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" s="54" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="54" t="n">
+        <v>0</v>
+      </c>
       <c r="E10" s="54"/>
       <c r="F10" s="54"/>
       <c r="G10" s="54"/>
@@ -5516,33 +5541,39 @@
       <c r="I10" s="54"/>
       <c r="J10" s="54"/>
       <c r="K10" s="54"/>
-      <c r="L10" s="55"/>
-      <c r="M10" s="55"/>
-      <c r="N10" s="55"/>
+      <c r="L10" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="55" t="n">
+        <v>32.24</v>
+      </c>
+      <c r="N10" s="55" t="n">
+        <v>16.13</v>
+      </c>
       <c r="O10" s="56"/>
       <c r="P10" s="31" t="n">
         <f aca="false">B10+C10+D10</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Q10" s="31" t="n">
         <f aca="false">AA10+AB10+AC10</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="R10" s="32" t="n">
         <f aca="false">B10*P1_PVP+C10*P2_PVP+D10*P3_PVP</f>
-        <v>0</v>
-      </c>
-      <c r="S10" s="32" t="str">
+        <v>139.96</v>
+      </c>
+      <c r="S10" s="32" t="n">
         <f aca="false">IF(P10&gt;0,R10/P10,"")</f>
-        <v/>
-      </c>
-      <c r="T10" s="32" t="str">
+        <v>34.99</v>
+      </c>
+      <c r="T10" s="32" t="n">
         <f aca="false">IF(P10&gt;0,N10/P10,"")</f>
-        <v/>
-      </c>
-      <c r="U10" s="57" t="str">
+        <v>4.0325</v>
+      </c>
+      <c r="U10" s="57" t="n">
         <f aca="false">IF(N10&gt;0,R10/N10,"")</f>
-        <v/>
+        <v>8.6769993800372</v>
       </c>
       <c r="V10" s="34" t="str">
         <f aca="false">IF(E10+F10+G10+H10+I10+J10&gt;0,(E10+F10+G10)/(E10+F10+G10+H10+I10+J10),"")</f>
@@ -5554,19 +5585,19 @@
       </c>
       <c r="X10" s="33" t="n">
         <f aca="false">W10-(E10*P1_IVAN+F10*P2_IVAN+G10*P3_IVAN)-(H10+I10+J10)*(COSTE_DEV-IVA_DEV)-AM10-AO10</f>
-        <v>0</v>
+        <v>-19.93</v>
       </c>
       <c r="Y10" s="33" t="n">
         <f aca="false">AH10-AI10-AJ10-AK10-AL10-AM10-AO10</f>
-        <v>0</v>
+        <v>30.8135371900827</v>
       </c>
       <c r="AA10" s="58" t="n">
         <f aca="false">MAX(0,B10-E10-H10)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AB10" s="58" t="n">
         <f aca="false">MAX(0,C10-F10-I10)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AC10" s="58" t="n">
         <f aca="false">MAX(0,D10-G10-J10)</f>
@@ -5574,11 +5605,11 @@
       </c>
       <c r="AD10" s="59" t="n">
         <f aca="false">E10+AA10*TASA_USADA</f>
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="AE10" s="59" t="n">
         <f aca="false">F10+AB10*TASA_USADA</f>
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="AF10" s="59" t="n">
         <f aca="false">G10+AC10*TASA_USADA</f>
@@ -5586,39 +5617,39 @@
       </c>
       <c r="AG10" s="59" t="n">
         <f aca="false">H10+I10+J10+(AA10+AB10+AC10)*(1-TASA_USADA)</f>
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="AH10" s="60" t="n">
         <f aca="false">AD10*P1_PVP+AE10*P2_PVP+AF10*P3_PVP</f>
-        <v>0</v>
+        <v>111.968</v>
       </c>
       <c r="AI10" s="60" t="n">
         <f aca="false">AD10*P1_CPROD+AE10*P2_CPROD+AF10*P3_CPROD</f>
-        <v>0</v>
+        <v>11.55792</v>
       </c>
       <c r="AJ10" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L10),L10,E10*P1_LOG+F10*P2_LOG+G10*P3_LOG)+IF(ISNUMBER(M10),M10,AA10*P1_LOG+AB10*P2_LOG+AC10*P3_LOG)*TASA_USADA</f>
-        <v>0</v>
+        <v>25.792</v>
       </c>
       <c r="AK10" s="60" t="n">
         <f aca="false">AG10*COSTE_DEV</f>
-        <v>0</v>
+        <v>6.448</v>
       </c>
       <c r="AL10" s="60" t="n">
         <f aca="false">AD10*P1_IVAN+AE10*P2_IVAN+AF10*P3_IVAN-AG10*IVA_DEV</f>
-        <v>0</v>
+        <v>17.4265428099174</v>
       </c>
       <c r="AM10" s="60" t="n">
         <f aca="false">N10*(1+RECARGO_ADS)</f>
-        <v>0</v>
+        <v>16.13</v>
       </c>
       <c r="AN10" s="58" t="n">
         <f aca="false">IF(ISNUMBER(L10),E10+F10+G10+AA10+AB10+AC10,0)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AO10" s="60" t="n">
         <f aca="false">P10*COMISION</f>
-        <v>0</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48515,12 +48546,12 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48528,13 +48559,13 @@
         <v>49</v>
       </c>
       <c r="B4" s="52" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C4" s="52" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D4" s="52" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E4" s="52" t="s">
         <v>84</v>
@@ -50673,34 +50704,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="62" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C4" s="29" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D4" s="29" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E4" s="29" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F4" s="29" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="63" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C5" s="64" t="n">
         <v>29.99</v>
@@ -50712,12 +50743,12 @@
         <v>49.99</v>
       </c>
       <c r="F5" s="65" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="63" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C6" s="66" t="n">
         <v>1</v>
@@ -50729,12 +50760,12 @@
         <v>3</v>
       </c>
       <c r="F6" s="65" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="63" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C7" s="64" t="n">
         <v>1.99</v>
@@ -50746,12 +50777,12 @@
         <v>1.99</v>
       </c>
       <c r="F7" s="65" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="63" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C8" s="64" t="n">
         <v>8.06</v>
@@ -50763,12 +50794,12 @@
         <v>8.06</v>
       </c>
       <c r="F8" s="65" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="63" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C9" s="32" t="n">
         <f aca="false">C6*C7*(1+IVA_PROD)</f>
@@ -50783,12 +50814,12 @@
         <v>7.2237</v>
       </c>
       <c r="F9" s="67" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="63" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C10" s="32" t="n">
         <f aca="false">C9+C8</f>
@@ -50803,12 +50834,12 @@
         <v>15.2837</v>
       </c>
       <c r="F10" s="67" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="68" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C11" s="33" t="n">
         <f aca="false">C5-C10</f>
@@ -50823,12 +50854,12 @@
         <v>34.7063</v>
       </c>
       <c r="F11" s="67" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="63" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C12" s="32" t="n">
         <f aca="false">C5*IVA_VENTAS/(1+IVA_VENTAS)</f>
@@ -50843,12 +50874,12 @@
         <v>8.67595041322314</v>
       </c>
       <c r="F12" s="67" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="63" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C13" s="32" t="n">
         <f aca="false">C6*C7*IVA_PROD+IF(LOG_IVA=1,C8*IVA_VENTAS/(1+IVA_VENTAS),0)</f>
@@ -50863,12 +50894,12 @@
         <v>1.2537</v>
       </c>
       <c r="F13" s="67" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="63" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C14" s="32" t="n">
         <f aca="false">IF(APLICA_IVA=1,C12-C13,0)</f>
@@ -50883,12 +50914,12 @@
         <v>7.42225041322314</v>
       </c>
       <c r="F14" s="67" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="68" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C15" s="33" t="n">
         <f aca="false">C11-C14</f>
@@ -50903,113 +50934,113 @@
         <v>27.2840495867769</v>
       </c>
       <c r="F15" s="67" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="62" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C17" s="29" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D17" s="29"/>
       <c r="E17" s="29"/>
       <c r="F17" s="29" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="63" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C18" s="69" t="n">
         <v>0.21</v>
       </c>
       <c r="F18" s="65" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="63" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C19" s="69" t="n">
         <v>0.21</v>
       </c>
       <c r="F19" s="65" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="63" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C20" s="70" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F20" s="65" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="63" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C21" s="70" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F21" s="65" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="63" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C22" s="64" t="n">
         <v>8.06</v>
       </c>
       <c r="F22" s="65" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="63" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C23" s="69" t="n">
         <v>0</v>
       </c>
       <c r="F23" s="65" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="63" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C24" s="69" t="n">
         <v>0.8</v>
       </c>
       <c r="F24" s="65" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="63" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C25" s="66" t="n">
         <v>30</v>
       </c>
       <c r="F25" s="65" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="63" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C26" s="69" t="n">
         <v>0.3</v>
@@ -51018,7 +51049,7 @@
         <v>0.05</v>
       </c>
       <c r="F26" s="65" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51029,69 +51060,69 @@
         <v>10000</v>
       </c>
       <c r="F27" s="65" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="63" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C28" s="4" t="n">
         <v>46300</v>
       </c>
       <c r="F28" s="65" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="63" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C29" s="70" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F29" s="65" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="63" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C30" s="70" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F30" s="65" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="63" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C31" s="64" t="n">
         <v>0.95</v>
       </c>
       <c r="F31" s="65" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="62" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C32" s="29" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D32" s="29"/>
       <c r="E32" s="29"/>
       <c r="F32" s="29" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="63" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C33" s="31" t="n">
         <f aca="false">IF(C20="SÍ",1,0)</f>
@@ -51101,7 +51132,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="63" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C34" s="31" t="n">
         <f aca="false">IF(C21="SÍ",1,0)</f>
@@ -51111,7 +51142,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="63" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C35" s="32" t="n">
         <f aca="false">IF(AND(APLICA_IVA=1,LOG_IVA=1),C22*IVA_VENTAS/(1+IVA_VENTAS),0)</f>
@@ -51121,7 +51152,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="63" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C36" s="32" t="n">
         <f aca="false">C22-C35</f>
@@ -51131,138 +51162,138 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="63" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C37" s="31" t="n">
         <f aca="false">(SUM(Diario!$E$6:$E$370)+SUM(Diario!$F$6:$F$370)+SUM(Diario!$G$6:$G$370))+(SUM(Diario!$H$6:$H$370)+SUM(Diario!$I$6:$I$370)+SUM(Diario!$J$6:$J$370))</f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F37" s="67" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="63" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C38" s="34" t="n">
         <f aca="false">IF(C37&gt;0,(SUM(Diario!$E$6:$E$370)+SUM(Diario!$F$6:$F$370)+SUM(Diario!$G$6:$G$370))/C37,"")</f>
-        <v>1</v>
+        <v>0.818181818181818</v>
       </c>
       <c r="F38" s="67" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="63" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C39" s="34" t="n">
         <f aca="false">IF(AND(C37&gt;=C25,C38&lt;&gt;""),C38,C24)</f>
         <v>0.8</v>
       </c>
       <c r="F39" s="67" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="63" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C40" s="34" t="n">
         <f aca="false">IF(SUM(Diario!$P$6:$P$370)&gt;0,SUM(Diario!$C$6:$C$370)/SUM(Diario!$P$6:$P$370),"")</f>
-        <v>0.333333333333333</v>
+        <v>0.318181818181818</v>
       </c>
       <c r="D40" s="34" t="n">
         <f aca="false">IF(SUM(Diario!$P$6:$P$370)&gt;0,SUM(Diario!$D$6:$D$370)/SUM(Diario!$P$6:$P$370),"")</f>
-        <v>0</v>
+        <v>0.0227272727272727</v>
       </c>
       <c r="F40" s="67" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="63" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C41" s="34" t="n">
         <f aca="false">IF(C40="",C26,C40)</f>
-        <v>0.333333333333333</v>
+        <v>0.318181818181818</v>
       </c>
       <c r="D41" s="34" t="n">
         <f aca="false">IF(D40="",D26,D40)</f>
-        <v>0</v>
+        <v>0.0227272727272727</v>
       </c>
       <c r="F41" s="67"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="63" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C42" s="32" t="n">
         <f aca="false">IF(SUM(Diario!$AN$6:$AN$370)&gt;0,(SUM(Diario!$L$6:$L$370)+SUM(Diario!$M$6:$M$370))/SUM(Diario!$AN$6:$AN$370),"")</f>
-        <v>7.64393939393939</v>
+        <v>7.63452380952381</v>
       </c>
       <c r="F42" s="67" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="63" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C43" s="32" t="n">
         <f aca="false">(1-C41-D41)*C5+C41*D5+D41*E5</f>
-        <v>33.3233333333333</v>
+        <v>33.6263636363636</v>
       </c>
       <c r="F43" s="67"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="63" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C44" s="32" t="n">
         <f aca="false">(1-C41-D41)*(C5-C9-IF(C42="",C8,C42)-C14)+C41*(D5-D9-IF(C42="",D8,C42)-D14)+D41*(E5-E9-IF(C42="",E8,C42)-E14)</f>
-        <v>17.2426721763085</v>
+        <v>17.4422229973883</v>
       </c>
       <c r="F44" s="67" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="63" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C45" s="32" t="n">
         <f aca="false">C39*C44-(1-C39)*C36-COMISION</f>
-        <v>11.2321377410468</v>
+        <v>11.3917783979106</v>
       </c>
       <c r="F45" s="67" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="68" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C46" s="33" t="n">
         <f aca="false">C45/(1+RECARGO_ADS)</f>
-        <v>11.2321377410468</v>
+        <v>11.3917783979106</v>
       </c>
       <c r="F46" s="67" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="68" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C47" s="72" t="n">
         <f aca="false">IF(C46&gt;0,C43/C46,"")</f>
-        <v>2.96678460517415</v>
+        <v>2.95180984582101</v>
       </c>
       <c r="F47" s="67" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -51296,147 +51327,147 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="73" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="74" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="74" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="74" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="74" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="73" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="74" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="74" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="74" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="73" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="74" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="74" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="74" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="73" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="74" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="74" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="74" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="73" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="74" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="74" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="74" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="73" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="74" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="74" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="74" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="74" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="73" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="74" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Contabilidad al 10/10 con el export del almacén subido desde el panel
55 pedidos (5-10 oct), 10 entregados, 2 devueltos, 8 en incidencia.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFjE4yx23BY3D6kaMQowKe
</commit_message>
<xml_diff>
--- a/contabilidad/CeraLux_Contabilidad.xlsx
+++ b/contabilidad/CeraLux_Contabilidad.xlsx
@@ -1779,46 +1779,46 @@
               <c:strCache>
                 <c:ptCount val="14"/>
                 <c:pt idx="0">
-                  <c:v>Sat 26/09</c:v>
+                  <c:v>Sun 27/09</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Sun 27/09</c:v>
+                  <c:v>Mon 28/09</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Mon 28/09</c:v>
+                  <c:v>Tue 29/09</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Tue 29/09</c:v>
+                  <c:v>Wed 30/09</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Wed 30/09</c:v>
+                  <c:v>Thu 01/10</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Thu 01/10</c:v>
+                  <c:v>Fri 02/10</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Fri 02/10</c:v>
+                  <c:v>Sat 03/10</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>Sat 03/10</c:v>
+                  <c:v>Sun 04/10</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Sun 04/10</c:v>
+                  <c:v>Mon 05/10</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Mon 05/10</c:v>
+                  <c:v>Tue 06/10</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Tue 06/10</c:v>
+                  <c:v>Wed 07/10</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>Wed 07/10</c:v>
+                  <c:v>Thu 08/10</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>Thu 08/10</c:v>
+                  <c:v>Fri 09/10</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>Fri 09/10</c:v>
+                  <c:v>Sat 10/10</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1854,22 +1854,22 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>62.6280826446281</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>62.6280826446281</c:v>
+                  <c:v>8.63823140495868</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>8.63823140495868</c:v>
+                  <c:v>28.2932892561984</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>28.2932892561984</c:v>
+                  <c:v>128.044396694215</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>122.108479338843</c:v>
+                  <c:v>36.5688760330579</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>30.8135371900827</c:v>
+                  <c:v>43.5711735537191</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1877,8 +1877,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="52780188"/>
-        <c:axId val="78457029"/>
+        <c:axId val="67286432"/>
+        <c:axId val="90468839"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -1942,46 +1942,46 @@
               <c:strCache>
                 <c:ptCount val="14"/>
                 <c:pt idx="0">
-                  <c:v>Sat 26/09</c:v>
+                  <c:v>Sun 27/09</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Sun 27/09</c:v>
+                  <c:v>Mon 28/09</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Mon 28/09</c:v>
+                  <c:v>Tue 29/09</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Tue 29/09</c:v>
+                  <c:v>Wed 30/09</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Wed 30/09</c:v>
+                  <c:v>Thu 01/10</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Thu 01/10</c:v>
+                  <c:v>Fri 02/10</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Fri 02/10</c:v>
+                  <c:v>Sat 03/10</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>Sat 03/10</c:v>
+                  <c:v>Sun 04/10</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Sun 04/10</c:v>
+                  <c:v>Mon 05/10</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Mon 05/10</c:v>
+                  <c:v>Tue 06/10</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Tue 06/10</c:v>
+                  <c:v>Wed 07/10</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>Wed 07/10</c:v>
+                  <c:v>Thu 08/10</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>Thu 08/10</c:v>
+                  <c:v>Fri 09/10</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>Fri 09/10</c:v>
+                  <c:v>Sat 10/10</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2017,22 +2017,22 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>67.67</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>67.67</c:v>
+                  <c:v>70.18</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>70.18</c:v>
+                  <c:v>47.78</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>47.78</c:v>
+                  <c:v>50.46</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>50.41</c:v>
+                  <c:v>41.21</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>16.13</c:v>
+                  <c:v>63.39</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2047,11 +2047,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="52780188"/>
-        <c:axId val="78457029"/>
+        <c:axId val="67286432"/>
+        <c:axId val="90468839"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="52780188"/>
+        <c:axId val="67286432"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2083,7 +2083,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78457029"/>
+        <c:crossAx val="90468839"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2091,7 +2091,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="78457029"/>
+        <c:axId val="90468839"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2133,7 +2133,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52780188"/>
+        <c:crossAx val="67286432"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2332,7 +2332,7 @@
                 <c:formatCode>#,##0" €";[RED]\-#,##0" €";\-</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>252.481619834711</c:v>
+                  <c:v>307.744049586777</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -2373,8 +2373,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="83250474"/>
-        <c:axId val="45140102"/>
+        <c:axId val="46058975"/>
+        <c:axId val="3194225"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2471,11 +2471,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="83250474"/>
-        <c:axId val="45140102"/>
+        <c:axId val="46058975"/>
+        <c:axId val="3194225"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="83250474"/>
+        <c:axId val="46058975"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2507,7 +2507,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="45140102"/>
+        <c:crossAx val="3194225"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2515,7 +2515,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="45140102"/>
+        <c:axId val="3194225"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2557,7 +2557,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83250474"/>
+        <c:crossAx val="46058975"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="F3" s="4" t="n">
         <f aca="true">TODAY()</f>
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="G3" s="4"/>
       <c r="H3" s="3" t="s">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="I3" s="5" t="n">
         <f aca="false">MAX(1,$F$3-$C$3+1)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J3" s="6" t="s">
         <v>5</v>
@@ -2951,32 +2951,32 @@
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="10" t="n">
         <f aca="false">F25</f>
-        <v>252.481619834711</v>
+        <v>307.744049586777</v>
       </c>
       <c r="C7" s="10"/>
       <c r="D7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$W$6:$W$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>202.4252</v>
+        <v>230.3994</v>
       </c>
       <c r="E7" s="10"/>
       <c r="F7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$X$6:$X$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+F24</f>
-        <v>-154.700495867769</v>
+        <v>-231.800909090909</v>
       </c>
       <c r="G7" s="10"/>
       <c r="H7" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="I7" s="11"/>
       <c r="J7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$R$6:$R$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>1479.56</v>
+        <v>1869.45</v>
       </c>
       <c r="K7" s="10"/>
       <c r="L7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>252.17</v>
+        <v>340.69</v>
       </c>
       <c r="M7" s="10"/>
     </row>
@@ -3009,32 +3009,32 @@
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="10" t="n">
         <f aca="false">IF(H7&gt;0,L7/H7,"")</f>
-        <v>5.73113636363636</v>
+        <v>6.19436363636364</v>
       </c>
       <c r="C10" s="10"/>
       <c r="D10" s="10" t="n">
         <f aca="false">CPA_BE</f>
-        <v>11.3917783979106</v>
+        <v>11.6204933104631</v>
       </c>
       <c r="E10" s="10"/>
       <c r="F10" s="12" t="n">
         <f aca="false">IF(L7&gt;0,J7/L7,"")</f>
-        <v>5.8673117341476</v>
+        <v>5.48724647039831</v>
       </c>
       <c r="G10" s="12"/>
       <c r="H10" s="12" t="n">
         <f aca="false">ROAS_BE</f>
-        <v>2.95180984582101</v>
+        <v>2.92500491088406</v>
       </c>
       <c r="I10" s="12"/>
       <c r="J10" s="10" t="n">
         <f aca="false">IF(H7&gt;0,J7/H7,"")</f>
-        <v>33.6263636363636</v>
+        <v>33.99</v>
       </c>
       <c r="K10" s="10"/>
       <c r="L10" s="13" t="n">
         <f aca="false">IF(H7&gt;0,(SUMIFS(Diario!$C$6:$C$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+SUMIFS(Diario!$D$6:$D$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3))/H7,"")</f>
-        <v>0.340909090909091</v>
+        <v>0.363636363636364</v>
       </c>
       <c r="M10" s="13"/>
     </row>
@@ -3067,17 +3067,17 @@
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C13" s="11"/>
       <c r="D13" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$Q$6:$Q$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="E13" s="11"/>
       <c r="F13" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$K$6:$K$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G13" s="11"/>
       <c r="H13" s="11" t="n">
@@ -3087,7 +3087,7 @@
       <c r="I13" s="11"/>
       <c r="J13" s="13" t="n">
         <f aca="false">IF(B13+H13&gt;0,B13/(B13+H13),"")</f>
-        <v>0.818181818181818</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="K13" s="13"/>
       <c r="L13" s="14" t="str">
@@ -3124,7 +3124,7 @@
       </c>
       <c r="F16" s="17" t="n">
         <f aca="false">SUMIFS(Diario!$AH$6:$AH$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>1187.646</v>
+        <v>1507.556</v>
       </c>
       <c r="H16" s="15" t="s">
         <v>29</v>
@@ -3146,11 +3146,11 @@
       <c r="D17" s="15"/>
       <c r="E17" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F17/$F$16,"")</f>
-        <v>-0.0973178876533916</v>
+        <v>-0.0990276978102306</v>
       </c>
       <c r="F17" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AI$6:$AI$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-115.5792</v>
+        <v>-149.2898</v>
       </c>
       <c r="H17" s="15" t="s">
         <v>31</v>
@@ -3160,7 +3160,7 @@
       <c r="K17" s="15"/>
       <c r="L17" s="20" t="n">
         <f aca="false">F25/I3</f>
-        <v>28.0535133149679</v>
+        <v>30.7744049586777</v>
       </c>
       <c r="M17" s="20"/>
     </row>
@@ -3172,11 +3172,11 @@
       <c r="D18" s="15"/>
       <c r="E18" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F18/$F$16,"")</f>
-        <v>-0.227540866554512</v>
+        <v>-0.22315190944814</v>
       </c>
       <c r="F18" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AJ$6:$AJ$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-270.238</v>
+        <v>-336.414</v>
       </c>
       <c r="H18" s="15" t="s">
         <v>33</v>
@@ -3186,7 +3186,7 @@
       <c r="K18" s="15"/>
       <c r="L18" s="18" t="n">
         <f aca="false">L17*30</f>
-        <v>841.605399449037</v>
+        <v>923.232148760331</v>
       </c>
       <c r="M18" s="18"/>
     </row>
@@ -3198,11 +3198,11 @@
       <c r="D19" s="15"/>
       <c r="E19" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F19/$F$16,"")</f>
-        <v>-0.0583641926971505</v>
+        <v>-0.0566718582924946</v>
       </c>
       <c r="F19" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AK$6:$AK$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-69.316</v>
+        <v>-85.436</v>
       </c>
       <c r="H19" s="21" t="s">
         <v>35</v>
@@ -3212,7 +3212,7 @@
       <c r="K19" s="21"/>
       <c r="L19" s="22" t="n">
         <f aca="false">IF(L16&gt;0,L18/L16,"")</f>
-        <v>0.0841605399449037</v>
+        <v>0.0923232148760331</v>
       </c>
       <c r="M19" s="22"/>
     </row>
@@ -3224,11 +3224,11 @@
       <c r="D20" s="15"/>
       <c r="E20" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F20/$F$16,"")</f>
-        <v>-0.0351956727846513</v>
+        <v>-0.0346587456784358</v>
       </c>
       <c r="F20" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AO$6:$AO$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-41.8</v>
+        <v>-52.25</v>
       </c>
       <c r="H20" s="15" t="s">
         <v>37</v>
@@ -3238,7 +3238,7 @@
       <c r="K20" s="15"/>
       <c r="L20" s="20" t="n">
         <f aca="false">BEN_PEDIDO</f>
-        <v>11.3917783979106</v>
+        <v>11.6204933104631</v>
       </c>
       <c r="M20" s="20"/>
     </row>
@@ -3250,11 +3250,11 @@
       <c r="D21" s="15"/>
       <c r="E21" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F21/$F$16,"")</f>
-        <v>-0.15666383767999</v>
+        <v>-0.156367093768472</v>
       </c>
       <c r="F21" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AL$6:$AL$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-186.061180165289</v>
+        <v>-235.732150413223</v>
       </c>
       <c r="H21" s="15" t="s">
         <v>39</v>
@@ -3264,7 +3264,7 @@
       <c r="K21" s="15"/>
       <c r="L21" s="20" t="n">
         <f aca="false">B10</f>
-        <v>5.73113636363636</v>
+        <v>6.19436363636364</v>
       </c>
       <c r="M21" s="20"/>
     </row>
@@ -3276,11 +3276,11 @@
       <c r="D22" s="15"/>
       <c r="E22" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F22/$F$16,"")</f>
-        <v>-0.212327579093434</v>
+        <v>-0.225988288328924</v>
       </c>
       <c r="F22" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AM$6:$AM$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-252.17</v>
+        <v>-340.69</v>
       </c>
       <c r="H22" s="15" t="s">
         <v>41</v>
@@ -3290,7 +3290,7 @@
       <c r="K22" s="15"/>
       <c r="L22" s="20" t="n">
         <f aca="false">IF(ISNUMBER(L21),L20-L21*(1+RECARGO_ADS),"")</f>
-        <v>5.66064203427427</v>
+        <v>5.42612967409949</v>
       </c>
       <c r="M22" s="20"/>
     </row>
@@ -3302,11 +3302,11 @@
       <c r="D23" s="23"/>
       <c r="E23" s="24" t="n">
         <f aca="false">IF($F$16&gt;0,F23/$F$16,"")</f>
-        <v>0.212589963536871</v>
+        <v>0.204134406673302</v>
       </c>
       <c r="F23" s="25" t="n">
         <f aca="false">SUM(F16:F22)</f>
-        <v>252.481619834711</v>
+        <v>307.744049586777</v>
       </c>
       <c r="H23" s="21" t="s">
         <v>43</v>
@@ -3316,7 +3316,7 @@
       <c r="K23" s="21"/>
       <c r="L23" s="26" t="n">
         <f aca="false">IF(NOT(ISNUMBER(L22)),"",IF(L22&lt;=0,"Baja el CPA",ROUNDUP((L16-F24/I3*30)/30/L22,0)))</f>
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="M23" s="26"/>
     </row>
@@ -3342,7 +3342,7 @@
       <c r="K24" s="15"/>
       <c r="L24" s="18" t="n">
         <f aca="false">IF(ISNUMBER(L23),L23*L21,"")</f>
-        <v>338.137045454545</v>
+        <v>384.050545454545</v>
       </c>
       <c r="M24" s="18"/>
     </row>
@@ -3354,11 +3354,11 @@
       <c r="D25" s="23"/>
       <c r="E25" s="24" t="n">
         <f aca="false">IF($F$16&gt;0,F25/$F$16,"")</f>
-        <v>0.212589963536871</v>
+        <v>0.204134406673302</v>
       </c>
       <c r="F25" s="25" t="n">
         <f aca="false">F23+F24</f>
-        <v>252.481619834711</v>
+        <v>307.744049586777</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3369,7 +3369,7 @@
       <c r="D26" s="27"/>
       <c r="F26" s="28" t="n">
         <f aca="false">IF(F16&gt;0,F25/F16,"")</f>
-        <v>0.212589963536871</v>
+        <v>0.204134406673302</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3405,7 +3405,7 @@
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="30" t="n">
         <f aca="false">$F$3-13</f>
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="C29" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B29)</f>
@@ -3431,7 +3431,7 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="30" t="n">
         <f aca="false">$F$3-12</f>
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="C30" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B30)</f>
@@ -3457,7 +3457,7 @@
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="30" t="n">
         <f aca="false">$F$3-11</f>
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="C31" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B31)</f>
@@ -3483,7 +3483,7 @@
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="30" t="n">
         <f aca="false">$F$3-10</f>
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="C32" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B32)</f>
@@ -3509,7 +3509,7 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="30" t="n">
         <f aca="false">$F$3-9</f>
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="C33" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B33)</f>
@@ -3535,7 +3535,7 @@
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="30" t="n">
         <f aca="false">$F$3-8</f>
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="C34" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B34)</f>
@@ -3561,7 +3561,7 @@
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="30" t="n">
         <f aca="false">$F$3-7</f>
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="C35" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B35)</f>
@@ -3587,7 +3587,7 @@
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="30" t="n">
         <f aca="false">$F$3-6</f>
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="C36" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B36)</f>
@@ -3613,153 +3613,153 @@
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="30" t="n">
         <f aca="false">$F$3-5</f>
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="C37" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B37)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D37" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B37)</f>
-        <v>0</v>
-      </c>
-      <c r="E37" s="32" t="str">
+        <v>67.67</v>
+      </c>
+      <c r="E37" s="32" t="n">
         <f aca="false">IF(C37&gt;0,D37/C37,"")</f>
-        <v/>
+        <v>7.51888888888889</v>
       </c>
       <c r="F37" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B37)</f>
-        <v>0</v>
-      </c>
-      <c r="G37" s="34" t="str">
+        <v>62.6280826446281</v>
+      </c>
+      <c r="G37" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B37))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B37))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B37)),"")</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="30" t="n">
         <f aca="false">$F$3-4</f>
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="C38" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B38)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D38" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B38)</f>
-        <v>67.67</v>
+        <v>70.18</v>
       </c>
       <c r="E38" s="32" t="n">
         <f aca="false">IF(C38&gt;0,D38/C38,"")</f>
-        <v>7.51888888888889</v>
+        <v>8.7725</v>
       </c>
       <c r="F38" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B38)</f>
-        <v>62.6280826446281</v>
+        <v>8.63823140495868</v>
       </c>
       <c r="G38" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B38))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B38))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B38)),"")</f>
-        <v>1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="30" t="n">
         <f aca="false">$F$3-3</f>
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="C39" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B39)</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D39" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B39)</f>
-        <v>70.18</v>
+        <v>47.78</v>
       </c>
       <c r="E39" s="32" t="n">
         <f aca="false">IF(C39&gt;0,D39/C39,"")</f>
-        <v>8.7725</v>
+        <v>6.82571428571429</v>
       </c>
       <c r="F39" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B39)</f>
-        <v>8.63823140495868</v>
+        <v>28.2932892561984</v>
       </c>
       <c r="G39" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B39))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B39))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B39)),"")</f>
-        <v>0.75</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="30" t="n">
         <f aca="false">$F$3-2</f>
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="C40" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B40)</f>
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="D40" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B40)</f>
-        <v>47.78</v>
+        <v>50.46</v>
       </c>
       <c r="E40" s="32" t="n">
         <f aca="false">IF(C40&gt;0,D40/C40,"")</f>
-        <v>6.82571428571429</v>
+        <v>3.15375</v>
       </c>
       <c r="F40" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B40)</f>
-        <v>28.2932892561984</v>
+        <v>128.044396694215</v>
       </c>
       <c r="G40" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B40))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B40))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B40)),"")</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="30" t="n">
         <f aca="false">$F$3-1</f>
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="C41" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B41)</f>
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D41" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B41)</f>
-        <v>50.41</v>
+        <v>41.21</v>
       </c>
       <c r="E41" s="32" t="n">
         <f aca="false">IF(C41&gt;0,D41/C41,"")</f>
-        <v>3.150625</v>
+        <v>6.86833333333333</v>
       </c>
       <c r="F41" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B41)</f>
-        <v>122.108479338843</v>
-      </c>
-      <c r="G41" s="34" t="n">
+        <v>36.5688760330579</v>
+      </c>
+      <c r="G41" s="34" t="str">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B41))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B41))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B41)),"")</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="30" t="n">
         <f aca="false">$F$3-0</f>
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="C42" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B42)</f>
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D42" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B42)</f>
-        <v>16.13</v>
+        <v>63.39</v>
       </c>
       <c r="E42" s="32" t="n">
         <f aca="false">IF(C42&gt;0,D42/C42,"")</f>
-        <v>4.0325</v>
+        <v>7.04333333333333</v>
       </c>
       <c r="F42" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B42)</f>
-        <v>30.8135371900827</v>
+        <v>43.5711735537191</v>
       </c>
       <c r="G42" s="34" t="str">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B42))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B42))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B42)),"")</f>
@@ -3830,23 +3830,23 @@
       </c>
       <c r="C47" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="D47" s="37" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>252.17</v>
+        <v>340.69</v>
       </c>
       <c r="E47" s="32" t="n">
         <f aca="false">IF(C47&gt;0,D47/C47,"")</f>
-        <v>5.73113636363636</v>
+        <v>6.19436363636364</v>
       </c>
       <c r="F47" s="37" t="n">
         <f aca="false">SUMIFS(Diario!$R$6:$R$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>1479.56</v>
+        <v>1869.45</v>
       </c>
       <c r="G47" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H47" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
@@ -3854,11 +3854,11 @@
       </c>
       <c r="I47" s="34" t="n">
         <f aca="false">IF(G47+H47&gt;0,G47/(G47+H47),"")</f>
-        <v>0.818181818181818</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="J47" s="37" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>252.481619834711</v>
+        <v>307.744049586777</v>
       </c>
       <c r="K47" s="37" t="n">
         <f aca="false">-SUMIFS(Gastos!$D$5:$D$304,Gastos!$A$5:$A$304,"&gt;="&amp;$B47,Gastos!$A$5:$A$304,"&lt;="&amp;EOMONTH($B47,0))</f>
@@ -3866,11 +3866,11 @@
       </c>
       <c r="L47" s="38" t="n">
         <f aca="false">J47+K47</f>
-        <v>252.481619834711</v>
+        <v>307.744049586777</v>
       </c>
       <c r="M47" s="34" t="n">
         <f aca="false">IF(OBJETIVO_MES&gt;0,L47/OBJETIVO_MES,"")</f>
-        <v>0.0252481619834711</v>
+        <v>0.0307744049586777</v>
       </c>
       <c r="O47" s="39" t="n">
         <f aca="false">OBJETIVO_MES</f>
@@ -4477,23 +4477,23 @@
       </c>
       <c r="C59" s="41" t="n">
         <f aca="false">SUM(C47:C58)</f>
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="D59" s="42" t="n">
         <f aca="false">SUM(D47:D58)</f>
-        <v>252.17</v>
+        <v>340.69</v>
       </c>
       <c r="E59" s="43" t="n">
         <f aca="false">IF(C59&gt;0,D59/C59,"")</f>
-        <v>5.73113636363636</v>
+        <v>6.19436363636364</v>
       </c>
       <c r="F59" s="42" t="n">
         <f aca="false">SUM(F47:F58)</f>
-        <v>1479.56</v>
+        <v>1869.45</v>
       </c>
       <c r="G59" s="41" t="n">
         <f aca="false">SUM(G47:G58)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H59" s="41" t="n">
         <f aca="false">SUM(H47:H58)</f>
@@ -4501,11 +4501,11 @@
       </c>
       <c r="I59" s="44" t="n">
         <f aca="false">IF(G59+H59&gt;0,G59/(G59+H59),"")</f>
-        <v>0.818181818181818</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="J59" s="42" t="n">
         <f aca="false">SUM(J47:J58)</f>
-        <v>252.481619834711</v>
+        <v>307.744049586777</v>
       </c>
       <c r="K59" s="42" t="n">
         <f aca="false">SUM(K47:K58)</f>
@@ -4513,7 +4513,7 @@
       </c>
       <c r="L59" s="42" t="n">
         <f aca="false">SUM(L47:L58)</f>
-        <v>252.481619834711</v>
+        <v>307.744049586777</v>
       </c>
       <c r="M59" s="45"/>
     </row>
@@ -4700,15 +4700,15 @@
       </c>
       <c r="B4" s="47" t="n">
         <f aca="false">SUM(B6:B370)</f>
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C4" s="47" t="n">
         <f aca="false">SUM(C6:C370)</f>
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D4" s="47" t="n">
         <f aca="false">SUM(D6:D370)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" s="47" t="n">
         <f aca="false">SUM(E6:E370)</f>
@@ -4716,7 +4716,7 @@
       </c>
       <c r="F4" s="47" t="n">
         <f aca="false">SUM(F6:F370)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4" s="47" t="n">
         <f aca="false">SUM(G6:G370)</f>
@@ -4736,119 +4736,119 @@
       </c>
       <c r="K4" s="47" t="n">
         <f aca="false">SUM(K6:K370)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L4" s="48" t="n">
         <f aca="false">SUM(L6:L370)</f>
-        <v>68.59</v>
+        <v>75.79</v>
       </c>
       <c r="M4" s="48" t="n">
         <f aca="false">SUM(M6:M370)</f>
-        <v>252.06</v>
+        <v>325.78</v>
       </c>
       <c r="N4" s="48" t="n">
         <f aca="false">SUM(N6:N370)</f>
-        <v>252.17</v>
+        <v>340.69</v>
       </c>
       <c r="P4" s="47" t="n">
         <f aca="false">SUM(P6:P370)</f>
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="Q4" s="47" t="n">
         <f aca="false">SUM(Q6:Q370)</f>
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="R4" s="48" t="n">
         <f aca="false">SUM(R6:R370)</f>
-        <v>1479.56</v>
+        <v>1869.45</v>
       </c>
       <c r="S4" s="48" t="n">
         <f aca="false">IF(P4&gt;0,R4/P4,"")</f>
-        <v>33.6263636363636</v>
+        <v>33.99</v>
       </c>
       <c r="T4" s="48" t="n">
         <f aca="false">IF(P4&gt;0,N4/P4,"")</f>
-        <v>5.73113636363636</v>
+        <v>6.19436363636364</v>
       </c>
       <c r="U4" s="49" t="n">
         <f aca="false">IF(N4&gt;0,R4/N4,"")</f>
-        <v>5.8673117341476</v>
+        <v>5.48724647039831</v>
       </c>
       <c r="V4" s="50" t="n">
         <f aca="false">IF(E4+F4+G4+H4+I4+J4&gt;0,(E4+F4+G4)/(E4+F4+G4+H4+I4+J4),"")</f>
-        <v>0.818181818181818</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="W4" s="48" t="n">
         <f aca="false">SUM(W6:W370)</f>
-        <v>202.4252</v>
+        <v>230.3994</v>
       </c>
       <c r="X4" s="48" t="n">
         <f aca="false">SUM(X6:X370)</f>
-        <v>-154.700495867769</v>
+        <v>-231.800909090909</v>
       </c>
       <c r="Y4" s="48" t="n">
         <f aca="false">SUM(Y6:Y370)</f>
-        <v>252.481619834711</v>
+        <v>307.744049586777</v>
       </c>
       <c r="AA4" s="47" t="n">
         <f aca="false">SUM(AA6:AA370)</f>
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="AB4" s="47" t="n">
         <f aca="false">SUM(AB6:AB370)</f>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="AC4" s="47" t="n">
         <f aca="false">SUM(AC6:AC370)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AD4" s="51" t="n">
         <f aca="false">SUM(AD6:AD370)</f>
-        <v>23.6</v>
+        <v>28.4</v>
       </c>
       <c r="AE4" s="51" t="n">
         <f aca="false">SUM(AE6:AE370)</f>
-        <v>11</v>
+        <v>14.4</v>
       </c>
       <c r="AF4" s="51" t="n">
         <f aca="false">SUM(AF6:AF370)</f>
-        <v>0.8</v>
+        <v>1.6</v>
       </c>
       <c r="AG4" s="51" t="n">
         <f aca="false">SUM(AG6:AG370)</f>
-        <v>8.6</v>
+        <v>10.6</v>
       </c>
       <c r="AH4" s="48" t="n">
         <f aca="false">SUM(AH6:AH370)</f>
-        <v>1187.646</v>
+        <v>1507.556</v>
       </c>
       <c r="AI4" s="48" t="n">
         <f aca="false">SUM(AI6:AI370)</f>
-        <v>115.5792</v>
+        <v>149.2898</v>
       </c>
       <c r="AJ4" s="48" t="n">
         <f aca="false">SUM(AJ6:AJ370)</f>
-        <v>270.238</v>
+        <v>336.414</v>
       </c>
       <c r="AK4" s="48" t="n">
         <f aca="false">SUM(AK6:AK370)</f>
-        <v>69.316</v>
+        <v>85.436</v>
       </c>
       <c r="AL4" s="48" t="n">
         <f aca="false">SUM(AL6:AL370)</f>
-        <v>186.061180165289</v>
+        <v>235.732150413223</v>
       </c>
       <c r="AM4" s="48" t="n">
         <f aca="false">SUM(AM6:AM370)</f>
-        <v>252.17</v>
+        <v>340.69</v>
       </c>
       <c r="AN4" s="47" t="n">
         <f aca="false">SUM(AN6:AN370)</f>
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="AO4" s="48" t="n">
         <f aca="false">SUM(AO6:AO370)</f>
-        <v>41.8</v>
+        <v>52.25</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5272,7 +5272,9 @@
       <c r="H8" s="54"/>
       <c r="I8" s="54"/>
       <c r="J8" s="54"/>
-      <c r="K8" s="54"/>
+      <c r="K8" s="54" t="n">
+        <v>1</v>
+      </c>
       <c r="L8" s="55" t="n">
         <v>8.06</v>
       </c>
@@ -5398,7 +5400,9 @@
         <v>1</v>
       </c>
       <c r="E9" s="54"/>
-      <c r="F9" s="54"/>
+      <c r="F9" s="54" t="n">
+        <v>1</v>
+      </c>
       <c r="G9" s="54"/>
       <c r="H9" s="54"/>
       <c r="I9" s="54" t="n">
@@ -5409,13 +5413,13 @@
         <v>1</v>
       </c>
       <c r="L9" s="55" t="n">
-        <v>0</v>
+        <v>7.2</v>
       </c>
       <c r="M9" s="55" t="n">
-        <v>110.9</v>
+        <v>103.7</v>
       </c>
       <c r="N9" s="55" t="n">
-        <v>50.41</v>
+        <v>50.46</v>
       </c>
       <c r="O9" s="56" t="s">
         <v>107</v>
@@ -5426,7 +5430,7 @@
       </c>
       <c r="Q9" s="31" t="n">
         <f aca="false">AA9+AB9+AC9</f>
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="R9" s="32" t="n">
         <f aca="false">B9*P1_PVP+C9*P2_PVP+D9*P3_PVP</f>
@@ -5438,27 +5442,27 @@
       </c>
       <c r="T9" s="32" t="n">
         <f aca="false">IF(P9&gt;0,N9/P9,"")</f>
-        <v>3.150625</v>
+        <v>3.15375</v>
       </c>
       <c r="U9" s="57" t="n">
         <f aca="false">IF(N9&gt;0,R9/N9,"")</f>
-        <v>11.1057329894862</v>
+        <v>11.0947284978201</v>
       </c>
       <c r="V9" s="34" t="n">
         <f aca="false">IF(E9+F9+G9+H9+I9+J9&gt;0,(E9+F9+G9)/(E9+F9+G9+H9+I9+J9),"")</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="W9" s="33" t="n">
         <f aca="false">E9*(P1_PVP-P1_CPROD)+F9*(P2_PVP-P2_CPROD)+G9*(P3_PVP-P3_CPROD)-IF(ISNUMBER(L9),L9,E9*P1_LOG+F9*P2_LOG+G9*P3_LOG)</f>
-        <v>0</v>
+        <v>27.9742</v>
       </c>
       <c r="X9" s="33" t="n">
         <f aca="false">W9-(E9*P1_IVAN+F9*P2_IVAN+G9*P3_IVAN)-(H9+I9+J9)*(COSTE_DEV-IVA_DEV)-AM9-AO9</f>
-        <v>-73.67</v>
+        <v>-51.8504132231405</v>
       </c>
       <c r="Y9" s="33" t="n">
         <f aca="false">AH9-AI9-AJ9-AK9-AL9-AM9-AO9</f>
-        <v>122.108479338843</v>
+        <v>128.044396694215</v>
       </c>
       <c r="AA9" s="58" t="n">
         <f aca="false">MAX(0,B9-E9-H9)</f>
@@ -5466,7 +5470,7 @@
       </c>
       <c r="AB9" s="58" t="n">
         <f aca="false">MAX(0,C9-F9-I9)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AC9" s="58" t="n">
         <f aca="false">MAX(0,D9-G9-J9)</f>
@@ -5478,7 +5482,7 @@
       </c>
       <c r="AE9" s="59" t="n">
         <f aca="false">F9+AB9*TASA_USADA</f>
-        <v>4</v>
+        <v>4.2</v>
       </c>
       <c r="AF9" s="59" t="n">
         <f aca="false">G9+AC9*TASA_USADA</f>
@@ -5486,31 +5490,31 @@
       </c>
       <c r="AG9" s="59" t="n">
         <f aca="false">H9+I9+J9+(AA9+AB9+AC9)*(1-TASA_USADA)</f>
-        <v>4</v>
+        <v>3.8</v>
       </c>
       <c r="AH9" s="60" t="n">
         <f aca="false">AD9*P1_PVP+AE9*P2_PVP+AF9*P3_PVP</f>
-        <v>415.88</v>
+        <v>423.878</v>
       </c>
       <c r="AI9" s="60" t="n">
         <f aca="false">AD9*P1_CPROD+AE9*P2_CPROD+AF9*P3_CPROD</f>
-        <v>42.37904</v>
+        <v>43.3422</v>
       </c>
       <c r="AJ9" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L9),L9,E9*P1_LOG+F9*P2_LOG+G9*P3_LOG)+IF(ISNUMBER(M9),M9,AA9*P1_LOG+AB9*P2_LOG+AC9*P3_LOG)*TASA_USADA</f>
-        <v>88.72</v>
+        <v>90.16</v>
       </c>
       <c r="AK9" s="60" t="n">
         <f aca="false">AG9*COSTE_DEV</f>
-        <v>32.24</v>
+        <v>30.628</v>
       </c>
       <c r="AL9" s="60" t="n">
         <f aca="false">AD9*P1_IVAN+AE9*P2_IVAN+AF9*P3_IVAN-AG9*IVA_DEV</f>
-        <v>64.822480661157</v>
+        <v>66.0434033057851</v>
       </c>
       <c r="AM9" s="60" t="n">
         <f aca="false">N9*(1+RECARGO_ADS)</f>
-        <v>50.41</v>
+        <v>50.46</v>
       </c>
       <c r="AN9" s="58" t="n">
         <f aca="false">IF(ISNUMBER(L9),E9+F9+G9+AA9+AB9+AC9,0)</f>
@@ -5529,7 +5533,7 @@
         <v>2</v>
       </c>
       <c r="C10" s="54" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>0</v>
@@ -5545,35 +5549,35 @@
         <v>0</v>
       </c>
       <c r="M10" s="55" t="n">
-        <v>32.24</v>
+        <v>45.43</v>
       </c>
       <c r="N10" s="55" t="n">
-        <v>16.13</v>
+        <v>41.21</v>
       </c>
       <c r="O10" s="56"/>
       <c r="P10" s="31" t="n">
         <f aca="false">B10+C10+D10</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q10" s="31" t="n">
         <f aca="false">AA10+AB10+AC10</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R10" s="32" t="n">
         <f aca="false">B10*P1_PVP+C10*P2_PVP+D10*P3_PVP</f>
-        <v>139.96</v>
+        <v>219.94</v>
       </c>
       <c r="S10" s="32" t="n">
         <f aca="false">IF(P10&gt;0,R10/P10,"")</f>
-        <v>34.99</v>
+        <v>36.6566666666667</v>
       </c>
       <c r="T10" s="32" t="n">
         <f aca="false">IF(P10&gt;0,N10/P10,"")</f>
-        <v>4.0325</v>
+        <v>6.86833333333333</v>
       </c>
       <c r="U10" s="57" t="n">
         <f aca="false">IF(N10&gt;0,R10/N10,"")</f>
-        <v>8.6769993800372</v>
+        <v>5.33705411307935</v>
       </c>
       <c r="V10" s="34" t="str">
         <f aca="false">IF(E10+F10+G10+H10+I10+J10&gt;0,(E10+F10+G10)/(E10+F10+G10+H10+I10+J10),"")</f>
@@ -5585,11 +5589,11 @@
       </c>
       <c r="X10" s="33" t="n">
         <f aca="false">W10-(E10*P1_IVAN+F10*P2_IVAN+G10*P3_IVAN)-(H10+I10+J10)*(COSTE_DEV-IVA_DEV)-AM10-AO10</f>
-        <v>-19.93</v>
+        <v>-46.91</v>
       </c>
       <c r="Y10" s="33" t="n">
         <f aca="false">AH10-AI10-AJ10-AK10-AL10-AM10-AO10</f>
-        <v>30.8135371900827</v>
+        <v>36.5688760330579</v>
       </c>
       <c r="AA10" s="58" t="n">
         <f aca="false">MAX(0,B10-E10-H10)</f>
@@ -5597,7 +5601,7 @@
       </c>
       <c r="AB10" s="58" t="n">
         <f aca="false">MAX(0,C10-F10-I10)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AC10" s="58" t="n">
         <f aca="false">MAX(0,D10-G10-J10)</f>
@@ -5609,7 +5613,7 @@
       </c>
       <c r="AE10" s="59" t="n">
         <f aca="false">F10+AB10*TASA_USADA</f>
-        <v>1.6</v>
+        <v>3.2</v>
       </c>
       <c r="AF10" s="59" t="n">
         <f aca="false">G10+AC10*TASA_USADA</f>
@@ -5617,48 +5621,54 @@
       </c>
       <c r="AG10" s="59" t="n">
         <f aca="false">H10+I10+J10+(AA10+AB10+AC10)*(1-TASA_USADA)</f>
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="AH10" s="60" t="n">
         <f aca="false">AD10*P1_PVP+AE10*P2_PVP+AF10*P3_PVP</f>
-        <v>111.968</v>
+        <v>175.952</v>
       </c>
       <c r="AI10" s="60" t="n">
         <f aca="false">AD10*P1_CPROD+AE10*P2_CPROD+AF10*P3_CPROD</f>
-        <v>11.55792</v>
+        <v>19.2632</v>
       </c>
       <c r="AJ10" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L10),L10,E10*P1_LOG+F10*P2_LOG+G10*P3_LOG)+IF(ISNUMBER(M10),M10,AA10*P1_LOG+AB10*P2_LOG+AC10*P3_LOG)*TASA_USADA</f>
-        <v>25.792</v>
+        <v>36.344</v>
       </c>
       <c r="AK10" s="60" t="n">
         <f aca="false">AG10*COSTE_DEV</f>
-        <v>6.448</v>
+        <v>9.672</v>
       </c>
       <c r="AL10" s="60" t="n">
         <f aca="false">AD10*P1_IVAN+AE10*P2_IVAN+AF10*P3_IVAN-AG10*IVA_DEV</f>
-        <v>17.4265428099174</v>
+        <v>27.1939239669421</v>
       </c>
       <c r="AM10" s="60" t="n">
         <f aca="false">N10*(1+RECARGO_ADS)</f>
-        <v>16.13</v>
+        <v>41.21</v>
       </c>
       <c r="AN10" s="58" t="n">
         <f aca="false">IF(ISNUMBER(L10),E10+F10+G10+AA10+AB10+AC10,0)</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AO10" s="60" t="n">
         <f aca="false">P10*COMISION</f>
-        <v>3.8</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="53" t="n">
         <v>46305</v>
       </c>
-      <c r="B11" s="54"/>
-      <c r="C11" s="54"/>
-      <c r="D11" s="54"/>
+      <c r="B11" s="54" t="n">
+        <v>6</v>
+      </c>
+      <c r="C11" s="54" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" s="54" t="n">
+        <v>1</v>
+      </c>
       <c r="E11" s="54"/>
       <c r="F11" s="54"/>
       <c r="G11" s="54"/>
@@ -5666,33 +5676,39 @@
       <c r="I11" s="54"/>
       <c r="J11" s="54"/>
       <c r="K11" s="54"/>
-      <c r="L11" s="55"/>
-      <c r="M11" s="55"/>
-      <c r="N11" s="55"/>
+      <c r="L11" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="55" t="n">
+        <v>67.73</v>
+      </c>
+      <c r="N11" s="55" t="n">
+        <v>63.39</v>
+      </c>
       <c r="O11" s="56"/>
       <c r="P11" s="31" t="n">
         <f aca="false">B11+C11+D11</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="Q11" s="31" t="n">
         <f aca="false">AA11+AB11+AC11</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="R11" s="32" t="n">
         <f aca="false">B11*P1_PVP+C11*P2_PVP+D11*P3_PVP</f>
-        <v>0</v>
-      </c>
-      <c r="S11" s="32" t="str">
+        <v>309.91</v>
+      </c>
+      <c r="S11" s="32" t="n">
         <f aca="false">IF(P11&gt;0,R11/P11,"")</f>
-        <v/>
-      </c>
-      <c r="T11" s="32" t="str">
+        <v>34.4344444444444</v>
+      </c>
+      <c r="T11" s="32" t="n">
         <f aca="false">IF(P11&gt;0,N11/P11,"")</f>
-        <v/>
-      </c>
-      <c r="U11" s="57" t="str">
+        <v>7.04333333333333</v>
+      </c>
+      <c r="U11" s="57" t="n">
         <f aca="false">IF(N11&gt;0,R11/N11,"")</f>
-        <v/>
+        <v>4.88894147341852</v>
       </c>
       <c r="V11" s="34" t="str">
         <f aca="false">IF(E11+F11+G11+H11+I11+J11&gt;0,(E11+F11+G11)/(E11+F11+G11+H11+I11+J11),"")</f>
@@ -5704,71 +5720,71 @@
       </c>
       <c r="X11" s="33" t="n">
         <f aca="false">W11-(E11*P1_IVAN+F11*P2_IVAN+G11*P3_IVAN)-(H11+I11+J11)*(COSTE_DEV-IVA_DEV)-AM11-AO11</f>
-        <v>0</v>
+        <v>-71.94</v>
       </c>
       <c r="Y11" s="33" t="n">
         <f aca="false">AH11-AI11-AJ11-AK11-AL11-AM11-AO11</f>
-        <v>0</v>
+        <v>43.5711735537191</v>
       </c>
       <c r="AA11" s="58" t="n">
         <f aca="false">MAX(0,B11-E11-H11)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB11" s="58" t="n">
         <f aca="false">MAX(0,C11-F11-I11)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AC11" s="58" t="n">
         <f aca="false">MAX(0,D11-G11-J11)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD11" s="59" t="n">
         <f aca="false">E11+AA11*TASA_USADA</f>
-        <v>0</v>
+        <v>4.8</v>
       </c>
       <c r="AE11" s="59" t="n">
         <f aca="false">F11+AB11*TASA_USADA</f>
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="AF11" s="59" t="n">
         <f aca="false">G11+AC11*TASA_USADA</f>
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="AG11" s="59" t="n">
         <f aca="false">H11+I11+J11+(AA11+AB11+AC11)*(1-TASA_USADA)</f>
-        <v>0</v>
+        <v>1.8</v>
       </c>
       <c r="AH11" s="60" t="n">
         <f aca="false">AD11*P1_PVP+AE11*P2_PVP+AF11*P3_PVP</f>
-        <v>0</v>
+        <v>247.928</v>
       </c>
       <c r="AI11" s="60" t="n">
         <f aca="false">AD11*P1_CPROD+AE11*P2_CPROD+AF11*P3_CPROD</f>
-        <v>0</v>
+        <v>25.04216</v>
       </c>
       <c r="AJ11" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L11),L11,E11*P1_LOG+F11*P2_LOG+G11*P3_LOG)+IF(ISNUMBER(M11),M11,AA11*P1_LOG+AB11*P2_LOG+AC11*P3_LOG)*TASA_USADA</f>
-        <v>0</v>
+        <v>54.184</v>
       </c>
       <c r="AK11" s="60" t="n">
         <f aca="false">AG11*COSTE_DEV</f>
-        <v>0</v>
+        <v>14.508</v>
       </c>
       <c r="AL11" s="60" t="n">
         <f aca="false">AD11*P1_IVAN+AE11*P2_IVAN+AF11*P3_IVAN-AG11*IVA_DEV</f>
-        <v>0</v>
+        <v>38.682666446281</v>
       </c>
       <c r="AM11" s="60" t="n">
         <f aca="false">N11*(1+RECARGO_ADS)</f>
-        <v>0</v>
+        <v>63.39</v>
       </c>
       <c r="AN11" s="58" t="n">
         <f aca="false">IF(ISNUMBER(L11),E11+F11+G11+AA11+AB11+AC11,0)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AO11" s="60" t="n">
         <f aca="false">P11*COMISION</f>
-        <v>0</v>
+        <v>8.55</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51166,7 +51182,7 @@
       </c>
       <c r="C37" s="31" t="n">
         <f aca="false">(SUM(Diario!$E$6:$E$370)+SUM(Diario!$F$6:$F$370)+SUM(Diario!$G$6:$G$370))+(SUM(Diario!$H$6:$H$370)+SUM(Diario!$I$6:$I$370)+SUM(Diario!$J$6:$J$370))</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F37" s="67" t="s">
         <v>183</v>
@@ -51178,7 +51194,7 @@
       </c>
       <c r="C38" s="34" t="n">
         <f aca="false">IF(C37&gt;0,(SUM(Diario!$E$6:$E$370)+SUM(Diario!$F$6:$F$370)+SUM(Diario!$G$6:$G$370))/C37,"")</f>
-        <v>0.818181818181818</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="F38" s="67" t="s">
         <v>185</v>
@@ -51202,11 +51218,11 @@
       </c>
       <c r="C40" s="34" t="n">
         <f aca="false">IF(SUM(Diario!$P$6:$P$370)&gt;0,SUM(Diario!$C$6:$C$370)/SUM(Diario!$P$6:$P$370),"")</f>
-        <v>0.318181818181818</v>
+        <v>0.327272727272727</v>
       </c>
       <c r="D40" s="34" t="n">
         <f aca="false">IF(SUM(Diario!$P$6:$P$370)&gt;0,SUM(Diario!$D$6:$D$370)/SUM(Diario!$P$6:$P$370),"")</f>
-        <v>0.0227272727272727</v>
+        <v>0.0363636363636364</v>
       </c>
       <c r="F40" s="67" t="s">
         <v>189</v>
@@ -51218,11 +51234,11 @@
       </c>
       <c r="C41" s="34" t="n">
         <f aca="false">IF(C40="",C26,C40)</f>
-        <v>0.318181818181818</v>
+        <v>0.327272727272727</v>
       </c>
       <c r="D41" s="34" t="n">
         <f aca="false">IF(D40="",D26,D40)</f>
-        <v>0.0227272727272727</v>
+        <v>0.0363636363636364</v>
       </c>
       <c r="F41" s="67"/>
     </row>
@@ -51232,7 +51248,7 @@
       </c>
       <c r="C42" s="32" t="n">
         <f aca="false">IF(SUM(Diario!$AN$6:$AN$370)&gt;0,(SUM(Diario!$L$6:$L$370)+SUM(Diario!$M$6:$M$370))/SUM(Diario!$AN$6:$AN$370),"")</f>
-        <v>7.63452380952381</v>
+        <v>7.57679245283019</v>
       </c>
       <c r="F42" s="67" t="s">
         <v>192</v>
@@ -51244,7 +51260,7 @@
       </c>
       <c r="C43" s="32" t="n">
         <f aca="false">(1-C41-D41)*C5+C41*D5+D41*E5</f>
-        <v>33.6263636363636</v>
+        <v>33.99</v>
       </c>
       <c r="F43" s="67"/>
     </row>
@@ -51254,7 +51270,7 @@
       </c>
       <c r="C44" s="32" t="n">
         <f aca="false">(1-C41-D41)*(C5-C9-IF(C42="",C8,C42)-C14)+C41*(D5-D9-IF(C42="",D8,C42)-D14)+D41*(E5-E9-IF(C42="",E8,C42)-E14)</f>
-        <v>17.4422229973883</v>
+        <v>17.7281166380789</v>
       </c>
       <c r="F44" s="67" t="s">
         <v>195</v>
@@ -51266,7 +51282,7 @@
       </c>
       <c r="C45" s="32" t="n">
         <f aca="false">C39*C44-(1-C39)*C36-COMISION</f>
-        <v>11.3917783979106</v>
+        <v>11.6204933104631</v>
       </c>
       <c r="F45" s="67" t="s">
         <v>197</v>
@@ -51278,7 +51294,7 @@
       </c>
       <c r="C46" s="33" t="n">
         <f aca="false">C45/(1+RECARGO_ADS)</f>
-        <v>11.3917783979106</v>
+        <v>11.6204933104631</v>
       </c>
       <c r="F46" s="67" t="s">
         <v>199</v>
@@ -51290,7 +51306,7 @@
       </c>
       <c r="C47" s="72" t="n">
         <f aca="false">IF(C46&gt;0,C43/C46,"")</f>
-        <v>2.95180984582101</v>
+        <v>2.92500491088406</v>
       </c>
       <c r="F47" s="67" t="s">
         <v>201</v>

</xml_diff>

<commit_message>
Contabilidad al 12/10 (export del almacén de hoy, 68 pedidos)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFjE4yx23BY3D6kaMQowKe
</commit_message>
<xml_diff>
--- a/contabilidad/CeraLux_Contabilidad.xlsx
+++ b/contabilidad/CeraLux_Contabilidad.xlsx
@@ -1779,46 +1779,46 @@
               <c:strCache>
                 <c:ptCount val="14"/>
                 <c:pt idx="0">
-                  <c:v>Sun 27/09</c:v>
+                  <c:v>Tue 29/09</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Mon 28/09</c:v>
+                  <c:v>Wed 30/09</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Tue 29/09</c:v>
+                  <c:v>Thu 01/10</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Wed 30/09</c:v>
+                  <c:v>Fri 02/10</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Thu 01/10</c:v>
+                  <c:v>Sat 03/10</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Fri 02/10</c:v>
+                  <c:v>Sun 04/10</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Sat 03/10</c:v>
+                  <c:v>Mon 05/10</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>Sun 04/10</c:v>
+                  <c:v>Tue 06/10</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Mon 05/10</c:v>
+                  <c:v>Wed 07/10</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Tue 06/10</c:v>
+                  <c:v>Thu 08/10</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Wed 07/10</c:v>
+                  <c:v>Fri 09/10</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>Thu 08/10</c:v>
+                  <c:v>Sat 10/10</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>Fri 09/10</c:v>
+                  <c:v>Sun 11/10</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>Sat 10/10</c:v>
+                  <c:v>Mon 12/10</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1848,28 +1848,28 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>62.6280826446281</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>8.63823140495868</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>62.6280826446281</c:v>
+                  <c:v>32.9863140495868</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>8.63823140495868</c:v>
+                  <c:v>128.044396694215</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>28.2932892561984</c:v>
+                  <c:v>36.5688760330579</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>128.044396694215</c:v>
+                  <c:v>57.0848429752066</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>36.5688760330579</c:v>
+                  <c:v>-27.9818347107438</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>43.5711735537191</c:v>
+                  <c:v>27.5821652892562</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1877,8 +1877,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="67286432"/>
-        <c:axId val="90468839"/>
+        <c:axId val="65940706"/>
+        <c:axId val="67586164"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -1942,46 +1942,46 @@
               <c:strCache>
                 <c:ptCount val="14"/>
                 <c:pt idx="0">
-                  <c:v>Sun 27/09</c:v>
+                  <c:v>Tue 29/09</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Mon 28/09</c:v>
+                  <c:v>Wed 30/09</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Tue 29/09</c:v>
+                  <c:v>Thu 01/10</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Wed 30/09</c:v>
+                  <c:v>Fri 02/10</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Thu 01/10</c:v>
+                  <c:v>Sat 03/10</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Fri 02/10</c:v>
+                  <c:v>Sun 04/10</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Sat 03/10</c:v>
+                  <c:v>Mon 05/10</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>Sun 04/10</c:v>
+                  <c:v>Tue 06/10</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Mon 05/10</c:v>
+                  <c:v>Wed 07/10</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Tue 06/10</c:v>
+                  <c:v>Thu 08/10</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Wed 07/10</c:v>
+                  <c:v>Fri 09/10</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>Thu 08/10</c:v>
+                  <c:v>Sat 10/10</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>Fri 09/10</c:v>
+                  <c:v>Sun 11/10</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>Sat 10/10</c:v>
+                  <c:v>Mon 12/10</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2011,28 +2011,28 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>67.67</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>70.18</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>67.67</c:v>
+                  <c:v>47.78</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>70.18</c:v>
+                  <c:v>50.46</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>47.78</c:v>
+                  <c:v>41.21</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>50.46</c:v>
+                  <c:v>64.81</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>41.21</c:v>
+                  <c:v>89.43</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>63.39</c:v>
+                  <c:v>34.45</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2047,11 +2047,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="67286432"/>
-        <c:axId val="90468839"/>
+        <c:axId val="65940706"/>
+        <c:axId val="67586164"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="67286432"/>
+        <c:axId val="65940706"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2083,7 +2083,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="90468839"/>
+        <c:crossAx val="67586164"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2091,7 +2091,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="90468839"/>
+        <c:axId val="67586164"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2133,7 +2133,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="67286432"/>
+        <c:crossAx val="65940706"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2332,7 +2332,7 @@
                 <c:formatCode>#,##0" €";[RED]\-#,##0" €";\-</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>307.744049586777</c:v>
+                  <c:v>325.551074380165</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -2373,8 +2373,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="46058975"/>
-        <c:axId val="3194225"/>
+        <c:axId val="85087024"/>
+        <c:axId val="50170899"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2471,11 +2471,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="46058975"/>
-        <c:axId val="3194225"/>
+        <c:axId val="85087024"/>
+        <c:axId val="50170899"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="46058975"/>
+        <c:axId val="85087024"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2507,7 +2507,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="3194225"/>
+        <c:crossAx val="50170899"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2515,7 +2515,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="3194225"/>
+        <c:axId val="50170899"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2557,7 +2557,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="46058975"/>
+        <c:crossAx val="85087024"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="F3" s="4" t="n">
         <f aca="true">TODAY()</f>
-        <v>46305</v>
+        <v>46307</v>
       </c>
       <c r="G3" s="4"/>
       <c r="H3" s="3" t="s">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="I3" s="5" t="n">
         <f aca="false">MAX(1,$F$3-$C$3+1)</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J3" s="6" t="s">
         <v>5</v>
@@ -2951,32 +2951,32 @@
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="10" t="n">
         <f aca="false">F25</f>
-        <v>307.744049586777</v>
+        <v>325.551074380166</v>
       </c>
       <c r="C7" s="10"/>
       <c r="D7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$W$6:$W$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>230.3994</v>
+        <v>250.5915</v>
       </c>
       <c r="E7" s="10"/>
       <c r="F7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$X$6:$X$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+F24</f>
-        <v>-231.800909090909</v>
+        <v>-354.045785123967</v>
       </c>
       <c r="G7" s="10"/>
       <c r="H7" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="I7" s="11"/>
       <c r="J7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$R$6:$R$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>1869.45</v>
+        <v>2289.32</v>
       </c>
       <c r="K7" s="10"/>
       <c r="L7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>340.69</v>
+        <v>465.99</v>
       </c>
       <c r="M7" s="10"/>
     </row>
@@ -3009,32 +3009,32 @@
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="10" t="n">
         <f aca="false">IF(H7&gt;0,L7/H7,"")</f>
-        <v>6.19436363636364</v>
+        <v>6.85279411764706</v>
       </c>
       <c r="C10" s="10"/>
       <c r="D10" s="10" t="n">
         <f aca="false">CPA_BE</f>
-        <v>11.6204933104631</v>
+        <v>11.4337112299465</v>
       </c>
       <c r="E10" s="10"/>
       <c r="F10" s="12" t="n">
         <f aca="false">IF(L7&gt;0,J7/L7,"")</f>
-        <v>5.48724647039831</v>
+        <v>4.91280928775296</v>
       </c>
       <c r="G10" s="12"/>
       <c r="H10" s="12" t="n">
         <f aca="false">ROAS_BE</f>
-        <v>2.92500491088406</v>
+        <v>2.94449194239382</v>
       </c>
       <c r="I10" s="12"/>
       <c r="J10" s="10" t="n">
         <f aca="false">IF(H7&gt;0,J7/H7,"")</f>
-        <v>33.99</v>
+        <v>33.6664705882353</v>
       </c>
       <c r="K10" s="10"/>
       <c r="L10" s="13" t="n">
         <f aca="false">IF(H7&gt;0,(SUMIFS(Diario!$C$6:$C$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+SUMIFS(Diario!$D$6:$D$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3))/H7,"")</f>
-        <v>0.363636363636364</v>
+        <v>0.338235294117647</v>
       </c>
       <c r="M10" s="13"/>
     </row>
@@ -3067,17 +3067,17 @@
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C13" s="11"/>
       <c r="D13" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$Q$6:$Q$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="E13" s="11"/>
       <c r="F13" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$K$6:$K$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G13" s="11"/>
       <c r="H13" s="11" t="n">
@@ -3087,7 +3087,7 @@
       <c r="I13" s="11"/>
       <c r="J13" s="13" t="n">
         <f aca="false">IF(B13+H13&gt;0,B13/(B13+H13),"")</f>
-        <v>0.833333333333333</v>
+        <v>0.846153846153846</v>
       </c>
       <c r="K13" s="13"/>
       <c r="L13" s="14" t="str">
@@ -3124,7 +3124,7 @@
       </c>
       <c r="F16" s="17" t="n">
         <f aca="false">SUMIFS(Diario!$AH$6:$AH$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>1507.556</v>
+        <v>1849.45</v>
       </c>
       <c r="H16" s="15" t="s">
         <v>29</v>
@@ -3146,11 +3146,11 @@
       <c r="D17" s="15"/>
       <c r="E17" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F17/$F$16,"")</f>
-        <v>-0.0990276978102306</v>
+        <v>-0.0976465976371353</v>
       </c>
       <c r="F17" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AI$6:$AI$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-149.2898</v>
+        <v>-180.5925</v>
       </c>
       <c r="H17" s="15" t="s">
         <v>31</v>
@@ -3160,7 +3160,7 @@
       <c r="K17" s="15"/>
       <c r="L17" s="20" t="n">
         <f aca="false">F25/I3</f>
-        <v>30.7744049586777</v>
+        <v>27.1292561983471</v>
       </c>
       <c r="M17" s="20"/>
     </row>
@@ -3172,11 +3172,11 @@
       <c r="D18" s="15"/>
       <c r="E18" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F18/$F$16,"")</f>
-        <v>-0.22315190944814</v>
+        <v>-0.226175349428208</v>
       </c>
       <c r="F18" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AJ$6:$AJ$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-336.414</v>
+        <v>-418.3</v>
       </c>
       <c r="H18" s="15" t="s">
         <v>33</v>
@@ -3186,7 +3186,7 @@
       <c r="K18" s="15"/>
       <c r="L18" s="18" t="n">
         <f aca="false">L17*30</f>
-        <v>923.232148760331</v>
+        <v>813.877685950414</v>
       </c>
       <c r="M18" s="18"/>
     </row>
@@ -3198,11 +3198,11 @@
       <c r="D19" s="15"/>
       <c r="E19" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F19/$F$16,"")</f>
-        <v>-0.0566718582924946</v>
+        <v>-0.0566546811214145</v>
       </c>
       <c r="F19" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AK$6:$AK$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-85.436</v>
+        <v>-104.78</v>
       </c>
       <c r="H19" s="21" t="s">
         <v>35</v>
@@ -3212,7 +3212,7 @@
       <c r="K19" s="21"/>
       <c r="L19" s="22" t="n">
         <f aca="false">IF(L16&gt;0,L18/L16,"")</f>
-        <v>0.0923232148760331</v>
+        <v>0.0813877685950414</v>
       </c>
       <c r="M19" s="22"/>
     </row>
@@ -3224,11 +3224,11 @@
       <c r="D20" s="15"/>
       <c r="E20" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F20/$F$16,"")</f>
-        <v>-0.0346587456784358</v>
+        <v>-0.0349293033063884</v>
       </c>
       <c r="F20" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AO$6:$AO$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-52.25</v>
+        <v>-64.6</v>
       </c>
       <c r="H20" s="15" t="s">
         <v>37</v>
@@ -3238,7 +3238,7 @@
       <c r="K20" s="15"/>
       <c r="L20" s="20" t="n">
         <f aca="false">BEN_PEDIDO</f>
-        <v>11.6204933104631</v>
+        <v>11.4337112299465</v>
       </c>
       <c r="M20" s="20"/>
     </row>
@@ -3250,11 +3250,11 @@
       <c r="D21" s="15"/>
       <c r="E21" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F21/$F$16,"")</f>
-        <v>-0.156367093768472</v>
+        <v>-0.156606788839836</v>
       </c>
       <c r="F21" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AL$6:$AL$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-235.732150413223</v>
+        <v>-289.636425619835</v>
       </c>
       <c r="H21" s="15" t="s">
         <v>39</v>
@@ -3264,7 +3264,7 @@
       <c r="K21" s="15"/>
       <c r="L21" s="20" t="n">
         <f aca="false">B10</f>
-        <v>6.19436363636364</v>
+        <v>6.85279411764706</v>
       </c>
       <c r="M21" s="20"/>
     </row>
@@ -3276,11 +3276,11 @@
       <c r="D22" s="15"/>
       <c r="E22" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F22/$F$16,"")</f>
-        <v>-0.225988288328924</v>
+        <v>-0.251961393927925</v>
       </c>
       <c r="F22" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AM$6:$AM$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-340.69</v>
+        <v>-465.99</v>
       </c>
       <c r="H22" s="15" t="s">
         <v>41</v>
@@ -3290,7 +3290,7 @@
       <c r="K22" s="15"/>
       <c r="L22" s="20" t="n">
         <f aca="false">IF(ISNUMBER(L21),L20-L21*(1+RECARGO_ADS),"")</f>
-        <v>5.42612967409949</v>
+        <v>4.58091711229946</v>
       </c>
       <c r="M22" s="20"/>
     </row>
@@ -3302,11 +3302,11 @@
       <c r="D23" s="23"/>
       <c r="E23" s="24" t="n">
         <f aca="false">IF($F$16&gt;0,F23/$F$16,"")</f>
-        <v>0.204134406673302</v>
+        <v>0.176025885739093</v>
       </c>
       <c r="F23" s="25" t="n">
         <f aca="false">SUM(F16:F22)</f>
-        <v>307.744049586777</v>
+        <v>325.551074380166</v>
       </c>
       <c r="H23" s="21" t="s">
         <v>43</v>
@@ -3316,7 +3316,7 @@
       <c r="K23" s="21"/>
       <c r="L23" s="26" t="n">
         <f aca="false">IF(NOT(ISNUMBER(L22)),"",IF(L22&lt;=0,"Baja el CPA",ROUNDUP((L16-F24/I3*30)/30/L22,0)))</f>
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="M23" s="26"/>
     </row>
@@ -3342,7 +3342,7 @@
       <c r="K24" s="15"/>
       <c r="L24" s="18" t="n">
         <f aca="false">IF(ISNUMBER(L23),L23*L21,"")</f>
-        <v>384.050545454545</v>
+        <v>500.253970588235</v>
       </c>
       <c r="M24" s="18"/>
     </row>
@@ -3354,11 +3354,11 @@
       <c r="D25" s="23"/>
       <c r="E25" s="24" t="n">
         <f aca="false">IF($F$16&gt;0,F25/$F$16,"")</f>
-        <v>0.204134406673302</v>
+        <v>0.176025885739093</v>
       </c>
       <c r="F25" s="25" t="n">
         <f aca="false">F23+F24</f>
-        <v>307.744049586777</v>
+        <v>325.551074380166</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3369,7 +3369,7 @@
       <c r="D26" s="27"/>
       <c r="F26" s="28" t="n">
         <f aca="false">IF(F16&gt;0,F25/F16,"")</f>
-        <v>0.204134406673302</v>
+        <v>0.176025885739093</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3405,7 +3405,7 @@
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="30" t="n">
         <f aca="false">$F$3-13</f>
-        <v>46292</v>
+        <v>46294</v>
       </c>
       <c r="C29" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B29)</f>
@@ -3431,7 +3431,7 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="30" t="n">
         <f aca="false">$F$3-12</f>
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="C30" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B30)</f>
@@ -3457,7 +3457,7 @@
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="30" t="n">
         <f aca="false">$F$3-11</f>
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="C31" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B31)</f>
@@ -3483,7 +3483,7 @@
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="30" t="n">
         <f aca="false">$F$3-10</f>
-        <v>46295</v>
+        <v>46297</v>
       </c>
       <c r="C32" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B32)</f>
@@ -3509,7 +3509,7 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="30" t="n">
         <f aca="false">$F$3-9</f>
-        <v>46296</v>
+        <v>46298</v>
       </c>
       <c r="C33" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B33)</f>
@@ -3535,7 +3535,7 @@
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="30" t="n">
         <f aca="false">$F$3-8</f>
-        <v>46297</v>
+        <v>46299</v>
       </c>
       <c r="C34" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B34)</f>
@@ -3561,75 +3561,75 @@
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="30" t="n">
         <f aca="false">$F$3-7</f>
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="C35" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B35)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D35" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B35)</f>
-        <v>0</v>
-      </c>
-      <c r="E35" s="32" t="str">
+        <v>67.67</v>
+      </c>
+      <c r="E35" s="32" t="n">
         <f aca="false">IF(C35&gt;0,D35/C35,"")</f>
-        <v/>
+        <v>7.51888888888889</v>
       </c>
       <c r="F35" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B35)</f>
-        <v>0</v>
-      </c>
-      <c r="G35" s="34" t="str">
+        <v>62.6280826446281</v>
+      </c>
+      <c r="G35" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B35))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B35))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B35)),"")</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="30" t="n">
         <f aca="false">$F$3-6</f>
-        <v>46299</v>
+        <v>46301</v>
       </c>
       <c r="C36" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B36)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D36" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B36)</f>
-        <v>0</v>
-      </c>
-      <c r="E36" s="32" t="str">
+        <v>70.18</v>
+      </c>
+      <c r="E36" s="32" t="n">
         <f aca="false">IF(C36&gt;0,D36/C36,"")</f>
-        <v/>
+        <v>8.7725</v>
       </c>
       <c r="F36" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B36)</f>
-        <v>0</v>
-      </c>
-      <c r="G36" s="34" t="str">
+        <v>8.63823140495868</v>
+      </c>
+      <c r="G36" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B36))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B36))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B36)),"")</f>
-        <v/>
+        <v>0.75</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="30" t="n">
         <f aca="false">$F$3-5</f>
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="C37" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B37)</f>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D37" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B37)</f>
-        <v>67.67</v>
+        <v>47.78</v>
       </c>
       <c r="E37" s="32" t="n">
         <f aca="false">IF(C37&gt;0,D37/C37,"")</f>
-        <v>7.51888888888889</v>
+        <v>6.82571428571429</v>
       </c>
       <c r="F37" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B37)</f>
-        <v>62.6280826446281</v>
+        <v>32.9863140495868</v>
       </c>
       <c r="G37" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B37))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B37))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B37)),"")</f>
@@ -3639,85 +3639,85 @@
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="30" t="n">
         <f aca="false">$F$3-4</f>
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="C38" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B38)</f>
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D38" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B38)</f>
-        <v>70.18</v>
+        <v>50.46</v>
       </c>
       <c r="E38" s="32" t="n">
         <f aca="false">IF(C38&gt;0,D38/C38,"")</f>
-        <v>8.7725</v>
+        <v>3.15375</v>
       </c>
       <c r="F38" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B38)</f>
-        <v>8.63823140495868</v>
+        <v>128.044396694215</v>
       </c>
       <c r="G38" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B38))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B38))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B38)),"")</f>
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="30" t="n">
         <f aca="false">$F$3-3</f>
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="C39" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B39)</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D39" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B39)</f>
-        <v>47.78</v>
+        <v>41.21</v>
       </c>
       <c r="E39" s="32" t="n">
         <f aca="false">IF(C39&gt;0,D39/C39,"")</f>
-        <v>6.82571428571429</v>
+        <v>6.86833333333333</v>
       </c>
       <c r="F39" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B39)</f>
-        <v>28.2932892561984</v>
-      </c>
-      <c r="G39" s="34" t="n">
+        <v>36.5688760330579</v>
+      </c>
+      <c r="G39" s="34" t="str">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B39))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B39))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B39)),"")</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="30" t="n">
         <f aca="false">$F$3-2</f>
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="C40" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B40)</f>
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D40" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B40)</f>
-        <v>50.46</v>
+        <v>64.81</v>
       </c>
       <c r="E40" s="32" t="n">
         <f aca="false">IF(C40&gt;0,D40/C40,"")</f>
-        <v>3.15375</v>
+        <v>6.481</v>
       </c>
       <c r="F40" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B40)</f>
-        <v>128.044396694215</v>
-      </c>
-      <c r="G40" s="34" t="n">
+        <v>57.0848429752066</v>
+      </c>
+      <c r="G40" s="34" t="str">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B40))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B40))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B40)),"")</f>
-        <v>0.5</v>
+        <v/>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="30" t="n">
         <f aca="false">$F$3-1</f>
-        <v>46304</v>
+        <v>46306</v>
       </c>
       <c r="C41" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B41)</f>
@@ -3725,15 +3725,15 @@
       </c>
       <c r="D41" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B41)</f>
-        <v>41.21</v>
+        <v>89.43</v>
       </c>
       <c r="E41" s="32" t="n">
         <f aca="false">IF(C41&gt;0,D41/C41,"")</f>
-        <v>6.86833333333333</v>
+        <v>14.905</v>
       </c>
       <c r="F41" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B41)</f>
-        <v>36.5688760330579</v>
+        <v>-27.9818347107438</v>
       </c>
       <c r="G41" s="34" t="str">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B41))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B41))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B41)),"")</f>
@@ -3743,23 +3743,23 @@
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="30" t="n">
         <f aca="false">$F$3-0</f>
-        <v>46305</v>
+        <v>46307</v>
       </c>
       <c r="C42" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B42)</f>
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D42" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B42)</f>
-        <v>63.39</v>
+        <v>34.45</v>
       </c>
       <c r="E42" s="32" t="n">
         <f aca="false">IF(C42&gt;0,D42/C42,"")</f>
-        <v>7.04333333333333</v>
+        <v>5.74166666666667</v>
       </c>
       <c r="F42" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B42)</f>
-        <v>43.5711735537191</v>
+        <v>27.5821652892562</v>
       </c>
       <c r="G42" s="34" t="str">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B42))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B42))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B42)),"")</f>
@@ -3830,23 +3830,23 @@
       </c>
       <c r="C47" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="D47" s="37" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>340.69</v>
+        <v>465.99</v>
       </c>
       <c r="E47" s="32" t="n">
         <f aca="false">IF(C47&gt;0,D47/C47,"")</f>
-        <v>6.19436363636364</v>
+        <v>6.85279411764706</v>
       </c>
       <c r="F47" s="37" t="n">
         <f aca="false">SUMIFS(Diario!$R$6:$R$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>1869.45</v>
+        <v>2289.32</v>
       </c>
       <c r="G47" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H47" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
@@ -3854,11 +3854,11 @@
       </c>
       <c r="I47" s="34" t="n">
         <f aca="false">IF(G47+H47&gt;0,G47/(G47+H47),"")</f>
-        <v>0.833333333333333</v>
+        <v>0.846153846153846</v>
       </c>
       <c r="J47" s="37" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>307.744049586777</v>
+        <v>325.551074380165</v>
       </c>
       <c r="K47" s="37" t="n">
         <f aca="false">-SUMIFS(Gastos!$D$5:$D$304,Gastos!$A$5:$A$304,"&gt;="&amp;$B47,Gastos!$A$5:$A$304,"&lt;="&amp;EOMONTH($B47,0))</f>
@@ -3866,11 +3866,11 @@
       </c>
       <c r="L47" s="38" t="n">
         <f aca="false">J47+K47</f>
-        <v>307.744049586777</v>
+        <v>325.551074380165</v>
       </c>
       <c r="M47" s="34" t="n">
         <f aca="false">IF(OBJETIVO_MES&gt;0,L47/OBJETIVO_MES,"")</f>
-        <v>0.0307744049586777</v>
+        <v>0.0325551074380165</v>
       </c>
       <c r="O47" s="39" t="n">
         <f aca="false">OBJETIVO_MES</f>
@@ -4477,23 +4477,23 @@
       </c>
       <c r="C59" s="41" t="n">
         <f aca="false">SUM(C47:C58)</f>
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="D59" s="42" t="n">
         <f aca="false">SUM(D47:D58)</f>
-        <v>340.69</v>
+        <v>465.99</v>
       </c>
       <c r="E59" s="43" t="n">
         <f aca="false">IF(C59&gt;0,D59/C59,"")</f>
-        <v>6.19436363636364</v>
+        <v>6.85279411764706</v>
       </c>
       <c r="F59" s="42" t="n">
         <f aca="false">SUM(F47:F58)</f>
-        <v>1869.45</v>
+        <v>2289.32</v>
       </c>
       <c r="G59" s="41" t="n">
         <f aca="false">SUM(G47:G58)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H59" s="41" t="n">
         <f aca="false">SUM(H47:H58)</f>
@@ -4501,11 +4501,11 @@
       </c>
       <c r="I59" s="44" t="n">
         <f aca="false">IF(G59+H59&gt;0,G59/(G59+H59),"")</f>
-        <v>0.833333333333333</v>
+        <v>0.846153846153846</v>
       </c>
       <c r="J59" s="42" t="n">
         <f aca="false">SUM(J47:J58)</f>
-        <v>307.744049586777</v>
+        <v>325.551074380165</v>
       </c>
       <c r="K59" s="42" t="n">
         <f aca="false">SUM(K47:K58)</f>
@@ -4513,7 +4513,7 @@
       </c>
       <c r="L59" s="42" t="n">
         <f aca="false">SUM(L47:L58)</f>
-        <v>307.744049586777</v>
+        <v>325.551074380165</v>
       </c>
       <c r="M59" s="45"/>
     </row>
@@ -4700,11 +4700,11 @@
       </c>
       <c r="B4" s="47" t="n">
         <f aca="false">SUM(B6:B370)</f>
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="C4" s="47" t="n">
         <f aca="false">SUM(C6:C370)</f>
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D4" s="47" t="n">
         <f aca="false">SUM(D6:D370)</f>
@@ -4712,7 +4712,7 @@
       </c>
       <c r="E4" s="47" t="n">
         <f aca="false">SUM(E6:E370)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F4" s="47" t="n">
         <f aca="false">SUM(F6:F370)</f>
@@ -4736,67 +4736,67 @@
       </c>
       <c r="K4" s="47" t="n">
         <f aca="false">SUM(K6:K370)</f>
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="L4" s="48" t="n">
         <f aca="false">SUM(L6:L370)</f>
-        <v>75.79</v>
+        <v>83.18</v>
       </c>
       <c r="M4" s="48" t="n">
         <f aca="false">SUM(M6:M370)</f>
-        <v>325.78</v>
+        <v>418.9</v>
       </c>
       <c r="N4" s="48" t="n">
         <f aca="false">SUM(N6:N370)</f>
-        <v>340.69</v>
+        <v>465.99</v>
       </c>
       <c r="P4" s="47" t="n">
         <f aca="false">SUM(P6:P370)</f>
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="Q4" s="47" t="n">
         <f aca="false">SUM(Q6:Q370)</f>
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="R4" s="48" t="n">
         <f aca="false">SUM(R6:R370)</f>
-        <v>1869.45</v>
+        <v>2289.32</v>
       </c>
       <c r="S4" s="48" t="n">
         <f aca="false">IF(P4&gt;0,R4/P4,"")</f>
-        <v>33.99</v>
+        <v>33.6664705882353</v>
       </c>
       <c r="T4" s="48" t="n">
         <f aca="false">IF(P4&gt;0,N4/P4,"")</f>
-        <v>6.19436363636364</v>
+        <v>6.85279411764706</v>
       </c>
       <c r="U4" s="49" t="n">
         <f aca="false">IF(N4&gt;0,R4/N4,"")</f>
-        <v>5.48724647039831</v>
+        <v>4.91280928775296</v>
       </c>
       <c r="V4" s="50" t="n">
         <f aca="false">IF(E4+F4+G4+H4+I4+J4&gt;0,(E4+F4+G4)/(E4+F4+G4+H4+I4+J4),"")</f>
-        <v>0.833333333333333</v>
+        <v>0.846153846153846</v>
       </c>
       <c r="W4" s="48" t="n">
         <f aca="false">SUM(W6:W370)</f>
-        <v>230.3994</v>
+        <v>250.5915</v>
       </c>
       <c r="X4" s="48" t="n">
         <f aca="false">SUM(X6:X370)</f>
-        <v>-231.800909090909</v>
+        <v>-354.045785123967</v>
       </c>
       <c r="Y4" s="48" t="n">
         <f aca="false">SUM(Y6:Y370)</f>
-        <v>307.744049586777</v>
+        <v>325.551074380165</v>
       </c>
       <c r="AA4" s="47" t="n">
         <f aca="false">SUM(AA6:AA370)</f>
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="AB4" s="47" t="n">
         <f aca="false">SUM(AB6:AB370)</f>
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="AC4" s="47" t="n">
         <f aca="false">SUM(AC6:AC370)</f>
@@ -4804,11 +4804,11 @@
       </c>
       <c r="AD4" s="51" t="n">
         <f aca="false">SUM(AD6:AD370)</f>
-        <v>28.4</v>
+        <v>36.6</v>
       </c>
       <c r="AE4" s="51" t="n">
         <f aca="false">SUM(AE6:AE370)</f>
-        <v>14.4</v>
+        <v>16.8</v>
       </c>
       <c r="AF4" s="51" t="n">
         <f aca="false">SUM(AF6:AF370)</f>
@@ -4816,39 +4816,39 @@
       </c>
       <c r="AG4" s="51" t="n">
         <f aca="false">SUM(AG6:AG370)</f>
-        <v>10.6</v>
+        <v>13</v>
       </c>
       <c r="AH4" s="48" t="n">
         <f aca="false">SUM(AH6:AH370)</f>
-        <v>1507.556</v>
+        <v>1849.45</v>
       </c>
       <c r="AI4" s="48" t="n">
         <f aca="false">SUM(AI6:AI370)</f>
-        <v>149.2898</v>
+        <v>180.5925</v>
       </c>
       <c r="AJ4" s="48" t="n">
         <f aca="false">SUM(AJ6:AJ370)</f>
-        <v>336.414</v>
+        <v>418.3</v>
       </c>
       <c r="AK4" s="48" t="n">
         <f aca="false">SUM(AK6:AK370)</f>
-        <v>85.436</v>
+        <v>104.78</v>
       </c>
       <c r="AL4" s="48" t="n">
         <f aca="false">SUM(AL6:AL370)</f>
-        <v>235.732150413223</v>
+        <v>289.636425619835</v>
       </c>
       <c r="AM4" s="48" t="n">
         <f aca="false">SUM(AM6:AM370)</f>
-        <v>340.69</v>
+        <v>465.99</v>
       </c>
       <c r="AN4" s="47" t="n">
         <f aca="false">SUM(AN6:AN370)</f>
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="AO4" s="48" t="n">
         <f aca="false">SUM(AO6:AO370)</f>
-        <v>52.25</v>
+        <v>64.6</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5138,7 +5138,7 @@
       <c r="I7" s="54"/>
       <c r="J7" s="54"/>
       <c r="K7" s="54" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L7" s="55" t="n">
         <v>22.11</v>
@@ -5265,7 +5265,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" s="54"/>
       <c r="G8" s="54"/>
@@ -5273,13 +5273,13 @@
       <c r="I8" s="54"/>
       <c r="J8" s="54"/>
       <c r="K8" s="54" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L8" s="55" t="n">
-        <v>8.06</v>
+        <v>15.45</v>
       </c>
       <c r="M8" s="55" t="n">
-        <v>45.97</v>
+        <v>38.58</v>
       </c>
       <c r="N8" s="55" t="n">
         <v>47.78</v>
@@ -5291,7 +5291,7 @@
       </c>
       <c r="Q8" s="31" t="n">
         <f aca="false">AA8+AB8+AC8</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="R8" s="32" t="n">
         <f aca="false">B8*P1_PVP+C8*P2_PVP+D8*P3_PVP</f>
@@ -5315,19 +5315,19 @@
       </c>
       <c r="W8" s="33" t="n">
         <f aca="false">E8*(P1_PVP-P1_CPROD)+F8*(P2_PVP-P2_CPROD)+G8*(P3_PVP-P3_CPROD)-IF(ISNUMBER(L8),L8,E8*P1_LOG+F8*P2_LOG+G8*P3_LOG)</f>
-        <v>19.5221</v>
+        <v>39.7142</v>
       </c>
       <c r="X8" s="33" t="n">
         <f aca="false">W8-(E8*P1_IVAN+F8*P2_IVAN+G8*P3_IVAN)-(H8+I8+J8)*(COSTE_DEV-IVA_DEV)-AM8-AO8</f>
-        <v>-39.6948760330579</v>
+        <v>-24.2897520661157</v>
       </c>
       <c r="Y8" s="33" t="n">
         <f aca="false">AH8-AI8-AJ8-AK8-AL8-AM8-AO8</f>
-        <v>28.2932892561984</v>
+        <v>32.9863140495868</v>
       </c>
       <c r="AA8" s="58" t="n">
         <f aca="false">MAX(0,B8-E8-H8)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AB8" s="58" t="n">
         <f aca="false">MAX(0,C8-F8-I8)</f>
@@ -5339,7 +5339,7 @@
       </c>
       <c r="AD8" s="59" t="n">
         <f aca="false">E8+AA8*TASA_USADA</f>
-        <v>5</v>
+        <v>5.2</v>
       </c>
       <c r="AE8" s="59" t="n">
         <f aca="false">F8+AB8*TASA_USADA</f>
@@ -5351,27 +5351,27 @@
       </c>
       <c r="AG8" s="59" t="n">
         <f aca="false">H8+I8+J8+(AA8+AB8+AC8)*(1-TASA_USADA)</f>
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="AH8" s="60" t="n">
         <f aca="false">AD8*P1_PVP+AE8*P2_PVP+AF8*P3_PVP</f>
-        <v>181.942</v>
+        <v>187.94</v>
       </c>
       <c r="AI8" s="60" t="n">
         <f aca="false">AD8*P1_CPROD+AE8*P2_CPROD+AF8*P3_CPROD</f>
-        <v>15.89214</v>
+        <v>16.37372</v>
       </c>
       <c r="AJ8" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L8),L8,E8*P1_LOG+F8*P2_LOG+G8*P3_LOG)+IF(ISNUMBER(M8),M8,AA8*P1_LOG+AB8*P2_LOG+AC8*P3_LOG)*TASA_USADA</f>
-        <v>44.836</v>
+        <v>46.314</v>
       </c>
       <c r="AK8" s="60" t="n">
         <f aca="false">AG8*COSTE_DEV</f>
-        <v>9.672</v>
+        <v>8.06</v>
       </c>
       <c r="AL8" s="60" t="n">
         <f aca="false">AD8*P1_IVAN+AE8*P2_IVAN+AF8*P3_IVAN-AG8*IVA_DEV</f>
-        <v>28.8185707438017</v>
+        <v>29.7759659504132</v>
       </c>
       <c r="AM8" s="60" t="n">
         <f aca="false">N8*(1+RECARGO_ADS)</f>
@@ -5410,7 +5410,7 @@
       </c>
       <c r="J9" s="54"/>
       <c r="K9" s="54" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L9" s="55" t="n">
         <v>7.2</v>
@@ -5664,7 +5664,7 @@
         <v>6</v>
       </c>
       <c r="C11" s="54" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>1</v>
@@ -5675,40 +5675,42 @@
       <c r="H11" s="54"/>
       <c r="I11" s="54"/>
       <c r="J11" s="54"/>
-      <c r="K11" s="54"/>
+      <c r="K11" s="54" t="n">
+        <v>2</v>
+      </c>
       <c r="L11" s="55" t="n">
         <v>0</v>
       </c>
       <c r="M11" s="55" t="n">
-        <v>67.73</v>
+        <v>74.93</v>
       </c>
       <c r="N11" s="55" t="n">
-        <v>63.39</v>
+        <v>64.81</v>
       </c>
       <c r="O11" s="56"/>
       <c r="P11" s="31" t="n">
         <f aca="false">B11+C11+D11</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q11" s="31" t="n">
         <f aca="false">AA11+AB11+AC11</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R11" s="32" t="n">
         <f aca="false">B11*P1_PVP+C11*P2_PVP+D11*P3_PVP</f>
-        <v>309.91</v>
+        <v>349.9</v>
       </c>
       <c r="S11" s="32" t="n">
         <f aca="false">IF(P11&gt;0,R11/P11,"")</f>
-        <v>34.4344444444444</v>
+        <v>34.99</v>
       </c>
       <c r="T11" s="32" t="n">
         <f aca="false">IF(P11&gt;0,N11/P11,"")</f>
-        <v>7.04333333333333</v>
+        <v>6.481</v>
       </c>
       <c r="U11" s="57" t="n">
         <f aca="false">IF(N11&gt;0,R11/N11,"")</f>
-        <v>4.88894147341852</v>
+        <v>5.39885820089492</v>
       </c>
       <c r="V11" s="34" t="str">
         <f aca="false">IF(E11+F11+G11+H11+I11+J11&gt;0,(E11+F11+G11)/(E11+F11+G11+H11+I11+J11),"")</f>
@@ -5720,11 +5722,11 @@
       </c>
       <c r="X11" s="33" t="n">
         <f aca="false">W11-(E11*P1_IVAN+F11*P2_IVAN+G11*P3_IVAN)-(H11+I11+J11)*(COSTE_DEV-IVA_DEV)-AM11-AO11</f>
-        <v>-71.94</v>
+        <v>-74.31</v>
       </c>
       <c r="Y11" s="33" t="n">
         <f aca="false">AH11-AI11-AJ11-AK11-AL11-AM11-AO11</f>
-        <v>43.5711735537191</v>
+        <v>57.0848429752066</v>
       </c>
       <c r="AA11" s="58" t="n">
         <f aca="false">MAX(0,B11-E11-H11)</f>
@@ -5732,7 +5734,7 @@
       </c>
       <c r="AB11" s="58" t="n">
         <f aca="false">MAX(0,C11-F11-I11)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AC11" s="58" t="n">
         <f aca="false">MAX(0,D11-G11-J11)</f>
@@ -5744,7 +5746,7 @@
       </c>
       <c r="AE11" s="59" t="n">
         <f aca="false">F11+AB11*TASA_USADA</f>
-        <v>1.6</v>
+        <v>2.4</v>
       </c>
       <c r="AF11" s="59" t="n">
         <f aca="false">G11+AC11*TASA_USADA</f>
@@ -5752,82 +5754,96 @@
       </c>
       <c r="AG11" s="59" t="n">
         <f aca="false">H11+I11+J11+(AA11+AB11+AC11)*(1-TASA_USADA)</f>
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="AH11" s="60" t="n">
         <f aca="false">AD11*P1_PVP+AE11*P2_PVP+AF11*P3_PVP</f>
-        <v>247.928</v>
+        <v>279.92</v>
       </c>
       <c r="AI11" s="60" t="n">
         <f aca="false">AD11*P1_CPROD+AE11*P2_CPROD+AF11*P3_CPROD</f>
-        <v>25.04216</v>
+        <v>28.8948</v>
       </c>
       <c r="AJ11" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L11),L11,E11*P1_LOG+F11*P2_LOG+G11*P3_LOG)+IF(ISNUMBER(M11),M11,AA11*P1_LOG+AB11*P2_LOG+AC11*P3_LOG)*TASA_USADA</f>
-        <v>54.184</v>
+        <v>59.944</v>
       </c>
       <c r="AK11" s="60" t="n">
         <f aca="false">AG11*COSTE_DEV</f>
-        <v>14.508</v>
+        <v>16.12</v>
       </c>
       <c r="AL11" s="60" t="n">
         <f aca="false">AD11*P1_IVAN+AE11*P2_IVAN+AF11*P3_IVAN-AG11*IVA_DEV</f>
-        <v>38.682666446281</v>
+        <v>43.5663570247934</v>
       </c>
       <c r="AM11" s="60" t="n">
         <f aca="false">N11*(1+RECARGO_ADS)</f>
-        <v>63.39</v>
+        <v>64.81</v>
       </c>
       <c r="AN11" s="58" t="n">
         <f aca="false">IF(ISNUMBER(L11),E11+F11+G11+AA11+AB11+AC11,0)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AO11" s="60" t="n">
         <f aca="false">P11*COMISION</f>
-        <v>8.55</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="53" t="n">
         <v>46306</v>
       </c>
-      <c r="B12" s="54"/>
-      <c r="C12" s="54"/>
-      <c r="D12" s="54"/>
+      <c r="B12" s="54" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="54" t="n">
+        <v>0</v>
+      </c>
       <c r="E12" s="54"/>
       <c r="F12" s="54"/>
       <c r="G12" s="54"/>
       <c r="H12" s="54"/>
       <c r="I12" s="54"/>
       <c r="J12" s="54"/>
-      <c r="K12" s="54"/>
-      <c r="L12" s="55"/>
-      <c r="M12" s="55"/>
-      <c r="N12" s="55"/>
+      <c r="K12" s="54" t="n">
+        <v>5</v>
+      </c>
+      <c r="L12" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="55" t="n">
+        <v>47.02</v>
+      </c>
+      <c r="N12" s="55" t="n">
+        <v>89.43</v>
+      </c>
       <c r="O12" s="56"/>
       <c r="P12" s="31" t="n">
         <f aca="false">B12+C12+D12</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q12" s="31" t="n">
         <f aca="false">AA12+AB12+AC12</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R12" s="32" t="n">
         <f aca="false">B12*P1_PVP+C12*P2_PVP+D12*P3_PVP</f>
-        <v>0</v>
-      </c>
-      <c r="S12" s="32" t="str">
+        <v>189.94</v>
+      </c>
+      <c r="S12" s="32" t="n">
         <f aca="false">IF(P12&gt;0,R12/P12,"")</f>
-        <v/>
-      </c>
-      <c r="T12" s="32" t="str">
+        <v>31.6566666666667</v>
+      </c>
+      <c r="T12" s="32" t="n">
         <f aca="false">IF(P12&gt;0,N12/P12,"")</f>
-        <v/>
-      </c>
-      <c r="U12" s="57" t="str">
+        <v>14.905</v>
+      </c>
+      <c r="U12" s="57" t="n">
         <f aca="false">IF(N12&gt;0,R12/N12,"")</f>
-        <v/>
+        <v>2.12389578441239</v>
       </c>
       <c r="V12" s="34" t="str">
         <f aca="false">IF(E12+F12+G12+H12+I12+J12&gt;0,(E12+F12+G12)/(E12+F12+G12+H12+I12+J12),"")</f>
@@ -5839,19 +5855,19 @@
       </c>
       <c r="X12" s="33" t="n">
         <f aca="false">W12-(E12*P1_IVAN+F12*P2_IVAN+G12*P3_IVAN)-(H12+I12+J12)*(COSTE_DEV-IVA_DEV)-AM12-AO12</f>
-        <v>0</v>
+        <v>-95.13</v>
       </c>
       <c r="Y12" s="33" t="n">
         <f aca="false">AH12-AI12-AJ12-AK12-AL12-AM12-AO12</f>
-        <v>0</v>
+        <v>-27.9818347107438</v>
       </c>
       <c r="AA12" s="58" t="n">
         <f aca="false">MAX(0,B12-E12-H12)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AB12" s="58" t="n">
         <f aca="false">MAX(0,C12-F12-I12)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC12" s="58" t="n">
         <f aca="false">MAX(0,D12-G12-J12)</f>
@@ -5859,11 +5875,11 @@
       </c>
       <c r="AD12" s="59" t="n">
         <f aca="false">E12+AA12*TASA_USADA</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AE12" s="59" t="n">
         <f aca="false">F12+AB12*TASA_USADA</f>
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="AF12" s="59" t="n">
         <f aca="false">G12+AC12*TASA_USADA</f>
@@ -5871,48 +5887,54 @@
       </c>
       <c r="AG12" s="59" t="n">
         <f aca="false">H12+I12+J12+(AA12+AB12+AC12)*(1-TASA_USADA)</f>
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="AH12" s="60" t="n">
         <f aca="false">AD12*P1_PVP+AE12*P2_PVP+AF12*P3_PVP</f>
-        <v>0</v>
+        <v>151.952</v>
       </c>
       <c r="AI12" s="60" t="n">
         <f aca="false">AD12*P1_CPROD+AE12*P2_CPROD+AF12*P3_CPROD</f>
-        <v>0</v>
+        <v>13.48424</v>
       </c>
       <c r="AJ12" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L12),L12,E12*P1_LOG+F12*P2_LOG+G12*P3_LOG)+IF(ISNUMBER(M12),M12,AA12*P1_LOG+AB12*P2_LOG+AC12*P3_LOG)*TASA_USADA</f>
-        <v>0</v>
+        <v>37.616</v>
       </c>
       <c r="AK12" s="60" t="n">
         <f aca="false">AG12*COSTE_DEV</f>
-        <v>0</v>
+        <v>9.672</v>
       </c>
       <c r="AL12" s="60" t="n">
         <f aca="false">AD12*P1_IVAN+AE12*P2_IVAN+AF12*P3_IVAN-AG12*IVA_DEV</f>
-        <v>0</v>
+        <v>24.0315947107438</v>
       </c>
       <c r="AM12" s="60" t="n">
         <f aca="false">N12*(1+RECARGO_ADS)</f>
-        <v>0</v>
+        <v>89.43</v>
       </c>
       <c r="AN12" s="58" t="n">
         <f aca="false">IF(ISNUMBER(L12),E12+F12+G12+AA12+AB12+AC12,0)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AO12" s="60" t="n">
         <f aca="false">P12*COMISION</f>
-        <v>0</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="53" t="n">
         <v>46307</v>
       </c>
-      <c r="B13" s="54"/>
-      <c r="C13" s="54"/>
-      <c r="D13" s="54"/>
+      <c r="B13" s="54" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="54" t="n">
+        <v>0</v>
+      </c>
       <c r="E13" s="54"/>
       <c r="F13" s="54"/>
       <c r="G13" s="54"/>
@@ -5920,33 +5942,39 @@
       <c r="I13" s="54"/>
       <c r="J13" s="54"/>
       <c r="K13" s="54"/>
-      <c r="L13" s="55"/>
-      <c r="M13" s="55"/>
-      <c r="N13" s="55"/>
+      <c r="L13" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="55" t="n">
+        <v>46.29</v>
+      </c>
+      <c r="N13" s="55" t="n">
+        <v>34.45</v>
+      </c>
       <c r="O13" s="56"/>
       <c r="P13" s="31" t="n">
         <f aca="false">B13+C13+D13</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q13" s="31" t="n">
         <f aca="false">AA13+AB13+AC13</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R13" s="32" t="n">
         <f aca="false">B13*P1_PVP+C13*P2_PVP+D13*P3_PVP</f>
-        <v>0</v>
-      </c>
-      <c r="S13" s="32" t="str">
+        <v>189.94</v>
+      </c>
+      <c r="S13" s="32" t="n">
         <f aca="false">IF(P13&gt;0,R13/P13,"")</f>
-        <v/>
-      </c>
-      <c r="T13" s="32" t="str">
+        <v>31.6566666666667</v>
+      </c>
+      <c r="T13" s="32" t="n">
         <f aca="false">IF(P13&gt;0,N13/P13,"")</f>
-        <v/>
-      </c>
-      <c r="U13" s="57" t="str">
+        <v>5.74166666666667</v>
+      </c>
+      <c r="U13" s="57" t="n">
         <f aca="false">IF(N13&gt;0,R13/N13,"")</f>
-        <v/>
+        <v>5.51349782293179</v>
       </c>
       <c r="V13" s="34" t="str">
         <f aca="false">IF(E13+F13+G13+H13+I13+J13&gt;0,(E13+F13+G13)/(E13+F13+G13+H13+I13+J13),"")</f>
@@ -5958,19 +5986,19 @@
       </c>
       <c r="X13" s="33" t="n">
         <f aca="false">W13-(E13*P1_IVAN+F13*P2_IVAN+G13*P3_IVAN)-(H13+I13+J13)*(COSTE_DEV-IVA_DEV)-AM13-AO13</f>
-        <v>0</v>
+        <v>-40.15</v>
       </c>
       <c r="Y13" s="33" t="n">
         <f aca="false">AH13-AI13-AJ13-AK13-AL13-AM13-AO13</f>
-        <v>0</v>
+        <v>27.5821652892562</v>
       </c>
       <c r="AA13" s="58" t="n">
         <f aca="false">MAX(0,B13-E13-H13)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AB13" s="58" t="n">
         <f aca="false">MAX(0,C13-F13-I13)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC13" s="58" t="n">
         <f aca="false">MAX(0,D13-G13-J13)</f>
@@ -5978,11 +6006,11 @@
       </c>
       <c r="AD13" s="59" t="n">
         <f aca="false">E13+AA13*TASA_USADA</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AE13" s="59" t="n">
         <f aca="false">F13+AB13*TASA_USADA</f>
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="AF13" s="59" t="n">
         <f aca="false">G13+AC13*TASA_USADA</f>
@@ -5990,39 +6018,39 @@
       </c>
       <c r="AG13" s="59" t="n">
         <f aca="false">H13+I13+J13+(AA13+AB13+AC13)*(1-TASA_USADA)</f>
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="AH13" s="60" t="n">
         <f aca="false">AD13*P1_PVP+AE13*P2_PVP+AF13*P3_PVP</f>
-        <v>0</v>
+        <v>151.952</v>
       </c>
       <c r="AI13" s="60" t="n">
         <f aca="false">AD13*P1_CPROD+AE13*P2_CPROD+AF13*P3_CPROD</f>
-        <v>0</v>
+        <v>13.48424</v>
       </c>
       <c r="AJ13" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L13),L13,E13*P1_LOG+F13*P2_LOG+G13*P3_LOG)+IF(ISNUMBER(M13),M13,AA13*P1_LOG+AB13*P2_LOG+AC13*P3_LOG)*TASA_USADA</f>
-        <v>0</v>
+        <v>37.032</v>
       </c>
       <c r="AK13" s="60" t="n">
         <f aca="false">AG13*COSTE_DEV</f>
-        <v>0</v>
+        <v>9.672</v>
       </c>
       <c r="AL13" s="60" t="n">
         <f aca="false">AD13*P1_IVAN+AE13*P2_IVAN+AF13*P3_IVAN-AG13*IVA_DEV</f>
-        <v>0</v>
+        <v>24.0315947107438</v>
       </c>
       <c r="AM13" s="60" t="n">
         <f aca="false">N13*(1+RECARGO_ADS)</f>
-        <v>0</v>
+        <v>34.45</v>
       </c>
       <c r="AN13" s="58" t="n">
         <f aca="false">IF(ISNUMBER(L13),E13+F13+G13+AA13+AB13+AC13,0)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AO13" s="60" t="n">
         <f aca="false">P13*COMISION</f>
-        <v>0</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51182,7 +51210,7 @@
       </c>
       <c r="C37" s="31" t="n">
         <f aca="false">(SUM(Diario!$E$6:$E$370)+SUM(Diario!$F$6:$F$370)+SUM(Diario!$G$6:$G$370))+(SUM(Diario!$H$6:$H$370)+SUM(Diario!$I$6:$I$370)+SUM(Diario!$J$6:$J$370))</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F37" s="67" t="s">
         <v>183</v>
@@ -51194,7 +51222,7 @@
       </c>
       <c r="C38" s="34" t="n">
         <f aca="false">IF(C37&gt;0,(SUM(Diario!$E$6:$E$370)+SUM(Diario!$F$6:$F$370)+SUM(Diario!$G$6:$G$370))/C37,"")</f>
-        <v>0.833333333333333</v>
+        <v>0.846153846153846</v>
       </c>
       <c r="F38" s="67" t="s">
         <v>185</v>
@@ -51218,11 +51246,11 @@
       </c>
       <c r="C40" s="34" t="n">
         <f aca="false">IF(SUM(Diario!$P$6:$P$370)&gt;0,SUM(Diario!$C$6:$C$370)/SUM(Diario!$P$6:$P$370),"")</f>
-        <v>0.327272727272727</v>
+        <v>0.308823529411765</v>
       </c>
       <c r="D40" s="34" t="n">
         <f aca="false">IF(SUM(Diario!$P$6:$P$370)&gt;0,SUM(Diario!$D$6:$D$370)/SUM(Diario!$P$6:$P$370),"")</f>
-        <v>0.0363636363636364</v>
+        <v>0.0294117647058824</v>
       </c>
       <c r="F40" s="67" t="s">
         <v>189</v>
@@ -51234,11 +51262,11 @@
       </c>
       <c r="C41" s="34" t="n">
         <f aca="false">IF(C40="",C26,C40)</f>
-        <v>0.327272727272727</v>
+        <v>0.308823529411765</v>
       </c>
       <c r="D41" s="34" t="n">
         <f aca="false">IF(D40="",D26,D40)</f>
-        <v>0.0363636363636364</v>
+        <v>0.0294117647058824</v>
       </c>
       <c r="F41" s="67"/>
     </row>
@@ -51248,7 +51276,7 @@
       </c>
       <c r="C42" s="32" t="n">
         <f aca="false">IF(SUM(Diario!$AN$6:$AN$370)&gt;0,(SUM(Diario!$L$6:$L$370)+SUM(Diario!$M$6:$M$370))/SUM(Diario!$AN$6:$AN$370),"")</f>
-        <v>7.57679245283019</v>
+        <v>7.60727272727273</v>
       </c>
       <c r="F42" s="67" t="s">
         <v>192</v>
@@ -51260,7 +51288,7 @@
       </c>
       <c r="C43" s="32" t="n">
         <f aca="false">(1-C41-D41)*C5+C41*D5+D41*E5</f>
-        <v>33.99</v>
+        <v>33.6664705882353</v>
       </c>
       <c r="F43" s="67"/>
     </row>
@@ -51270,7 +51298,7 @@
       </c>
       <c r="C44" s="32" t="n">
         <f aca="false">(1-C41-D41)*(C5-C9-IF(C42="",C8,C42)-C14)+C41*(D5-D9-IF(C42="",D8,C42)-D14)+D41*(E5-E9-IF(C42="",E8,C42)-E14)</f>
-        <v>17.7281166380789</v>
+        <v>17.4946390374332</v>
       </c>
       <c r="F44" s="67" t="s">
         <v>195</v>
@@ -51282,7 +51310,7 @@
       </c>
       <c r="C45" s="32" t="n">
         <f aca="false">C39*C44-(1-C39)*C36-COMISION</f>
-        <v>11.6204933104631</v>
+        <v>11.4337112299465</v>
       </c>
       <c r="F45" s="67" t="s">
         <v>197</v>
@@ -51294,7 +51322,7 @@
       </c>
       <c r="C46" s="33" t="n">
         <f aca="false">C45/(1+RECARGO_ADS)</f>
-        <v>11.6204933104631</v>
+        <v>11.4337112299465</v>
       </c>
       <c r="F46" s="67" t="s">
         <v>199</v>
@@ -51306,7 +51334,7 @@
       </c>
       <c r="C47" s="72" t="n">
         <f aca="false">IF(C46&gt;0,C43/C46,"")</f>
-        <v>2.92500491088406</v>
+        <v>2.94449194239382</v>
       </c>
       <c r="F47" s="67" t="s">
         <v>201</v>

</xml_diff>

<commit_message>
Auditoría 14/10: importadores aceptan cabeceras COSTO y no cuentan carritos sin confirmar
Dropi cambió COSTE por COSTO en el export: la página ponía 8,06 € de envío a todo y
el script fallaba. Un carrito en 'Pendiente de confirmación' ya no cuenta como pedido.
Contabilidad regenerada con el export del 14/10 (86 pedidos, liquidación 445,42 €).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFjE4yx23BY3D6kaMQowKe
</commit_message>
<xml_diff>
--- a/contabilidad/CeraLux_Contabilidad.xlsx
+++ b/contabilidad/CeraLux_Contabilidad.xlsx
@@ -1779,46 +1779,46 @@
               <c:strCache>
                 <c:ptCount val="14"/>
                 <c:pt idx="0">
-                  <c:v>Tue 29/09</c:v>
+                  <c:v>Thu 01/10</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Wed 30/09</c:v>
+                  <c:v>Fri 02/10</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Thu 01/10</c:v>
+                  <c:v>Sat 03/10</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Fri 02/10</c:v>
+                  <c:v>Sun 04/10</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Sat 03/10</c:v>
+                  <c:v>Mon 05/10</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Sun 04/10</c:v>
+                  <c:v>Tue 06/10</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Mon 05/10</c:v>
+                  <c:v>Wed 07/10</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>Tue 06/10</c:v>
+                  <c:v>Thu 08/10</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Wed 07/10</c:v>
+                  <c:v>Fri 09/10</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Thu 08/10</c:v>
+                  <c:v>Sat 10/10</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Fri 09/10</c:v>
+                  <c:v>Sun 11/10</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>Sat 10/10</c:v>
+                  <c:v>Mon 12/10</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>Sun 11/10</c:v>
+                  <c:v>Tue 13/10</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>Mon 12/10</c:v>
+                  <c:v>Wed 14/10</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1842,34 +1842,34 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>62.6280826446281</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>8.63823140495868</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>62.6280826446281</c:v>
+                  <c:v>38.9722314049587</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>8.63823140495868</c:v>
+                  <c:v>107.506859504132</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>32.9863140495868</c:v>
+                  <c:v>27.0542314049587</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>128.044396694215</c:v>
+                  <c:v>47.6401983471074</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>36.5688760330579</c:v>
+                  <c:v>-28.0618347107438</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>57.0848429752066</c:v>
+                  <c:v>93.2363801652893</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>-27.9818347107438</c:v>
+                  <c:v>23.9875041322314</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>27.5821652892562</c:v>
+                  <c:v>1.54396694214877</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1877,8 +1877,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="65940706"/>
-        <c:axId val="67586164"/>
+        <c:axId val="75265296"/>
+        <c:axId val="12966900"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -1942,46 +1942,46 @@
               <c:strCache>
                 <c:ptCount val="14"/>
                 <c:pt idx="0">
-                  <c:v>Tue 29/09</c:v>
+                  <c:v>Thu 01/10</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Wed 30/09</c:v>
+                  <c:v>Fri 02/10</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Thu 01/10</c:v>
+                  <c:v>Sat 03/10</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Fri 02/10</c:v>
+                  <c:v>Sun 04/10</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Sat 03/10</c:v>
+                  <c:v>Mon 05/10</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Sun 04/10</c:v>
+                  <c:v>Tue 06/10</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Mon 05/10</c:v>
+                  <c:v>Wed 07/10</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>Tue 06/10</c:v>
+                  <c:v>Thu 08/10</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Wed 07/10</c:v>
+                  <c:v>Fri 09/10</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Thu 08/10</c:v>
+                  <c:v>Sat 10/10</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Fri 09/10</c:v>
+                  <c:v>Sun 11/10</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>Sat 10/10</c:v>
+                  <c:v>Mon 12/10</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>Sun 11/10</c:v>
+                  <c:v>Tue 13/10</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>Mon 12/10</c:v>
+                  <c:v>Wed 14/10</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2005,34 +2005,34 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>67.67</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>70.18</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>67.67</c:v>
+                  <c:v>47.78</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>70.18</c:v>
+                  <c:v>50.46</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>47.78</c:v>
+                  <c:v>41.21</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>50.46</c:v>
+                  <c:v>64.81</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>41.21</c:v>
+                  <c:v>89.51</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>64.81</c:v>
+                  <c:v>78.33</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>89.43</c:v>
+                  <c:v>68.04</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>34.45</c:v>
+                  <c:v>40.38</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2047,11 +2047,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="65940706"/>
-        <c:axId val="67586164"/>
+        <c:axId val="75265296"/>
+        <c:axId val="12966900"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="65940706"/>
+        <c:axId val="75265296"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2083,7 +2083,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="67586164"/>
+        <c:crossAx val="12966900"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2091,7 +2091,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="67586164"/>
+        <c:axId val="12966900"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2133,7 +2133,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="65940706"/>
+        <c:crossAx val="75265296"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2332,7 +2332,7 @@
                 <c:formatCode>#,##0" €";[RED]\-#,##0" €";\-</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>325.551074380165</c:v>
+                  <c:v>383.14585123967</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -2373,8 +2373,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="85087024"/>
-        <c:axId val="50170899"/>
+        <c:axId val="60977798"/>
+        <c:axId val="32316078"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2471,11 +2471,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="85087024"/>
-        <c:axId val="50170899"/>
+        <c:axId val="60977798"/>
+        <c:axId val="32316078"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="85087024"/>
+        <c:axId val="60977798"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2507,7 +2507,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="50170899"/>
+        <c:crossAx val="32316078"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2515,7 +2515,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="50170899"/>
+        <c:axId val="32316078"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2557,7 +2557,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="85087024"/>
+        <c:crossAx val="60977798"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="F3" s="4" t="n">
         <f aca="true">TODAY()</f>
-        <v>46307</v>
+        <v>46309</v>
       </c>
       <c r="G3" s="4"/>
       <c r="H3" s="3" t="s">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="I3" s="5" t="n">
         <f aca="false">MAX(1,$F$3-$C$3+1)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="J3" s="6" t="s">
         <v>5</v>
@@ -2951,32 +2951,32 @@
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="10" t="n">
         <f aca="false">F25</f>
-        <v>325.551074380166</v>
+        <v>383.145851239669</v>
       </c>
       <c r="C7" s="10"/>
       <c r="D7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$W$6:$W$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>250.5915</v>
+        <v>445.4167</v>
       </c>
       <c r="E7" s="10"/>
       <c r="F7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$X$6:$X$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+F24</f>
-        <v>-354.045785123967</v>
+        <v>-388.38694214876</v>
       </c>
       <c r="G7" s="10"/>
       <c r="H7" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="I7" s="11"/>
       <c r="J7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$R$6:$R$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>2289.32</v>
+        <v>2909.14</v>
       </c>
       <c r="K7" s="10"/>
       <c r="L7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>465.99</v>
+        <v>618.37</v>
       </c>
       <c r="M7" s="10"/>
     </row>
@@ -3009,32 +3009,32 @@
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="10" t="n">
         <f aca="false">IF(H7&gt;0,L7/H7,"")</f>
-        <v>6.85279411764706</v>
+        <v>7.1903488372093</v>
       </c>
       <c r="C10" s="10"/>
       <c r="D10" s="10" t="n">
         <f aca="false">CPA_BE</f>
-        <v>11.4337112299465</v>
+        <v>11.5304572408976</v>
       </c>
       <c r="E10" s="10"/>
       <c r="F10" s="12" t="n">
         <f aca="false">IF(L7&gt;0,J7/L7,"")</f>
-        <v>4.91280928775296</v>
+        <v>4.70452965053285</v>
       </c>
       <c r="G10" s="12"/>
       <c r="H10" s="12" t="n">
         <f aca="false">ROAS_BE</f>
-        <v>2.94449194239382</v>
+        <v>2.93372661600471</v>
       </c>
       <c r="I10" s="12"/>
       <c r="J10" s="10" t="n">
         <f aca="false">IF(H7&gt;0,J7/H7,"")</f>
-        <v>33.6664705882353</v>
+        <v>33.8272093023256</v>
       </c>
       <c r="K10" s="10"/>
       <c r="L10" s="13" t="n">
         <f aca="false">IF(H7&gt;0,(SUMIFS(Diario!$C$6:$C$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+SUMIFS(Diario!$D$6:$D$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3))/H7,"")</f>
-        <v>0.338235294117647</v>
+        <v>0.325581395348837</v>
       </c>
       <c r="M10" s="13"/>
     </row>
@@ -3067,27 +3067,27 @@
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="C13" s="11"/>
       <c r="D13" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$Q$6:$Q$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="E13" s="11"/>
       <c r="F13" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$K$6:$K$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G13" s="11"/>
       <c r="H13" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I13" s="11"/>
       <c r="J13" s="13" t="n">
         <f aca="false">IF(B13+H13&gt;0,B13/(B13+H13),"")</f>
-        <v>0.846153846153846</v>
+        <v>0.826086956521739</v>
       </c>
       <c r="K13" s="13"/>
       <c r="L13" s="14" t="str">
@@ -3124,7 +3124,7 @@
       </c>
       <c r="F16" s="17" t="n">
         <f aca="false">SUMIFS(Diario!$AH$6:$AH$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>1849.45</v>
+        <v>2337.306</v>
       </c>
       <c r="H16" s="15" t="s">
         <v>29</v>
@@ -3146,11 +3146,11 @@
       <c r="D17" s="15"/>
       <c r="E17" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F17/$F$16,"")</f>
-        <v>-0.0976465976371353</v>
+        <v>-0.0978692990990482</v>
       </c>
       <c r="F17" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AI$6:$AI$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-180.5925</v>
+        <v>-228.7505</v>
       </c>
       <c r="H17" s="15" t="s">
         <v>31</v>
@@ -3160,7 +3160,7 @@
       <c r="K17" s="15"/>
       <c r="L17" s="20" t="n">
         <f aca="false">F25/I3</f>
-        <v>27.1292561983471</v>
+        <v>27.3675608028335</v>
       </c>
       <c r="M17" s="20"/>
     </row>
@@ -3172,11 +3172,11 @@
       <c r="D18" s="15"/>
       <c r="E18" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F18/$F$16,"")</f>
-        <v>-0.226175349428208</v>
+        <v>-0.224872566963846</v>
       </c>
       <c r="F18" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AJ$6:$AJ$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-418.3</v>
+        <v>-525.596</v>
       </c>
       <c r="H18" s="15" t="s">
         <v>33</v>
@@ -3186,7 +3186,7 @@
       <c r="K18" s="15"/>
       <c r="L18" s="18" t="n">
         <f aca="false">L17*30</f>
-        <v>813.877685950414</v>
+        <v>821.026824085006</v>
       </c>
       <c r="M18" s="18"/>
     </row>
@@ -3198,11 +3198,11 @@
       <c r="D19" s="15"/>
       <c r="E19" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F19/$F$16,"")</f>
-        <v>-0.0566546811214145</v>
+        <v>-0.0572436814007237</v>
       </c>
       <c r="F19" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AK$6:$AK$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-104.78</v>
+        <v>-133.796</v>
       </c>
       <c r="H19" s="21" t="s">
         <v>35</v>
@@ -3212,7 +3212,7 @@
       <c r="K19" s="21"/>
       <c r="L19" s="22" t="n">
         <f aca="false">IF(L16&gt;0,L18/L16,"")</f>
-        <v>0.0813877685950414</v>
+        <v>0.0821026824085006</v>
       </c>
       <c r="M19" s="22"/>
     </row>
@@ -3224,11 +3224,11 @@
       <c r="D20" s="15"/>
       <c r="E20" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F20/$F$16,"")</f>
-        <v>-0.0349293033063884</v>
+        <v>-0.0349547727169656</v>
       </c>
       <c r="F20" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AO$6:$AO$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-64.6</v>
+        <v>-81.7</v>
       </c>
       <c r="H20" s="15" t="s">
         <v>37</v>
@@ -3238,7 +3238,7 @@
       <c r="K20" s="15"/>
       <c r="L20" s="20" t="n">
         <f aca="false">BEN_PEDIDO</f>
-        <v>11.4337112299465</v>
+        <v>11.5304572408976</v>
       </c>
       <c r="M20" s="20"/>
     </row>
@@ -3250,11 +3250,11 @@
       <c r="D21" s="15"/>
       <c r="E21" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F21/$F$16,"")</f>
-        <v>-0.156606788839836</v>
+        <v>-0.156568138172892</v>
       </c>
       <c r="F21" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AL$6:$AL$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-289.636425619835</v>
+        <v>-365.947648760331</v>
       </c>
       <c r="H21" s="15" t="s">
         <v>39</v>
@@ -3264,7 +3264,7 @@
       <c r="K21" s="15"/>
       <c r="L21" s="20" t="n">
         <f aca="false">B10</f>
-        <v>6.85279411764706</v>
+        <v>7.1903488372093</v>
       </c>
       <c r="M21" s="20"/>
     </row>
@@ -3276,11 +3276,11 @@
       <c r="D22" s="15"/>
       <c r="E22" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F22/$F$16,"")</f>
-        <v>-0.251961393927925</v>
+        <v>-0.264565273010894</v>
       </c>
       <c r="F22" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AM$6:$AM$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-465.99</v>
+        <v>-618.37</v>
       </c>
       <c r="H22" s="15" t="s">
         <v>41</v>
@@ -3290,7 +3290,7 @@
       <c r="K22" s="15"/>
       <c r="L22" s="20" t="n">
         <f aca="false">IF(ISNUMBER(L21),L20-L21*(1+RECARGO_ADS),"")</f>
-        <v>4.58091711229946</v>
+        <v>4.3401084036883</v>
       </c>
       <c r="M22" s="20"/>
     </row>
@@ -3302,11 +3302,11 @@
       <c r="D23" s="23"/>
       <c r="E23" s="24" t="n">
         <f aca="false">IF($F$16&gt;0,F23/$F$16,"")</f>
-        <v>0.176025885739093</v>
+        <v>0.16392626863563</v>
       </c>
       <c r="F23" s="25" t="n">
         <f aca="false">SUM(F16:F22)</f>
-        <v>325.551074380166</v>
+        <v>383.145851239669</v>
       </c>
       <c r="H23" s="21" t="s">
         <v>43</v>
@@ -3316,7 +3316,7 @@
       <c r="K23" s="21"/>
       <c r="L23" s="26" t="n">
         <f aca="false">IF(NOT(ISNUMBER(L22)),"",IF(L22&lt;=0,"Baja el CPA",ROUNDUP((L16-F24/I3*30)/30/L22,0)))</f>
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="M23" s="26"/>
     </row>
@@ -3342,7 +3342,7 @@
       <c r="K24" s="15"/>
       <c r="L24" s="18" t="n">
         <f aca="false">IF(ISNUMBER(L23),L23*L21,"")</f>
-        <v>500.253970588235</v>
+        <v>553.656860465116</v>
       </c>
       <c r="M24" s="18"/>
     </row>
@@ -3354,11 +3354,11 @@
       <c r="D25" s="23"/>
       <c r="E25" s="24" t="n">
         <f aca="false">IF($F$16&gt;0,F25/$F$16,"")</f>
-        <v>0.176025885739093</v>
+        <v>0.16392626863563</v>
       </c>
       <c r="F25" s="25" t="n">
         <f aca="false">F23+F24</f>
-        <v>325.551074380166</v>
+        <v>383.145851239669</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3369,7 +3369,7 @@
       <c r="D26" s="27"/>
       <c r="F26" s="28" t="n">
         <f aca="false">IF(F16&gt;0,F25/F16,"")</f>
-        <v>0.176025885739093</v>
+        <v>0.16392626863563</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3405,7 +3405,7 @@
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="30" t="n">
         <f aca="false">$F$3-13</f>
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="C29" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B29)</f>
@@ -3431,7 +3431,7 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="30" t="n">
         <f aca="false">$F$3-12</f>
-        <v>46295</v>
+        <v>46297</v>
       </c>
       <c r="C30" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B30)</f>
@@ -3457,7 +3457,7 @@
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="30" t="n">
         <f aca="false">$F$3-11</f>
-        <v>46296</v>
+        <v>46298</v>
       </c>
       <c r="C31" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B31)</f>
@@ -3483,7 +3483,7 @@
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="30" t="n">
         <f aca="false">$F$3-10</f>
-        <v>46297</v>
+        <v>46299</v>
       </c>
       <c r="C32" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B32)</f>
@@ -3509,75 +3509,75 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="30" t="n">
         <f aca="false">$F$3-9</f>
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="C33" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B33)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D33" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B33)</f>
-        <v>0</v>
-      </c>
-      <c r="E33" s="32" t="str">
+        <v>67.67</v>
+      </c>
+      <c r="E33" s="32" t="n">
         <f aca="false">IF(C33&gt;0,D33/C33,"")</f>
-        <v/>
+        <v>7.51888888888889</v>
       </c>
       <c r="F33" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B33)</f>
-        <v>0</v>
-      </c>
-      <c r="G33" s="34" t="str">
+        <v>62.6280826446281</v>
+      </c>
+      <c r="G33" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B33))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B33))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B33)),"")</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="30" t="n">
         <f aca="false">$F$3-8</f>
-        <v>46299</v>
+        <v>46301</v>
       </c>
       <c r="C34" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B34)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D34" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B34)</f>
-        <v>0</v>
-      </c>
-      <c r="E34" s="32" t="str">
+        <v>70.18</v>
+      </c>
+      <c r="E34" s="32" t="n">
         <f aca="false">IF(C34&gt;0,D34/C34,"")</f>
-        <v/>
+        <v>8.7725</v>
       </c>
       <c r="F34" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B34)</f>
-        <v>0</v>
-      </c>
-      <c r="G34" s="34" t="str">
+        <v>8.63823140495868</v>
+      </c>
+      <c r="G34" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B34))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B34))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B34)),"")</f>
-        <v/>
+        <v>0.75</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="30" t="n">
         <f aca="false">$F$3-7</f>
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="C35" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B35)</f>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D35" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B35)</f>
-        <v>67.67</v>
+        <v>47.78</v>
       </c>
       <c r="E35" s="32" t="n">
         <f aca="false">IF(C35&gt;0,D35/C35,"")</f>
-        <v>7.51888888888889</v>
+        <v>6.82571428571429</v>
       </c>
       <c r="F35" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B35)</f>
-        <v>62.6280826446281</v>
+        <v>38.9722314049587</v>
       </c>
       <c r="G35" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B35))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B35))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B35)),"")</f>
@@ -3587,49 +3587,49 @@
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="30" t="n">
         <f aca="false">$F$3-6</f>
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="C36" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B36)</f>
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D36" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B36)</f>
-        <v>70.18</v>
+        <v>50.46</v>
       </c>
       <c r="E36" s="32" t="n">
         <f aca="false">IF(C36&gt;0,D36/C36,"")</f>
-        <v>8.7725</v>
+        <v>3.15375</v>
       </c>
       <c r="F36" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B36)</f>
-        <v>8.63823140495868</v>
+        <v>107.506859504132</v>
       </c>
       <c r="G36" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B36))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B36))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B36)),"")</f>
-        <v>0.75</v>
+        <v>0.666666666666667</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="30" t="n">
         <f aca="false">$F$3-5</f>
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="C37" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B37)</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D37" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B37)</f>
-        <v>47.78</v>
+        <v>41.21</v>
       </c>
       <c r="E37" s="32" t="n">
         <f aca="false">IF(C37&gt;0,D37/C37,"")</f>
-        <v>6.82571428571429</v>
+        <v>8.242</v>
       </c>
       <c r="F37" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B37)</f>
-        <v>32.9863140495868</v>
+        <v>27.0542314049587</v>
       </c>
       <c r="G37" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B37))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B37))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B37)),"")</f>
@@ -3639,33 +3639,33 @@
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="30" t="n">
         <f aca="false">$F$3-4</f>
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="C38" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B38)</f>
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="D38" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B38)</f>
-        <v>50.46</v>
+        <v>64.81</v>
       </c>
       <c r="E38" s="32" t="n">
         <f aca="false">IF(C38&gt;0,D38/C38,"")</f>
-        <v>3.15375</v>
+        <v>7.20111111111111</v>
       </c>
       <c r="F38" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B38)</f>
-        <v>128.044396694215</v>
+        <v>47.6401983471074</v>
       </c>
       <c r="G38" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B38))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B38))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B38)),"")</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="30" t="n">
         <f aca="false">$F$3-3</f>
-        <v>46304</v>
+        <v>46306</v>
       </c>
       <c r="C39" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B39)</f>
@@ -3673,15 +3673,15 @@
       </c>
       <c r="D39" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B39)</f>
-        <v>41.21</v>
+        <v>89.51</v>
       </c>
       <c r="E39" s="32" t="n">
         <f aca="false">IF(C39&gt;0,D39/C39,"")</f>
-        <v>6.86833333333333</v>
+        <v>14.9183333333333</v>
       </c>
       <c r="F39" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B39)</f>
-        <v>36.5688760330579</v>
+        <v>-28.0618347107438</v>
       </c>
       <c r="G39" s="34" t="str">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B39))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B39))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B39)),"")</f>
@@ -3691,23 +3691,23 @@
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="30" t="n">
         <f aca="false">$F$3-2</f>
-        <v>46305</v>
+        <v>46307</v>
       </c>
       <c r="C40" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B40)</f>
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D40" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B40)</f>
-        <v>64.81</v>
+        <v>78.33</v>
       </c>
       <c r="E40" s="32" t="n">
         <f aca="false">IF(C40&gt;0,D40/C40,"")</f>
-        <v>6.481</v>
+        <v>5.595</v>
       </c>
       <c r="F40" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B40)</f>
-        <v>57.0848429752066</v>
+        <v>93.2363801652893</v>
       </c>
       <c r="G40" s="34" t="str">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B40))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B40))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B40)),"")</f>
@@ -3717,23 +3717,23 @@
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="30" t="n">
         <f aca="false">$F$3-1</f>
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="C41" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B41)</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D41" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B41)</f>
-        <v>89.43</v>
+        <v>68.04</v>
       </c>
       <c r="E41" s="32" t="n">
         <f aca="false">IF(C41&gt;0,D41/C41,"")</f>
-        <v>14.905</v>
+        <v>8.505</v>
       </c>
       <c r="F41" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B41)</f>
-        <v>-27.9818347107438</v>
+        <v>23.9875041322314</v>
       </c>
       <c r="G41" s="34" t="str">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B41))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B41))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B41)),"")</f>
@@ -3743,23 +3743,23 @@
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="30" t="n">
         <f aca="false">$F$3-0</f>
-        <v>46307</v>
+        <v>46309</v>
       </c>
       <c r="C42" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B42)</f>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D42" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B42)</f>
-        <v>34.45</v>
+        <v>40.38</v>
       </c>
       <c r="E42" s="32" t="n">
         <f aca="false">IF(C42&gt;0,D42/C42,"")</f>
-        <v>5.74166666666667</v>
+        <v>10.095</v>
       </c>
       <c r="F42" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B42)</f>
-        <v>27.5821652892562</v>
+        <v>1.54396694214877</v>
       </c>
       <c r="G42" s="34" t="str">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B42))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B42))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B42)),"")</f>
@@ -3830,35 +3830,35 @@
       </c>
       <c r="C47" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="D47" s="37" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>465.99</v>
+        <v>618.37</v>
       </c>
       <c r="E47" s="32" t="n">
         <f aca="false">IF(C47&gt;0,D47/C47,"")</f>
-        <v>6.85279411764706</v>
+        <v>7.1903488372093</v>
       </c>
       <c r="F47" s="37" t="n">
         <f aca="false">SUMIFS(Diario!$R$6:$R$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>2289.32</v>
+        <v>2909.14</v>
       </c>
       <c r="G47" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="H47" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I47" s="34" t="n">
         <f aca="false">IF(G47+H47&gt;0,G47/(G47+H47),"")</f>
-        <v>0.846153846153846</v>
+        <v>0.826086956521739</v>
       </c>
       <c r="J47" s="37" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>325.551074380165</v>
+        <v>383.14585123967</v>
       </c>
       <c r="K47" s="37" t="n">
         <f aca="false">-SUMIFS(Gastos!$D$5:$D$304,Gastos!$A$5:$A$304,"&gt;="&amp;$B47,Gastos!$A$5:$A$304,"&lt;="&amp;EOMONTH($B47,0))</f>
@@ -3866,11 +3866,11 @@
       </c>
       <c r="L47" s="38" t="n">
         <f aca="false">J47+K47</f>
-        <v>325.551074380165</v>
+        <v>383.14585123967</v>
       </c>
       <c r="M47" s="34" t="n">
         <f aca="false">IF(OBJETIVO_MES&gt;0,L47/OBJETIVO_MES,"")</f>
-        <v>0.0325551074380165</v>
+        <v>0.038314585123967</v>
       </c>
       <c r="O47" s="39" t="n">
         <f aca="false">OBJETIVO_MES</f>
@@ -4477,35 +4477,35 @@
       </c>
       <c r="C59" s="41" t="n">
         <f aca="false">SUM(C47:C58)</f>
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="D59" s="42" t="n">
         <f aca="false">SUM(D47:D58)</f>
-        <v>465.99</v>
+        <v>618.37</v>
       </c>
       <c r="E59" s="43" t="n">
         <f aca="false">IF(C59&gt;0,D59/C59,"")</f>
-        <v>6.85279411764706</v>
+        <v>7.1903488372093</v>
       </c>
       <c r="F59" s="42" t="n">
         <f aca="false">SUM(F47:F58)</f>
-        <v>2289.32</v>
+        <v>2909.14</v>
       </c>
       <c r="G59" s="41" t="n">
         <f aca="false">SUM(G47:G58)</f>
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="H59" s="41" t="n">
         <f aca="false">SUM(H47:H58)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I59" s="44" t="n">
         <f aca="false">IF(G59+H59&gt;0,G59/(G59+H59),"")</f>
-        <v>0.846153846153846</v>
+        <v>0.826086956521739</v>
       </c>
       <c r="J59" s="42" t="n">
         <f aca="false">SUM(J47:J58)</f>
-        <v>325.551074380165</v>
+        <v>383.14585123967</v>
       </c>
       <c r="K59" s="42" t="n">
         <f aca="false">SUM(K47:K58)</f>
@@ -4513,7 +4513,7 @@
       </c>
       <c r="L59" s="42" t="n">
         <f aca="false">SUM(L47:L58)</f>
-        <v>325.551074380165</v>
+        <v>383.14585123967</v>
       </c>
       <c r="M59" s="45"/>
     </row>
@@ -4700,27 +4700,27 @@
       </c>
       <c r="B4" s="47" t="n">
         <f aca="false">SUM(B6:B370)</f>
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="C4" s="47" t="n">
         <f aca="false">SUM(C6:C370)</f>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D4" s="47" t="n">
         <f aca="false">SUM(D6:D370)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E4" s="47" t="n">
         <f aca="false">SUM(E6:E370)</f>
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="F4" s="47" t="n">
         <f aca="false">SUM(F6:F370)</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G4" s="47" t="n">
         <f aca="false">SUM(G6:G370)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" s="47" t="n">
         <f aca="false">SUM(H6:H370)</f>
@@ -4728,7 +4728,7 @@
       </c>
       <c r="I4" s="47" t="n">
         <f aca="false">SUM(I6:I370)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J4" s="47" t="n">
         <f aca="false">SUM(J6:J370)</f>
@@ -4736,119 +4736,119 @@
       </c>
       <c r="K4" s="47" t="n">
         <f aca="false">SUM(K6:K370)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L4" s="48" t="n">
         <f aca="false">SUM(L6:L370)</f>
-        <v>83.18</v>
+        <v>139.38</v>
       </c>
       <c r="M4" s="48" t="n">
         <f aca="false">SUM(M6:M370)</f>
-        <v>418.9</v>
+        <v>482.77</v>
       </c>
       <c r="N4" s="48" t="n">
         <f aca="false">SUM(N6:N370)</f>
-        <v>465.99</v>
+        <v>618.37</v>
       </c>
       <c r="P4" s="47" t="n">
         <f aca="false">SUM(P6:P370)</f>
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="Q4" s="47" t="n">
         <f aca="false">SUM(Q6:Q370)</f>
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="R4" s="48" t="n">
         <f aca="false">SUM(R6:R370)</f>
-        <v>2289.32</v>
+        <v>2909.14</v>
       </c>
       <c r="S4" s="48" t="n">
         <f aca="false">IF(P4&gt;0,R4/P4,"")</f>
-        <v>33.6664705882353</v>
+        <v>33.8272093023256</v>
       </c>
       <c r="T4" s="48" t="n">
         <f aca="false">IF(P4&gt;0,N4/P4,"")</f>
-        <v>6.85279411764706</v>
+        <v>7.1903488372093</v>
       </c>
       <c r="U4" s="49" t="n">
         <f aca="false">IF(N4&gt;0,R4/N4,"")</f>
-        <v>4.91280928775296</v>
+        <v>4.70452965053285</v>
       </c>
       <c r="V4" s="50" t="n">
         <f aca="false">IF(E4+F4+G4+H4+I4+J4&gt;0,(E4+F4+G4)/(E4+F4+G4+H4+I4+J4),"")</f>
-        <v>0.846153846153846</v>
+        <v>0.826086956521739</v>
       </c>
       <c r="W4" s="48" t="n">
         <f aca="false">SUM(W6:W370)</f>
-        <v>250.5915</v>
+        <v>445.4167</v>
       </c>
       <c r="X4" s="48" t="n">
         <f aca="false">SUM(X6:X370)</f>
-        <v>-354.045785123967</v>
+        <v>-388.38694214876</v>
       </c>
       <c r="Y4" s="48" t="n">
         <f aca="false">SUM(Y6:Y370)</f>
-        <v>325.551074380165</v>
+        <v>383.14585123967</v>
       </c>
       <c r="AA4" s="47" t="n">
         <f aca="false">SUM(AA6:AA370)</f>
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="AB4" s="47" t="n">
         <f aca="false">SUM(AB6:AB370)</f>
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="AC4" s="47" t="n">
         <f aca="false">SUM(AC6:AC370)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AD4" s="51" t="n">
         <f aca="false">SUM(AD6:AD370)</f>
-        <v>36.6</v>
+        <v>48</v>
       </c>
       <c r="AE4" s="51" t="n">
         <f aca="false">SUM(AE6:AE370)</f>
-        <v>16.8</v>
+        <v>17.2</v>
       </c>
       <c r="AF4" s="51" t="n">
         <f aca="false">SUM(AF6:AF370)</f>
-        <v>1.6</v>
+        <v>4.2</v>
       </c>
       <c r="AG4" s="51" t="n">
         <f aca="false">SUM(AG6:AG370)</f>
-        <v>13</v>
+        <v>16.6</v>
       </c>
       <c r="AH4" s="48" t="n">
         <f aca="false">SUM(AH6:AH370)</f>
-        <v>1849.45</v>
+        <v>2337.306</v>
       </c>
       <c r="AI4" s="48" t="n">
         <f aca="false">SUM(AI6:AI370)</f>
-        <v>180.5925</v>
+        <v>228.7505</v>
       </c>
       <c r="AJ4" s="48" t="n">
         <f aca="false">SUM(AJ6:AJ370)</f>
-        <v>418.3</v>
+        <v>525.596</v>
       </c>
       <c r="AK4" s="48" t="n">
         <f aca="false">SUM(AK6:AK370)</f>
-        <v>104.78</v>
+        <v>133.796</v>
       </c>
       <c r="AL4" s="48" t="n">
         <f aca="false">SUM(AL6:AL370)</f>
-        <v>289.636425619835</v>
+        <v>365.947648760331</v>
       </c>
       <c r="AM4" s="48" t="n">
         <f aca="false">SUM(AM6:AM370)</f>
-        <v>465.99</v>
+        <v>618.37</v>
       </c>
       <c r="AN4" s="47" t="n">
         <f aca="false">SUM(AN6:AN370)</f>
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="AO4" s="48" t="n">
         <f aca="false">SUM(AO6:AO370)</f>
-        <v>64.6</v>
+        <v>81.7</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4997,7 +4997,7 @@
       <c r="I6" s="54"/>
       <c r="J6" s="54"/>
       <c r="K6" s="54" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L6" s="55" t="n">
         <v>38.42</v>
@@ -5267,19 +5267,21 @@
       <c r="E8" s="54" t="n">
         <v>2</v>
       </c>
-      <c r="F8" s="54"/>
+      <c r="F8" s="54" t="n">
+        <v>1</v>
+      </c>
       <c r="G8" s="54"/>
       <c r="H8" s="54"/>
       <c r="I8" s="54"/>
       <c r="J8" s="54"/>
       <c r="K8" s="54" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L8" s="55" t="n">
-        <v>15.45</v>
+        <v>22.65</v>
       </c>
       <c r="M8" s="55" t="n">
-        <v>38.58</v>
+        <v>31.38</v>
       </c>
       <c r="N8" s="55" t="n">
         <v>47.78</v>
@@ -5291,7 +5293,7 @@
       </c>
       <c r="Q8" s="31" t="n">
         <f aca="false">AA8+AB8+AC8</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R8" s="32" t="n">
         <f aca="false">B8*P1_PVP+C8*P2_PVP+D8*P3_PVP</f>
@@ -5315,15 +5317,15 @@
       </c>
       <c r="W8" s="33" t="n">
         <f aca="false">E8*(P1_PVP-P1_CPROD)+F8*(P2_PVP-P2_CPROD)+G8*(P3_PVP-P3_CPROD)-IF(ISNUMBER(L8),L8,E8*P1_LOG+F8*P2_LOG+G8*P3_LOG)</f>
-        <v>39.7142</v>
+        <v>67.6884</v>
       </c>
       <c r="X8" s="33" t="n">
         <f aca="false">W8-(E8*P1_IVAN+F8*P2_IVAN+G8*P3_IVAN)-(H8+I8+J8)*(COSTE_DEV-IVA_DEV)-AM8-AO8</f>
-        <v>-24.2897520661157</v>
+        <v>-2.4201652892562</v>
       </c>
       <c r="Y8" s="33" t="n">
         <f aca="false">AH8-AI8-AJ8-AK8-AL8-AM8-AO8</f>
-        <v>32.9863140495868</v>
+        <v>38.9722314049587</v>
       </c>
       <c r="AA8" s="58" t="n">
         <f aca="false">MAX(0,B8-E8-H8)</f>
@@ -5331,7 +5333,7 @@
       </c>
       <c r="AB8" s="58" t="n">
         <f aca="false">MAX(0,C8-F8-I8)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC8" s="58" t="n">
         <f aca="false">MAX(0,D8-G8-J8)</f>
@@ -5343,7 +5345,7 @@
       </c>
       <c r="AE8" s="59" t="n">
         <f aca="false">F8+AB8*TASA_USADA</f>
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="AF8" s="59" t="n">
         <f aca="false">G8+AC8*TASA_USADA</f>
@@ -5351,27 +5353,27 @@
       </c>
       <c r="AG8" s="59" t="n">
         <f aca="false">H8+I8+J8+(AA8+AB8+AC8)*(1-TASA_USADA)</f>
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="AH8" s="60" t="n">
         <f aca="false">AD8*P1_PVP+AE8*P2_PVP+AF8*P3_PVP</f>
-        <v>187.94</v>
+        <v>195.938</v>
       </c>
       <c r="AI8" s="60" t="n">
         <f aca="false">AD8*P1_CPROD+AE8*P2_CPROD+AF8*P3_CPROD</f>
-        <v>16.37372</v>
+        <v>17.33688</v>
       </c>
       <c r="AJ8" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L8),L8,E8*P1_LOG+F8*P2_LOG+G8*P3_LOG)+IF(ISNUMBER(M8),M8,AA8*P1_LOG+AB8*P2_LOG+AC8*P3_LOG)*TASA_USADA</f>
-        <v>46.314</v>
+        <v>47.754</v>
       </c>
       <c r="AK8" s="60" t="n">
         <f aca="false">AG8*COSTE_DEV</f>
-        <v>8.06</v>
+        <v>6.448</v>
       </c>
       <c r="AL8" s="60" t="n">
         <f aca="false">AD8*P1_IVAN+AE8*P2_IVAN+AF8*P3_IVAN-AG8*IVA_DEV</f>
-        <v>29.7759659504132</v>
+        <v>30.9968885950413</v>
       </c>
       <c r="AM8" s="60" t="n">
         <f aca="false">N8*(1+RECARGO_ADS)</f>
@@ -5399,24 +5401,28 @@
       <c r="D9" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="54"/>
+      <c r="E9" s="54" t="n">
+        <v>3</v>
+      </c>
       <c r="F9" s="54" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="54"/>
       <c r="H9" s="54"/>
       <c r="I9" s="54" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J9" s="54"/>
       <c r="K9" s="54" t="n">
         <v>3</v>
       </c>
       <c r="L9" s="55" t="n">
-        <v>7.2</v>
+        <v>42.15</v>
       </c>
       <c r="M9" s="55" t="n">
-        <v>103.7</v>
+        <v>54.7</v>
       </c>
       <c r="N9" s="55" t="n">
         <v>50.46</v>
@@ -5430,7 +5436,7 @@
       </c>
       <c r="Q9" s="31" t="n">
         <f aca="false">AA9+AB9+AC9</f>
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="R9" s="32" t="n">
         <f aca="false">B9*P1_PVP+C9*P2_PVP+D9*P3_PVP</f>
@@ -5450,67 +5456,67 @@
       </c>
       <c r="V9" s="34" t="n">
         <f aca="false">IF(E9+F9+G9+H9+I9+J9&gt;0,(E9+F9+G9)/(E9+F9+G9+H9+I9+J9),"")</f>
-        <v>0.5</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="W9" s="33" t="n">
         <f aca="false">E9*(P1_PVP-P1_CPROD)+F9*(P2_PVP-P2_CPROD)+G9*(P3_PVP-P3_CPROD)-IF(ISNUMBER(L9),L9,E9*P1_LOG+F9*P2_LOG+G9*P3_LOG)</f>
-        <v>27.9742</v>
+        <v>153.711</v>
       </c>
       <c r="X9" s="33" t="n">
         <f aca="false">W9-(E9*P1_IVAN+F9*P2_IVAN+G9*P3_IVAN)-(H9+I9+J9)*(COSTE_DEV-IVA_DEV)-AM9-AO9</f>
-        <v>-51.8504132231405</v>
+        <v>29.8785950413223</v>
       </c>
       <c r="Y9" s="33" t="n">
         <f aca="false">AH9-AI9-AJ9-AK9-AL9-AM9-AO9</f>
-        <v>128.044396694215</v>
+        <v>107.506859504132</v>
       </c>
       <c r="AA9" s="58" t="n">
         <f aca="false">MAX(0,B9-E9-H9)</f>
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="AB9" s="58" t="n">
         <f aca="false">MAX(0,C9-F9-I9)</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AC9" s="58" t="n">
         <f aca="false">MAX(0,D9-G9-J9)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD9" s="59" t="n">
         <f aca="false">E9+AA9*TASA_USADA</f>
-        <v>7.2</v>
+        <v>7.8</v>
       </c>
       <c r="AE9" s="59" t="n">
         <f aca="false">F9+AB9*TASA_USADA</f>
-        <v>4.2</v>
+        <v>2.8</v>
       </c>
       <c r="AF9" s="59" t="n">
         <f aca="false">G9+AC9*TASA_USADA</f>
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="AG9" s="59" t="n">
         <f aca="false">H9+I9+J9+(AA9+AB9+AC9)*(1-TASA_USADA)</f>
-        <v>3.8</v>
+        <v>4.4</v>
       </c>
       <c r="AH9" s="60" t="n">
         <f aca="false">AD9*P1_PVP+AE9*P2_PVP+AF9*P3_PVP</f>
-        <v>423.878</v>
+        <v>395.884</v>
       </c>
       <c r="AI9" s="60" t="n">
         <f aca="false">AD9*P1_CPROD+AE9*P2_CPROD+AF9*P3_CPROD</f>
-        <v>43.3422</v>
+        <v>39.48956</v>
       </c>
       <c r="AJ9" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L9),L9,E9*P1_LOG+F9*P2_LOG+G9*P3_LOG)+IF(ISNUMBER(M9),M9,AA9*P1_LOG+AB9*P2_LOG+AC9*P3_LOG)*TASA_USADA</f>
-        <v>90.16</v>
+        <v>85.91</v>
       </c>
       <c r="AK9" s="60" t="n">
         <f aca="false">AG9*COSTE_DEV</f>
-        <v>30.628</v>
+        <v>35.464</v>
       </c>
       <c r="AL9" s="60" t="n">
         <f aca="false">AD9*P1_IVAN+AE9*P2_IVAN+AF9*P3_IVAN-AG9*IVA_DEV</f>
-        <v>66.0434033057851</v>
+        <v>61.8535804958678</v>
       </c>
       <c r="AM9" s="60" t="n">
         <f aca="false">N9*(1+RECARGO_ADS)</f>
@@ -5518,7 +5524,7 @@
       </c>
       <c r="AN9" s="58" t="n">
         <f aca="false">IF(ISNUMBER(L9),E9+F9+G9+AA9+AB9+AC9,0)</f>
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="AO9" s="60" t="n">
         <f aca="false">P9*COMISION</f>
@@ -5533,23 +5539,27 @@
         <v>2</v>
       </c>
       <c r="C10" s="54" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="54"/>
+      <c r="E10" s="54" t="n">
+        <v>1</v>
+      </c>
       <c r="F10" s="54"/>
       <c r="G10" s="54"/>
       <c r="H10" s="54"/>
       <c r="I10" s="54"/>
       <c r="J10" s="54"/>
-      <c r="K10" s="54"/>
+      <c r="K10" s="54" t="n">
+        <v>1</v>
+      </c>
       <c r="L10" s="55" t="n">
-        <v>0</v>
+        <v>7.2</v>
       </c>
       <c r="M10" s="55" t="n">
-        <v>45.43</v>
+        <v>30.17</v>
       </c>
       <c r="N10" s="55" t="n">
         <v>41.21</v>
@@ -5557,51 +5567,51 @@
       <c r="O10" s="56"/>
       <c r="P10" s="31" t="n">
         <f aca="false">B10+C10+D10</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q10" s="31" t="n">
         <f aca="false">AA10+AB10+AC10</f>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="R10" s="32" t="n">
         <f aca="false">B10*P1_PVP+C10*P2_PVP+D10*P3_PVP</f>
-        <v>219.94</v>
+        <v>179.95</v>
       </c>
       <c r="S10" s="32" t="n">
         <f aca="false">IF(P10&gt;0,R10/P10,"")</f>
-        <v>36.6566666666667</v>
+        <v>35.99</v>
       </c>
       <c r="T10" s="32" t="n">
         <f aca="false">IF(P10&gt;0,N10/P10,"")</f>
-        <v>6.86833333333333</v>
+        <v>8.242</v>
       </c>
       <c r="U10" s="57" t="n">
         <f aca="false">IF(N10&gt;0,R10/N10,"")</f>
-        <v>5.33705411307935</v>
-      </c>
-      <c r="V10" s="34" t="str">
+        <v>4.36665857801505</v>
+      </c>
+      <c r="V10" s="34" t="n">
         <f aca="false">IF(E10+F10+G10+H10+I10+J10&gt;0,(E10+F10+G10)/(E10+F10+G10+H10+I10+J10),"")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="W10" s="33" t="n">
         <f aca="false">E10*(P1_PVP-P1_CPROD)+F10*(P2_PVP-P2_CPROD)+G10*(P3_PVP-P3_CPROD)-IF(ISNUMBER(L10),L10,E10*P1_LOG+F10*P2_LOG+G10*P3_LOG)</f>
-        <v>0</v>
+        <v>20.3821</v>
       </c>
       <c r="X10" s="33" t="n">
         <f aca="false">W10-(E10*P1_IVAN+F10*P2_IVAN+G10*P3_IVAN)-(H10+I10+J10)*(COSTE_DEV-IVA_DEV)-AM10-AO10</f>
-        <v>-46.91</v>
+        <v>-30.3648760330579</v>
       </c>
       <c r="Y10" s="33" t="n">
         <f aca="false">AH10-AI10-AJ10-AK10-AL10-AM10-AO10</f>
-        <v>36.5688760330579</v>
+        <v>27.0542314049587</v>
       </c>
       <c r="AA10" s="58" t="n">
         <f aca="false">MAX(0,B10-E10-H10)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB10" s="58" t="n">
         <f aca="false">MAX(0,C10-F10-I10)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AC10" s="58" t="n">
         <f aca="false">MAX(0,D10-G10-J10)</f>
@@ -5609,11 +5619,11 @@
       </c>
       <c r="AD10" s="59" t="n">
         <f aca="false">E10+AA10*TASA_USADA</f>
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="AE10" s="59" t="n">
         <f aca="false">F10+AB10*TASA_USADA</f>
-        <v>3.2</v>
+        <v>2.4</v>
       </c>
       <c r="AF10" s="59" t="n">
         <f aca="false">G10+AC10*TASA_USADA</f>
@@ -5621,27 +5631,27 @@
       </c>
       <c r="AG10" s="59" t="n">
         <f aca="false">H10+I10+J10+(AA10+AB10+AC10)*(1-TASA_USADA)</f>
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="AH10" s="60" t="n">
         <f aca="false">AD10*P1_PVP+AE10*P2_PVP+AF10*P3_PVP</f>
-        <v>175.952</v>
+        <v>149.958</v>
       </c>
       <c r="AI10" s="60" t="n">
         <f aca="false">AD10*P1_CPROD+AE10*P2_CPROD+AF10*P3_CPROD</f>
-        <v>19.2632</v>
+        <v>15.89214</v>
       </c>
       <c r="AJ10" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L10),L10,E10*P1_LOG+F10*P2_LOG+G10*P3_LOG)+IF(ISNUMBER(M10),M10,AA10*P1_LOG+AB10*P2_LOG+AC10*P3_LOG)*TASA_USADA</f>
-        <v>36.344</v>
+        <v>31.336</v>
       </c>
       <c r="AK10" s="60" t="n">
         <f aca="false">AG10*COSTE_DEV</f>
-        <v>9.672</v>
+        <v>6.448</v>
       </c>
       <c r="AL10" s="60" t="n">
         <f aca="false">AD10*P1_IVAN+AE10*P2_IVAN+AF10*P3_IVAN-AG10*IVA_DEV</f>
-        <v>27.1939239669421</v>
+        <v>23.2676285950413</v>
       </c>
       <c r="AM10" s="60" t="n">
         <f aca="false">N10*(1+RECARGO_ADS)</f>
@@ -5649,11 +5659,11 @@
       </c>
       <c r="AN10" s="58" t="n">
         <f aca="false">IF(ISNUMBER(L10),E10+F10+G10+AA10+AB10+AC10,0)</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AO10" s="60" t="n">
         <f aca="false">P10*COMISION</f>
-        <v>5.7</v>
+        <v>4.75</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5664,25 +5674,27 @@
         <v>6</v>
       </c>
       <c r="C11" s="54" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="54"/>
+      <c r="E11" s="54" t="n">
+        <v>1</v>
+      </c>
       <c r="F11" s="54"/>
       <c r="G11" s="54"/>
       <c r="H11" s="54"/>
       <c r="I11" s="54"/>
       <c r="J11" s="54"/>
       <c r="K11" s="54" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L11" s="55" t="n">
-        <v>0</v>
+        <v>6.85</v>
       </c>
       <c r="M11" s="55" t="n">
-        <v>74.93</v>
+        <v>60.02</v>
       </c>
       <c r="N11" s="55" t="n">
         <v>64.81</v>
@@ -5690,51 +5702,51 @@
       <c r="O11" s="56"/>
       <c r="P11" s="31" t="n">
         <f aca="false">B11+C11+D11</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Q11" s="31" t="n">
         <f aca="false">AA11+AB11+AC11</f>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="R11" s="32" t="n">
         <f aca="false">B11*P1_PVP+C11*P2_PVP+D11*P3_PVP</f>
-        <v>349.9</v>
+        <v>309.91</v>
       </c>
       <c r="S11" s="32" t="n">
         <f aca="false">IF(P11&gt;0,R11/P11,"")</f>
-        <v>34.99</v>
+        <v>34.4344444444444</v>
       </c>
       <c r="T11" s="32" t="n">
         <f aca="false">IF(P11&gt;0,N11/P11,"")</f>
-        <v>6.481</v>
+        <v>7.20111111111111</v>
       </c>
       <c r="U11" s="57" t="n">
         <f aca="false">IF(N11&gt;0,R11/N11,"")</f>
-        <v>5.39885820089492</v>
-      </c>
-      <c r="V11" s="34" t="str">
+        <v>4.7818237926246</v>
+      </c>
+      <c r="V11" s="34" t="n">
         <f aca="false">IF(E11+F11+G11+H11+I11+J11&gt;0,(E11+F11+G11)/(E11+F11+G11+H11+I11+J11),"")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="W11" s="33" t="n">
         <f aca="false">E11*(P1_PVP-P1_CPROD)+F11*(P2_PVP-P2_CPROD)+G11*(P3_PVP-P3_CPROD)-IF(ISNUMBER(L11),L11,E11*P1_LOG+F11*P2_LOG+G11*P3_LOG)</f>
-        <v>0</v>
+        <v>20.7321</v>
       </c>
       <c r="X11" s="33" t="n">
         <f aca="false">W11-(E11*P1_IVAN+F11*P2_IVAN+G11*P3_IVAN)-(H11+I11+J11)*(COSTE_DEV-IVA_DEV)-AM11-AO11</f>
-        <v>-74.31</v>
+        <v>-57.4148760330579</v>
       </c>
       <c r="Y11" s="33" t="n">
         <f aca="false">AH11-AI11-AJ11-AK11-AL11-AM11-AO11</f>
-        <v>57.0848429752066</v>
+        <v>47.6401983471074</v>
       </c>
       <c r="AA11" s="58" t="n">
         <f aca="false">MAX(0,B11-E11-H11)</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AB11" s="58" t="n">
         <f aca="false">MAX(0,C11-F11-I11)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AC11" s="58" t="n">
         <f aca="false">MAX(0,D11-G11-J11)</f>
@@ -5742,11 +5754,11 @@
       </c>
       <c r="AD11" s="59" t="n">
         <f aca="false">E11+AA11*TASA_USADA</f>
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="AE11" s="59" t="n">
         <f aca="false">F11+AB11*TASA_USADA</f>
-        <v>2.4</v>
+        <v>1.6</v>
       </c>
       <c r="AF11" s="59" t="n">
         <f aca="false">G11+AC11*TASA_USADA</f>
@@ -5754,27 +5766,27 @@
       </c>
       <c r="AG11" s="59" t="n">
         <f aca="false">H11+I11+J11+(AA11+AB11+AC11)*(1-TASA_USADA)</f>
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="AH11" s="60" t="n">
         <f aca="false">AD11*P1_PVP+AE11*P2_PVP+AF11*P3_PVP</f>
-        <v>279.92</v>
+        <v>253.926</v>
       </c>
       <c r="AI11" s="60" t="n">
         <f aca="false">AD11*P1_CPROD+AE11*P2_CPROD+AF11*P3_CPROD</f>
-        <v>28.8948</v>
+        <v>25.52374</v>
       </c>
       <c r="AJ11" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L11),L11,E11*P1_LOG+F11*P2_LOG+G11*P3_LOG)+IF(ISNUMBER(M11),M11,AA11*P1_LOG+AB11*P2_LOG+AC11*P3_LOG)*TASA_USADA</f>
-        <v>59.944</v>
+        <v>54.866</v>
       </c>
       <c r="AK11" s="60" t="n">
         <f aca="false">AG11*COSTE_DEV</f>
-        <v>16.12</v>
+        <v>12.896</v>
       </c>
       <c r="AL11" s="60" t="n">
         <f aca="false">AD11*P1_IVAN+AE11*P2_IVAN+AF11*P3_IVAN-AG11*IVA_DEV</f>
-        <v>43.5663570247934</v>
+        <v>39.6400616528926</v>
       </c>
       <c r="AM11" s="60" t="n">
         <f aca="false">N11*(1+RECARGO_ADS)</f>
@@ -5782,11 +5794,11 @@
       </c>
       <c r="AN11" s="58" t="n">
         <f aca="false">IF(ISNUMBER(L11),E11+F11+G11+AA11+AB11+AC11,0)</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AO11" s="60" t="n">
         <f aca="false">P11*COMISION</f>
-        <v>9.5</v>
+        <v>8.55</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5808,9 +5820,7 @@
       <c r="H12" s="54"/>
       <c r="I12" s="54"/>
       <c r="J12" s="54"/>
-      <c r="K12" s="54" t="n">
-        <v>5</v>
-      </c>
+      <c r="K12" s="54"/>
       <c r="L12" s="55" t="n">
         <v>0</v>
       </c>
@@ -5818,7 +5828,7 @@
         <v>47.02</v>
       </c>
       <c r="N12" s="55" t="n">
-        <v>89.43</v>
+        <v>89.51</v>
       </c>
       <c r="O12" s="56"/>
       <c r="P12" s="31" t="n">
@@ -5839,11 +5849,11 @@
       </c>
       <c r="T12" s="32" t="n">
         <f aca="false">IF(P12&gt;0,N12/P12,"")</f>
-        <v>14.905</v>
+        <v>14.9183333333333</v>
       </c>
       <c r="U12" s="57" t="n">
         <f aca="false">IF(N12&gt;0,R12/N12,"")</f>
-        <v>2.12389578441239</v>
+        <v>2.12199754217406</v>
       </c>
       <c r="V12" s="34" t="str">
         <f aca="false">IF(E12+F12+G12+H12+I12+J12&gt;0,(E12+F12+G12)/(E12+F12+G12+H12+I12+J12),"")</f>
@@ -5855,11 +5865,11 @@
       </c>
       <c r="X12" s="33" t="n">
         <f aca="false">W12-(E12*P1_IVAN+F12*P2_IVAN+G12*P3_IVAN)-(H12+I12+J12)*(COSTE_DEV-IVA_DEV)-AM12-AO12</f>
-        <v>-95.13</v>
+        <v>-95.21</v>
       </c>
       <c r="Y12" s="33" t="n">
         <f aca="false">AH12-AI12-AJ12-AK12-AL12-AM12-AO12</f>
-        <v>-27.9818347107438</v>
+        <v>-28.0618347107438</v>
       </c>
       <c r="AA12" s="58" t="n">
         <f aca="false">MAX(0,B12-E12-H12)</f>
@@ -5911,7 +5921,7 @@
       </c>
       <c r="AM12" s="60" t="n">
         <f aca="false">N12*(1+RECARGO_ADS)</f>
-        <v>89.43</v>
+        <v>89.51</v>
       </c>
       <c r="AN12" s="58" t="n">
         <f aca="false">IF(ISNUMBER(L12),E12+F12+G12+AA12+AB12+AC12,0)</f>
@@ -5927,13 +5937,13 @@
         <v>46307</v>
       </c>
       <c r="B13" s="54" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C13" s="54" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D13" s="54" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E13" s="54"/>
       <c r="F13" s="54"/>
@@ -5941,40 +5951,42 @@
       <c r="H13" s="54"/>
       <c r="I13" s="54"/>
       <c r="J13" s="54"/>
-      <c r="K13" s="54"/>
+      <c r="K13" s="54" t="n">
+        <v>2</v>
+      </c>
       <c r="L13" s="55" t="n">
         <v>0</v>
       </c>
       <c r="M13" s="55" t="n">
-        <v>46.29</v>
+        <v>103.76</v>
       </c>
       <c r="N13" s="55" t="n">
-        <v>34.45</v>
+        <v>78.33</v>
       </c>
       <c r="O13" s="56"/>
       <c r="P13" s="31" t="n">
         <f aca="false">B13+C13+D13</f>
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="Q13" s="31" t="n">
         <f aca="false">AA13+AB13+AC13</f>
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="R13" s="32" t="n">
         <f aca="false">B13*P1_PVP+C13*P2_PVP+D13*P3_PVP</f>
-        <v>189.94</v>
+        <v>489.86</v>
       </c>
       <c r="S13" s="32" t="n">
         <f aca="false">IF(P13&gt;0,R13/P13,"")</f>
-        <v>31.6566666666667</v>
+        <v>34.99</v>
       </c>
       <c r="T13" s="32" t="n">
         <f aca="false">IF(P13&gt;0,N13/P13,"")</f>
-        <v>5.74166666666667</v>
+        <v>5.595</v>
       </c>
       <c r="U13" s="57" t="n">
         <f aca="false">IF(N13&gt;0,R13/N13,"")</f>
-        <v>5.51349782293179</v>
+        <v>6.25379803395889</v>
       </c>
       <c r="V13" s="34" t="str">
         <f aca="false">IF(E13+F13+G13+H13+I13+J13&gt;0,(E13+F13+G13)/(E13+F13+G13+H13+I13+J13),"")</f>
@@ -5986,80 +5998,86 @@
       </c>
       <c r="X13" s="33" t="n">
         <f aca="false">W13-(E13*P1_IVAN+F13*P2_IVAN+G13*P3_IVAN)-(H13+I13+J13)*(COSTE_DEV-IVA_DEV)-AM13-AO13</f>
-        <v>-40.15</v>
+        <v>-91.63</v>
       </c>
       <c r="Y13" s="33" t="n">
         <f aca="false">AH13-AI13-AJ13-AK13-AL13-AM13-AO13</f>
-        <v>27.5821652892562</v>
+        <v>93.2363801652893</v>
       </c>
       <c r="AA13" s="58" t="n">
         <f aca="false">MAX(0,B13-E13-H13)</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="AB13" s="58" t="n">
         <f aca="false">MAX(0,C13-F13-I13)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AC13" s="58" t="n">
         <f aca="false">MAX(0,D13-G13-J13)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AD13" s="59" t="n">
         <f aca="false">E13+AA13*TASA_USADA</f>
-        <v>4</v>
+        <v>7.2</v>
       </c>
       <c r="AE13" s="59" t="n">
         <f aca="false">F13+AB13*TASA_USADA</f>
-        <v>0.8</v>
+        <v>2.4</v>
       </c>
       <c r="AF13" s="59" t="n">
         <f aca="false">G13+AC13*TASA_USADA</f>
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="AG13" s="59" t="n">
         <f aca="false">H13+I13+J13+(AA13+AB13+AC13)*(1-TASA_USADA)</f>
-        <v>1.2</v>
+        <v>2.8</v>
       </c>
       <c r="AH13" s="60" t="n">
         <f aca="false">AD13*P1_PVP+AE13*P2_PVP+AF13*P3_PVP</f>
-        <v>151.952</v>
+        <v>391.888</v>
       </c>
       <c r="AI13" s="60" t="n">
         <f aca="false">AD13*P1_CPROD+AE13*P2_CPROD+AF13*P3_CPROD</f>
-        <v>13.48424</v>
+        <v>40.45272</v>
       </c>
       <c r="AJ13" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L13),L13,E13*P1_LOG+F13*P2_LOG+G13*P3_LOG)+IF(ISNUMBER(M13),M13,AA13*P1_LOG+AB13*P2_LOG+AC13*P3_LOG)*TASA_USADA</f>
-        <v>37.032</v>
+        <v>83.008</v>
       </c>
       <c r="AK13" s="60" t="n">
         <f aca="false">AG13*COSTE_DEV</f>
-        <v>9.672</v>
+        <v>22.568</v>
       </c>
       <c r="AL13" s="60" t="n">
         <f aca="false">AD13*P1_IVAN+AE13*P2_IVAN+AF13*P3_IVAN-AG13*IVA_DEV</f>
-        <v>24.0315947107438</v>
+        <v>60.9928998347107</v>
       </c>
       <c r="AM13" s="60" t="n">
         <f aca="false">N13*(1+RECARGO_ADS)</f>
-        <v>34.45</v>
+        <v>78.33</v>
       </c>
       <c r="AN13" s="58" t="n">
         <f aca="false">IF(ISNUMBER(L13),E13+F13+G13+AA13+AB13+AC13,0)</f>
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="AO13" s="60" t="n">
         <f aca="false">P13*COMISION</f>
-        <v>5.7</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="53" t="n">
         <v>46308</v>
       </c>
-      <c r="B14" s="54"/>
-      <c r="C14" s="54"/>
-      <c r="D14" s="54"/>
+      <c r="B14" s="54" t="n">
+        <v>6</v>
+      </c>
+      <c r="C14" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="54" t="n">
+        <v>1</v>
+      </c>
       <c r="E14" s="54"/>
       <c r="F14" s="54"/>
       <c r="G14" s="54"/>
@@ -6067,33 +6085,39 @@
       <c r="I14" s="54"/>
       <c r="J14" s="54"/>
       <c r="K14" s="54"/>
-      <c r="L14" s="55"/>
-      <c r="M14" s="55"/>
-      <c r="N14" s="55"/>
+      <c r="L14" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="55" t="n">
+        <v>60.53</v>
+      </c>
+      <c r="N14" s="55" t="n">
+        <v>68.04</v>
+      </c>
       <c r="O14" s="56"/>
       <c r="P14" s="31" t="n">
         <f aca="false">B14+C14+D14</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="Q14" s="31" t="n">
         <f aca="false">AA14+AB14+AC14</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="R14" s="32" t="n">
         <f aca="false">B14*P1_PVP+C14*P2_PVP+D14*P3_PVP</f>
-        <v>0</v>
-      </c>
-      <c r="S14" s="32" t="str">
+        <v>269.92</v>
+      </c>
+      <c r="S14" s="32" t="n">
         <f aca="false">IF(P14&gt;0,R14/P14,"")</f>
-        <v/>
-      </c>
-      <c r="T14" s="32" t="str">
+        <v>33.74</v>
+      </c>
+      <c r="T14" s="32" t="n">
         <f aca="false">IF(P14&gt;0,N14/P14,"")</f>
-        <v/>
-      </c>
-      <c r="U14" s="57" t="str">
+        <v>8.505</v>
+      </c>
+      <c r="U14" s="57" t="n">
         <f aca="false">IF(N14&gt;0,R14/N14,"")</f>
-        <v/>
+        <v>3.96707818930041</v>
       </c>
       <c r="V14" s="34" t="str">
         <f aca="false">IF(E14+F14+G14+H14+I14+J14&gt;0,(E14+F14+G14)/(E14+F14+G14+H14+I14+J14),"")</f>
@@ -6105,80 +6129,86 @@
       </c>
       <c r="X14" s="33" t="n">
         <f aca="false">W14-(E14*P1_IVAN+F14*P2_IVAN+G14*P3_IVAN)-(H14+I14+J14)*(COSTE_DEV-IVA_DEV)-AM14-AO14</f>
-        <v>0</v>
+        <v>-75.64</v>
       </c>
       <c r="Y14" s="33" t="n">
         <f aca="false">AH14-AI14-AJ14-AK14-AL14-AM14-AO14</f>
-        <v>0</v>
+        <v>23.9875041322314</v>
       </c>
       <c r="AA14" s="58" t="n">
         <f aca="false">MAX(0,B14-E14-H14)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB14" s="58" t="n">
         <f aca="false">MAX(0,C14-F14-I14)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC14" s="58" t="n">
         <f aca="false">MAX(0,D14-G14-J14)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD14" s="59" t="n">
         <f aca="false">E14+AA14*TASA_USADA</f>
-        <v>0</v>
+        <v>4.8</v>
       </c>
       <c r="AE14" s="59" t="n">
         <f aca="false">F14+AB14*TASA_USADA</f>
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="AF14" s="59" t="n">
         <f aca="false">G14+AC14*TASA_USADA</f>
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="AG14" s="59" t="n">
         <f aca="false">H14+I14+J14+(AA14+AB14+AC14)*(1-TASA_USADA)</f>
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="AH14" s="60" t="n">
         <f aca="false">AD14*P1_PVP+AE14*P2_PVP+AF14*P3_PVP</f>
-        <v>0</v>
+        <v>215.936</v>
       </c>
       <c r="AI14" s="60" t="n">
         <f aca="false">AD14*P1_CPROD+AE14*P2_CPROD+AF14*P3_CPROD</f>
-        <v>0</v>
+        <v>21.18952</v>
       </c>
       <c r="AJ14" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L14),L14,E14*P1_LOG+F14*P2_LOG+G14*P3_LOG)+IF(ISNUMBER(M14),M14,AA14*P1_LOG+AB14*P2_LOG+AC14*P3_LOG)*TASA_USADA</f>
-        <v>0</v>
+        <v>48.424</v>
       </c>
       <c r="AK14" s="60" t="n">
         <f aca="false">AG14*COSTE_DEV</f>
-        <v>0</v>
+        <v>12.896</v>
       </c>
       <c r="AL14" s="60" t="n">
         <f aca="false">AD14*P1_IVAN+AE14*P2_IVAN+AF14*P3_IVAN-AG14*IVA_DEV</f>
-        <v>0</v>
+        <v>33.7989758677686</v>
       </c>
       <c r="AM14" s="60" t="n">
         <f aca="false">N14*(1+RECARGO_ADS)</f>
-        <v>0</v>
+        <v>68.04</v>
       </c>
       <c r="AN14" s="58" t="n">
         <f aca="false">IF(ISNUMBER(L14),E14+F14+G14+AA14+AB14+AC14,0)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AO14" s="60" t="n">
         <f aca="false">P14*COMISION</f>
-        <v>0</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="53" t="n">
         <v>46309</v>
       </c>
-      <c r="B15" s="54"/>
-      <c r="C15" s="54"/>
-      <c r="D15" s="54"/>
+      <c r="B15" s="54" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="54" t="n">
+        <v>0</v>
+      </c>
       <c r="E15" s="54"/>
       <c r="F15" s="54"/>
       <c r="G15" s="54"/>
@@ -6186,33 +6216,39 @@
       <c r="I15" s="54"/>
       <c r="J15" s="54"/>
       <c r="K15" s="54"/>
-      <c r="L15" s="55"/>
-      <c r="M15" s="55"/>
-      <c r="N15" s="55"/>
+      <c r="L15" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="55" t="n">
+        <v>32.24</v>
+      </c>
+      <c r="N15" s="55" t="n">
+        <v>40.38</v>
+      </c>
       <c r="O15" s="56"/>
       <c r="P15" s="31" t="n">
         <f aca="false">B15+C15+D15</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Q15" s="31" t="n">
         <f aca="false">AA15+AB15+AC15</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="R15" s="32" t="n">
         <f aca="false">B15*P1_PVP+C15*P2_PVP+D15*P3_PVP</f>
-        <v>0</v>
-      </c>
-      <c r="S15" s="32" t="str">
+        <v>129.96</v>
+      </c>
+      <c r="S15" s="32" t="n">
         <f aca="false">IF(P15&gt;0,R15/P15,"")</f>
-        <v/>
-      </c>
-      <c r="T15" s="32" t="str">
+        <v>32.49</v>
+      </c>
+      <c r="T15" s="32" t="n">
         <f aca="false">IF(P15&gt;0,N15/P15,"")</f>
-        <v/>
-      </c>
-      <c r="U15" s="57" t="str">
+        <v>10.095</v>
+      </c>
+      <c r="U15" s="57" t="n">
         <f aca="false">IF(N15&gt;0,R15/N15,"")</f>
-        <v/>
+        <v>3.2184249628529</v>
       </c>
       <c r="V15" s="34" t="str">
         <f aca="false">IF(E15+F15+G15+H15+I15+J15&gt;0,(E15+F15+G15)/(E15+F15+G15+H15+I15+J15),"")</f>
@@ -6224,19 +6260,19 @@
       </c>
       <c r="X15" s="33" t="n">
         <f aca="false">W15-(E15*P1_IVAN+F15*P2_IVAN+G15*P3_IVAN)-(H15+I15+J15)*(COSTE_DEV-IVA_DEV)-AM15-AO15</f>
-        <v>0</v>
+        <v>-44.18</v>
       </c>
       <c r="Y15" s="33" t="n">
         <f aca="false">AH15-AI15-AJ15-AK15-AL15-AM15-AO15</f>
-        <v>0</v>
+        <v>1.54396694214877</v>
       </c>
       <c r="AA15" s="58" t="n">
         <f aca="false">MAX(0,B15-E15-H15)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AB15" s="58" t="n">
         <f aca="false">MAX(0,C15-F15-I15)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC15" s="58" t="n">
         <f aca="false">MAX(0,D15-G15-J15)</f>
@@ -6244,11 +6280,11 @@
       </c>
       <c r="AD15" s="59" t="n">
         <f aca="false">E15+AA15*TASA_USADA</f>
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="AE15" s="59" t="n">
         <f aca="false">F15+AB15*TASA_USADA</f>
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="AF15" s="59" t="n">
         <f aca="false">G15+AC15*TASA_USADA</f>
@@ -6256,39 +6292,39 @@
       </c>
       <c r="AG15" s="59" t="n">
         <f aca="false">H15+I15+J15+(AA15+AB15+AC15)*(1-TASA_USADA)</f>
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="AH15" s="60" t="n">
         <f aca="false">AD15*P1_PVP+AE15*P2_PVP+AF15*P3_PVP</f>
-        <v>0</v>
+        <v>103.968</v>
       </c>
       <c r="AI15" s="60" t="n">
         <f aca="false">AD15*P1_CPROD+AE15*P2_CPROD+AF15*P3_CPROD</f>
-        <v>0</v>
+        <v>9.6316</v>
       </c>
       <c r="AJ15" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L15),L15,E15*P1_LOG+F15*P2_LOG+G15*P3_LOG)+IF(ISNUMBER(M15),M15,AA15*P1_LOG+AB15*P2_LOG+AC15*P3_LOG)*TASA_USADA</f>
-        <v>0</v>
+        <v>25.792</v>
       </c>
       <c r="AK15" s="60" t="n">
         <f aca="false">AG15*COSTE_DEV</f>
-        <v>0</v>
+        <v>6.448</v>
       </c>
       <c r="AL15" s="60" t="n">
         <f aca="false">AD15*P1_IVAN+AE15*P2_IVAN+AF15*P3_IVAN-AG15*IVA_DEV</f>
-        <v>0</v>
+        <v>16.3724330578512</v>
       </c>
       <c r="AM15" s="60" t="n">
         <f aca="false">N15*(1+RECARGO_ADS)</f>
-        <v>0</v>
+        <v>40.38</v>
       </c>
       <c r="AN15" s="58" t="n">
         <f aca="false">IF(ISNUMBER(L15),E15+F15+G15+AA15+AB15+AC15,0)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AO15" s="60" t="n">
         <f aca="false">P15*COMISION</f>
-        <v>0</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51210,7 +51246,7 @@
       </c>
       <c r="C37" s="31" t="n">
         <f aca="false">(SUM(Diario!$E$6:$E$370)+SUM(Diario!$F$6:$F$370)+SUM(Diario!$G$6:$G$370))+(SUM(Diario!$H$6:$H$370)+SUM(Diario!$I$6:$I$370)+SUM(Diario!$J$6:$J$370))</f>
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="F37" s="67" t="s">
         <v>183</v>
@@ -51222,7 +51258,7 @@
       </c>
       <c r="C38" s="34" t="n">
         <f aca="false">IF(C37&gt;0,(SUM(Diario!$E$6:$E$370)+SUM(Diario!$F$6:$F$370)+SUM(Diario!$G$6:$G$370))/C37,"")</f>
-        <v>0.846153846153846</v>
+        <v>0.826086956521739</v>
       </c>
       <c r="F38" s="67" t="s">
         <v>185</v>
@@ -51246,11 +51282,11 @@
       </c>
       <c r="C40" s="34" t="n">
         <f aca="false">IF(SUM(Diario!$P$6:$P$370)&gt;0,SUM(Diario!$C$6:$C$370)/SUM(Diario!$P$6:$P$370),"")</f>
-        <v>0.308823529411765</v>
+        <v>0.267441860465116</v>
       </c>
       <c r="D40" s="34" t="n">
         <f aca="false">IF(SUM(Diario!$P$6:$P$370)&gt;0,SUM(Diario!$D$6:$D$370)/SUM(Diario!$P$6:$P$370),"")</f>
-        <v>0.0294117647058824</v>
+        <v>0.0581395348837209</v>
       </c>
       <c r="F40" s="67" t="s">
         <v>189</v>
@@ -51262,11 +51298,11 @@
       </c>
       <c r="C41" s="34" t="n">
         <f aca="false">IF(C40="",C26,C40)</f>
-        <v>0.308823529411765</v>
+        <v>0.267441860465116</v>
       </c>
       <c r="D41" s="34" t="n">
         <f aca="false">IF(D40="",D26,D40)</f>
-        <v>0.0294117647058824</v>
+        <v>0.0581395348837209</v>
       </c>
       <c r="F41" s="67"/>
     </row>
@@ -51276,7 +51312,7 @@
       </c>
       <c r="C42" s="32" t="n">
         <f aca="false">IF(SUM(Diario!$AN$6:$AN$370)&gt;0,(SUM(Diario!$L$6:$L$370)+SUM(Diario!$M$6:$M$370))/SUM(Diario!$AN$6:$AN$370),"")</f>
-        <v>7.60727272727273</v>
+        <v>7.58719512195122</v>
       </c>
       <c r="F42" s="67" t="s">
         <v>192</v>
@@ -51288,7 +51324,7 @@
       </c>
       <c r="C43" s="32" t="n">
         <f aca="false">(1-C41-D41)*C5+C41*D5+D41*E5</f>
-        <v>33.6664705882353</v>
+        <v>33.8272093023256</v>
       </c>
       <c r="F43" s="67"/>
     </row>
@@ -51298,7 +51334,7 @@
       </c>
       <c r="C44" s="32" t="n">
         <f aca="false">(1-C41-D41)*(C5-C9-IF(C42="",C8,C42)-C14)+C41*(D5-D9-IF(C42="",D8,C42)-D14)+D41*(E5-E9-IF(C42="",E8,C42)-E14)</f>
-        <v>17.4946390374332</v>
+        <v>17.615571551122</v>
       </c>
       <c r="F44" s="67" t="s">
         <v>195</v>
@@ -51310,7 +51346,7 @@
       </c>
       <c r="C45" s="32" t="n">
         <f aca="false">C39*C44-(1-C39)*C36-COMISION</f>
-        <v>11.4337112299465</v>
+        <v>11.5304572408976</v>
       </c>
       <c r="F45" s="67" t="s">
         <v>197</v>
@@ -51322,7 +51358,7 @@
       </c>
       <c r="C46" s="33" t="n">
         <f aca="false">C45/(1+RECARGO_ADS)</f>
-        <v>11.4337112299465</v>
+        <v>11.5304572408976</v>
       </c>
       <c r="F46" s="67" t="s">
         <v>199</v>
@@ -51334,7 +51370,7 @@
       </c>
       <c r="C47" s="72" t="n">
         <f aca="false">IF(C46&gt;0,C43/C46,"")</f>
-        <v>2.94449194239382</v>
+        <v>2.93372661600471</v>
       </c>
       <c r="F47" s="67" t="s">
         <v>201</v>

</xml_diff>

<commit_message>
Panel: aviso de pedidos de Shopify que no llegan a Dropi; contabilidad al 15/10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFjE4yx23BY3D6kaMQowKe
</commit_message>
<xml_diff>
--- a/contabilidad/CeraLux_Contabilidad.xlsx
+++ b/contabilidad/CeraLux_Contabilidad.xlsx
@@ -1779,46 +1779,46 @@
               <c:strCache>
                 <c:ptCount val="14"/>
                 <c:pt idx="0">
-                  <c:v>Thu 01/10</c:v>
+                  <c:v>Fri 02/10</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Fri 02/10</c:v>
+                  <c:v>Sat 03/10</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Sat 03/10</c:v>
+                  <c:v>Sun 04/10</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Sun 04/10</c:v>
+                  <c:v>Mon 05/10</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Mon 05/10</c:v>
+                  <c:v>Tue 06/10</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Tue 06/10</c:v>
+                  <c:v>Wed 07/10</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Wed 07/10</c:v>
+                  <c:v>Thu 08/10</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>Thu 08/10</c:v>
+                  <c:v>Fri 09/10</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Fri 09/10</c:v>
+                  <c:v>Sat 10/10</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Sat 10/10</c:v>
+                  <c:v>Sun 11/10</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Sun 11/10</c:v>
+                  <c:v>Mon 12/10</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>Mon 12/10</c:v>
+                  <c:v>Tue 13/10</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>Tue 13/10</c:v>
+                  <c:v>Wed 14/10</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>Wed 14/10</c:v>
+                  <c:v>Thu 15/10</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1839,37 +1839,37 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>69.356477551932</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>62.6280826446281</c:v>
+                  <c:v>14.6518851909761</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>8.63823140495868</c:v>
+                  <c:v>44.9424257315166</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>38.9722314049587</c:v>
+                  <c:v>121.456059861514</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>107.506859504132</c:v>
+                  <c:v>46.2723698905517</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>27.0542314049587</c:v>
+                  <c:v>69.3591467500559</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>47.6401983471074</c:v>
+                  <c:v>-18.6963077953987</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>-28.0618347107438</c:v>
+                  <c:v>103.415090462363</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>93.2363801652893</c:v>
+                  <c:v>51.1591824882734</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>23.9875041322314</c:v>
+                  <c:v>23.4605896805897</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1.54396694214877</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1877,8 +1877,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="75265296"/>
-        <c:axId val="12966900"/>
+        <c:axId val="21505844"/>
+        <c:axId val="21662608"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -1942,46 +1942,46 @@
               <c:strCache>
                 <c:ptCount val="14"/>
                 <c:pt idx="0">
-                  <c:v>Thu 01/10</c:v>
+                  <c:v>Fri 02/10</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Fri 02/10</c:v>
+                  <c:v>Sat 03/10</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Sat 03/10</c:v>
+                  <c:v>Sun 04/10</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Sun 04/10</c:v>
+                  <c:v>Mon 05/10</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Mon 05/10</c:v>
+                  <c:v>Tue 06/10</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Tue 06/10</c:v>
+                  <c:v>Wed 07/10</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Wed 07/10</c:v>
+                  <c:v>Thu 08/10</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>Thu 08/10</c:v>
+                  <c:v>Fri 09/10</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Fri 09/10</c:v>
+                  <c:v>Sat 10/10</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Sat 10/10</c:v>
+                  <c:v>Sun 11/10</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Sun 11/10</c:v>
+                  <c:v>Mon 12/10</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>Mon 12/10</c:v>
+                  <c:v>Tue 13/10</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>Tue 13/10</c:v>
+                  <c:v>Wed 14/10</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>Wed 14/10</c:v>
+                  <c:v>Thu 15/10</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2002,37 +2002,37 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>67.67</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>67.67</c:v>
+                  <c:v>70.18</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>70.18</c:v>
+                  <c:v>47.78</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>47.78</c:v>
+                  <c:v>50.46</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>50.46</c:v>
+                  <c:v>41.21</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>41.21</c:v>
+                  <c:v>64.81</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>64.81</c:v>
+                  <c:v>89.51</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>89.51</c:v>
+                  <c:v>78.33</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>78.33</c:v>
+                  <c:v>68.05</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>68.04</c:v>
+                  <c:v>73.18</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>40.38</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2047,11 +2047,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="75265296"/>
-        <c:axId val="12966900"/>
+        <c:axId val="21505844"/>
+        <c:axId val="21662608"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="75265296"/>
+        <c:axId val="21505844"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2083,7 +2083,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="12966900"/>
+        <c:crossAx val="21662608"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2091,7 +2091,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="12966900"/>
+        <c:axId val="21662608"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2133,7 +2133,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75265296"/>
+        <c:crossAx val="21505844"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2332,7 +2332,7 @@
                 <c:formatCode>#,##0" €";[RED]\-#,##0" €";\-</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>383.14585123967</c:v>
+                  <c:v>525.376919812374</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -2373,8 +2373,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="60977798"/>
-        <c:axId val="32316078"/>
+        <c:axId val="40202871"/>
+        <c:axId val="23891191"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2471,11 +2471,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="60977798"/>
-        <c:axId val="32316078"/>
+        <c:axId val="40202871"/>
+        <c:axId val="23891191"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="60977798"/>
+        <c:axId val="40202871"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2507,7 +2507,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="32316078"/>
+        <c:crossAx val="23891191"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2515,7 +2515,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="32316078"/>
+        <c:axId val="23891191"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2557,7 +2557,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60977798"/>
+        <c:crossAx val="40202871"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="F3" s="4" t="n">
         <f aca="true">TODAY()</f>
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="G3" s="4"/>
       <c r="H3" s="3" t="s">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="I3" s="5" t="n">
         <f aca="false">MAX(1,$F$3-$C$3+1)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J3" s="6" t="s">
         <v>5</v>
@@ -2903,7 +2903,7 @@
       <c r="K3" s="6"/>
       <c r="L3" s="7" t="n">
         <f aca="false">TASA_USADA</f>
-        <v>0.8</v>
+        <v>0.864864864864865</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2951,32 +2951,32 @@
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="10" t="n">
         <f aca="false">F25</f>
-        <v>383.145851239669</v>
+        <v>525.376919812374</v>
       </c>
       <c r="C7" s="10"/>
       <c r="D7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$W$6:$W$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>445.4167</v>
+        <v>757.8287</v>
       </c>
       <c r="E7" s="10"/>
       <c r="F7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$X$6:$X$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+F24</f>
-        <v>-388.38694214876</v>
+        <v>-192.099090909091</v>
       </c>
       <c r="G7" s="10"/>
       <c r="H7" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="I7" s="11"/>
       <c r="J7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$R$6:$R$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>2909.14</v>
+        <v>3049.1</v>
       </c>
       <c r="K7" s="10"/>
       <c r="L7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>618.37</v>
+        <v>651.18</v>
       </c>
       <c r="M7" s="10"/>
     </row>
@@ -3009,32 +3009,32 @@
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="10" t="n">
         <f aca="false">IF(H7&gt;0,L7/H7,"")</f>
-        <v>7.1903488372093</v>
+        <v>7.23533333333333</v>
       </c>
       <c r="C10" s="10"/>
       <c r="D10" s="10" t="n">
         <f aca="false">CPA_BE</f>
-        <v>11.5304572408976</v>
+        <v>13.227012565312</v>
       </c>
       <c r="E10" s="10"/>
       <c r="F10" s="12" t="n">
         <f aca="false">IF(L7&gt;0,J7/L7,"")</f>
-        <v>4.70452965053285</v>
+        <v>4.6824226788292</v>
       </c>
       <c r="G10" s="12"/>
       <c r="H10" s="12" t="n">
         <f aca="false">ROAS_BE</f>
-        <v>2.93372661600471</v>
+        <v>2.5613409469147</v>
       </c>
       <c r="I10" s="12"/>
       <c r="J10" s="10" t="n">
         <f aca="false">IF(H7&gt;0,J7/H7,"")</f>
-        <v>33.8272093023256</v>
+        <v>33.8788888888889</v>
       </c>
       <c r="K10" s="10"/>
       <c r="L10" s="13" t="n">
         <f aca="false">IF(H7&gt;0,(SUMIFS(Diario!$C$6:$C$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+SUMIFS(Diario!$D$6:$D$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3))/H7,"")</f>
-        <v>0.325581395348837</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="M10" s="13"/>
     </row>
@@ -3067,27 +3067,27 @@
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="C13" s="11"/>
       <c r="D13" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$Q$6:$Q$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="E13" s="11"/>
       <c r="F13" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$K$6:$K$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="G13" s="11"/>
       <c r="H13" s="11" t="n">
         <f aca="false">SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I13" s="11"/>
       <c r="J13" s="13" t="n">
         <f aca="false">IF(B13+H13&gt;0,B13/(B13+H13),"")</f>
-        <v>0.826086956521739</v>
+        <v>0.864864864864865</v>
       </c>
       <c r="K13" s="13"/>
       <c r="L13" s="14" t="str">
@@ -3124,7 +3124,7 @@
       </c>
       <c r="F16" s="17" t="n">
         <f aca="false">SUMIFS(Diario!$AH$6:$AH$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>2337.306</v>
+        <v>2614.08648648649</v>
       </c>
       <c r="H16" s="15" t="s">
         <v>29</v>
@@ -3146,11 +3146,11 @@
       <c r="D17" s="15"/>
       <c r="E17" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F17/$F$16,"")</f>
-        <v>-0.0978692990990482</v>
+        <v>-0.0974649663155544</v>
       </c>
       <c r="F17" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AI$6:$AI$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-228.7505</v>
+        <v>-254.781851351351</v>
       </c>
       <c r="H17" s="15" t="s">
         <v>31</v>
@@ -3160,7 +3160,7 @@
       <c r="K17" s="15"/>
       <c r="L17" s="20" t="n">
         <f aca="false">F25/I3</f>
-        <v>27.3675608028335</v>
+        <v>35.0251279874916</v>
       </c>
       <c r="M17" s="20"/>
     </row>
@@ -3172,11 +3172,11 @@
       <c r="D18" s="15"/>
       <c r="E18" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F18/$F$16,"")</f>
-        <v>-0.224872566963846</v>
+        <v>-0.225606382054813</v>
       </c>
       <c r="F18" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AJ$6:$AJ$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-525.596</v>
+        <v>-589.754594594595</v>
       </c>
       <c r="H18" s="15" t="s">
         <v>33</v>
@@ -3186,7 +3186,7 @@
       <c r="K18" s="15"/>
       <c r="L18" s="18" t="n">
         <f aca="false">L17*30</f>
-        <v>821.026824085006</v>
+        <v>1050.75383962475</v>
       </c>
       <c r="M18" s="18"/>
     </row>
@@ -3198,11 +3198,11 @@
       <c r="D19" s="15"/>
       <c r="E19" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F19/$F$16,"")</f>
-        <v>-0.0572436814007237</v>
+        <v>-0.0374995347452265</v>
       </c>
       <c r="F19" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AK$6:$AK$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-133.796</v>
+        <v>-98.027027027027</v>
       </c>
       <c r="H19" s="21" t="s">
         <v>35</v>
@@ -3212,7 +3212,7 @@
       <c r="K19" s="21"/>
       <c r="L19" s="22" t="n">
         <f aca="false">IF(L16&gt;0,L18/L16,"")</f>
-        <v>0.0821026824085006</v>
+        <v>0.105075383962475</v>
       </c>
       <c r="M19" s="22"/>
     </row>
@@ -3224,11 +3224,11 @@
       <c r="D20" s="15"/>
       <c r="E20" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F20/$F$16,"")</f>
-        <v>-0.0349547727169656</v>
+        <v>-0.0327074105780325</v>
       </c>
       <c r="F20" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AO$6:$AO$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-81.7</v>
+        <v>-85.5</v>
       </c>
       <c r="H20" s="15" t="s">
         <v>37</v>
@@ -3238,7 +3238,7 @@
       <c r="K20" s="15"/>
       <c r="L20" s="20" t="n">
         <f aca="false">BEN_PEDIDO</f>
-        <v>11.5304572408976</v>
+        <v>13.227012565312</v>
       </c>
       <c r="M20" s="20"/>
     </row>
@@ -3250,11 +3250,11 @@
       <c r="D21" s="15"/>
       <c r="E21" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F21/$F$16,"")</f>
-        <v>-0.156568138172892</v>
+        <v>-0.156638311631185</v>
       </c>
       <c r="F21" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AL$6:$AL$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-365.947648760331</v>
+        <v>-409.466093701139</v>
       </c>
       <c r="H21" s="15" t="s">
         <v>39</v>
@@ -3264,7 +3264,7 @@
       <c r="K21" s="15"/>
       <c r="L21" s="20" t="n">
         <f aca="false">B10</f>
-        <v>7.1903488372093</v>
+        <v>7.23533333333333</v>
       </c>
       <c r="M21" s="20"/>
     </row>
@@ -3276,11 +3276,11 @@
       <c r="D22" s="15"/>
       <c r="E22" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F22/$F$16,"")</f>
-        <v>-0.264565273010894</v>
+        <v>-0.249104229476061</v>
       </c>
       <c r="F22" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AM$6:$AM$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-618.37</v>
+        <v>-651.18</v>
       </c>
       <c r="H22" s="15" t="s">
         <v>41</v>
@@ -3290,7 +3290,7 @@
       <c r="K22" s="15"/>
       <c r="L22" s="20" t="n">
         <f aca="false">IF(ISNUMBER(L21),L20-L21*(1+RECARGO_ADS),"")</f>
-        <v>4.3401084036883</v>
+        <v>5.9916792319787</v>
       </c>
       <c r="M22" s="20"/>
     </row>
@@ -3302,11 +3302,11 @@
       <c r="D23" s="23"/>
       <c r="E23" s="24" t="n">
         <f aca="false">IF($F$16&gt;0,F23/$F$16,"")</f>
-        <v>0.16392626863563</v>
+        <v>0.200979165199128</v>
       </c>
       <c r="F23" s="25" t="n">
         <f aca="false">SUM(F16:F22)</f>
-        <v>383.145851239669</v>
+        <v>525.376919812374</v>
       </c>
       <c r="H23" s="21" t="s">
         <v>43</v>
@@ -3316,7 +3316,7 @@
       <c r="K23" s="21"/>
       <c r="L23" s="26" t="n">
         <f aca="false">IF(NOT(ISNUMBER(L22)),"",IF(L22&lt;=0,"Baja el CPA",ROUNDUP((L16-F24/I3*30)/30/L22,0)))</f>
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="M23" s="26"/>
     </row>
@@ -3342,7 +3342,7 @@
       <c r="K24" s="15"/>
       <c r="L24" s="18" t="n">
         <f aca="false">IF(ISNUMBER(L23),L23*L21,"")</f>
-        <v>553.656860465116</v>
+        <v>405.178666666667</v>
       </c>
       <c r="M24" s="18"/>
     </row>
@@ -3354,11 +3354,11 @@
       <c r="D25" s="23"/>
       <c r="E25" s="24" t="n">
         <f aca="false">IF($F$16&gt;0,F25/$F$16,"")</f>
-        <v>0.16392626863563</v>
+        <v>0.200979165199128</v>
       </c>
       <c r="F25" s="25" t="n">
         <f aca="false">F23+F24</f>
-        <v>383.145851239669</v>
+        <v>525.376919812374</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3369,7 +3369,7 @@
       <c r="D26" s="27"/>
       <c r="F26" s="28" t="n">
         <f aca="false">IF(F16&gt;0,F25/F16,"")</f>
-        <v>0.16392626863563</v>
+        <v>0.200979165199128</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3405,7 +3405,7 @@
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="30" t="n">
         <f aca="false">$F$3-13</f>
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="C29" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B29)</f>
@@ -3431,7 +3431,7 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="30" t="n">
         <f aca="false">$F$3-12</f>
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="C30" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B30)</f>
@@ -3457,7 +3457,7 @@
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="30" t="n">
         <f aca="false">$F$3-11</f>
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="C31" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B31)</f>
@@ -3483,153 +3483,153 @@
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="30" t="n">
         <f aca="false">$F$3-10</f>
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="C32" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B32)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D32" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B32)</f>
-        <v>0</v>
-      </c>
-      <c r="E32" s="32" t="str">
+        <v>67.67</v>
+      </c>
+      <c r="E32" s="32" t="n">
         <f aca="false">IF(C32&gt;0,D32/C32,"")</f>
-        <v/>
+        <v>7.51888888888889</v>
       </c>
       <c r="F32" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B32)</f>
-        <v>0</v>
-      </c>
-      <c r="G32" s="34" t="str">
+        <v>69.356477551932</v>
+      </c>
+      <c r="G32" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B32))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B32))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B32)),"")</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="30" t="n">
         <f aca="false">$F$3-9</f>
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="C33" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B33)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D33" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B33)</f>
-        <v>67.67</v>
+        <v>70.18</v>
       </c>
       <c r="E33" s="32" t="n">
         <f aca="false">IF(C33&gt;0,D33/C33,"")</f>
-        <v>7.51888888888889</v>
+        <v>8.7725</v>
       </c>
       <c r="F33" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B33)</f>
-        <v>62.6280826446281</v>
+        <v>14.6518851909761</v>
       </c>
       <c r="G33" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B33))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B33))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B33)),"")</f>
-        <v>1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="30" t="n">
         <f aca="false">$F$3-8</f>
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="C34" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B34)</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D34" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B34)</f>
-        <v>70.18</v>
+        <v>47.78</v>
       </c>
       <c r="E34" s="32" t="n">
         <f aca="false">IF(C34&gt;0,D34/C34,"")</f>
-        <v>8.7725</v>
+        <v>6.82571428571429</v>
       </c>
       <c r="F34" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B34)</f>
-        <v>8.63823140495868</v>
+        <v>44.9424257315166</v>
       </c>
       <c r="G34" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B34))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B34))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B34)),"")</f>
-        <v>0.75</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="30" t="n">
         <f aca="false">$F$3-7</f>
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="C35" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B35)</f>
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="D35" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B35)</f>
-        <v>47.78</v>
+        <v>50.46</v>
       </c>
       <c r="E35" s="32" t="n">
         <f aca="false">IF(C35&gt;0,D35/C35,"")</f>
-        <v>6.82571428571429</v>
+        <v>3.15375</v>
       </c>
       <c r="F35" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B35)</f>
-        <v>38.9722314049587</v>
+        <v>121.456059861514</v>
       </c>
       <c r="G35" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B35))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B35))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B35)),"")</f>
-        <v>1</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="30" t="n">
         <f aca="false">$F$3-6</f>
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="C36" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B36)</f>
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="D36" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B36)</f>
-        <v>50.46</v>
+        <v>41.21</v>
       </c>
       <c r="E36" s="32" t="n">
         <f aca="false">IF(C36&gt;0,D36/C36,"")</f>
-        <v>3.15375</v>
+        <v>8.242</v>
       </c>
       <c r="F36" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B36)</f>
-        <v>107.506859504132</v>
+        <v>46.2723698905517</v>
       </c>
       <c r="G36" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B36))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B36))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B36)),"")</f>
-        <v>0.666666666666667</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="30" t="n">
         <f aca="false">$F$3-5</f>
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="C37" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B37)</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D37" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B37)</f>
-        <v>41.21</v>
+        <v>64.81</v>
       </c>
       <c r="E37" s="32" t="n">
         <f aca="false">IF(C37&gt;0,D37/C37,"")</f>
-        <v>8.242</v>
+        <v>7.20111111111111</v>
       </c>
       <c r="F37" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B37)</f>
-        <v>27.0542314049587</v>
+        <v>69.3591467500559</v>
       </c>
       <c r="G37" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B37))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B37))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B37)),"")</f>
@@ -3639,127 +3639,127 @@
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="30" t="n">
         <f aca="false">$F$3-4</f>
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="C38" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B38)</f>
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D38" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B38)</f>
-        <v>64.81</v>
+        <v>89.51</v>
       </c>
       <c r="E38" s="32" t="n">
         <f aca="false">IF(C38&gt;0,D38/C38,"")</f>
-        <v>7.20111111111111</v>
+        <v>14.9183333333333</v>
       </c>
       <c r="F38" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B38)</f>
-        <v>47.6401983471074</v>
-      </c>
-      <c r="G38" s="34" t="n">
+        <v>-18.6963077953987</v>
+      </c>
+      <c r="G38" s="34" t="str">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B38))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B38))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B38)),"")</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="30" t="n">
         <f aca="false">$F$3-3</f>
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="C39" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B39)</f>
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="D39" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B39)</f>
-        <v>89.51</v>
+        <v>78.33</v>
       </c>
       <c r="E39" s="32" t="n">
         <f aca="false">IF(C39&gt;0,D39/C39,"")</f>
-        <v>14.9183333333333</v>
+        <v>5.595</v>
       </c>
       <c r="F39" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B39)</f>
-        <v>-28.0618347107438</v>
-      </c>
-      <c r="G39" s="34" t="str">
+        <v>103.415090462363</v>
+      </c>
+      <c r="G39" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B39))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B39))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B39)),"")</f>
-        <v/>
+        <v>0.833333333333333</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="30" t="n">
         <f aca="false">$F$3-2</f>
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="C40" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B40)</f>
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="D40" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B40)</f>
-        <v>78.33</v>
+        <v>68.05</v>
       </c>
       <c r="E40" s="32" t="n">
         <f aca="false">IF(C40&gt;0,D40/C40,"")</f>
-        <v>5.595</v>
+        <v>7.56111111111111</v>
       </c>
       <c r="F40" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B40)</f>
-        <v>93.2363801652893</v>
-      </c>
-      <c r="G40" s="34" t="str">
+        <v>51.1591824882734</v>
+      </c>
+      <c r="G40" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B40))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B40))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B40)),"")</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="30" t="n">
         <f aca="false">$F$3-1</f>
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C41" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B41)</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D41" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B41)</f>
-        <v>68.04</v>
+        <v>73.18</v>
       </c>
       <c r="E41" s="32" t="n">
         <f aca="false">IF(C41&gt;0,D41/C41,"")</f>
-        <v>8.505</v>
+        <v>10.4542857142857</v>
       </c>
       <c r="F41" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B41)</f>
-        <v>23.9875041322314</v>
-      </c>
-      <c r="G41" s="34" t="str">
+        <v>23.4605896805897</v>
+      </c>
+      <c r="G41" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B41))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B41))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B41)),"")</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="30" t="n">
         <f aca="false">$F$3-0</f>
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="C42" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,$B42)</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D42" s="32" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,$B42)</f>
-        <v>40.38</v>
-      </c>
-      <c r="E42" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" s="32" t="str">
         <f aca="false">IF(C42&gt;0,D42/C42,"")</f>
-        <v>10.095</v>
+        <v/>
       </c>
       <c r="F42" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B42)</f>
-        <v>1.54396694214877</v>
+        <v>0</v>
       </c>
       <c r="G42" s="34" t="str">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B42))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B42))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B42)),"")</f>
@@ -3830,35 +3830,35 @@
       </c>
       <c r="C47" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$P$6:$P$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="D47" s="37" t="n">
         <f aca="false">SUMIFS(Diario!$N$6:$N$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>618.37</v>
+        <v>651.18</v>
       </c>
       <c r="E47" s="32" t="n">
         <f aca="false">IF(C47&gt;0,D47/C47,"")</f>
-        <v>7.1903488372093</v>
+        <v>7.23533333333333</v>
       </c>
       <c r="F47" s="37" t="n">
         <f aca="false">SUMIFS(Diario!$R$6:$R$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>2909.14</v>
+        <v>3049.1</v>
       </c>
       <c r="G47" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="H47" s="31" t="n">
         <f aca="false">SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I47" s="34" t="n">
         <f aca="false">IF(G47+H47&gt;0,G47/(G47+H47),"")</f>
-        <v>0.826086956521739</v>
+        <v>0.864864864864865</v>
       </c>
       <c r="J47" s="37" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>383.14585123967</v>
+        <v>525.376919812374</v>
       </c>
       <c r="K47" s="37" t="n">
         <f aca="false">-SUMIFS(Gastos!$D$5:$D$304,Gastos!$A$5:$A$304,"&gt;="&amp;$B47,Gastos!$A$5:$A$304,"&lt;="&amp;EOMONTH($B47,0))</f>
@@ -3866,11 +3866,11 @@
       </c>
       <c r="L47" s="38" t="n">
         <f aca="false">J47+K47</f>
-        <v>383.14585123967</v>
+        <v>525.376919812374</v>
       </c>
       <c r="M47" s="34" t="n">
         <f aca="false">IF(OBJETIVO_MES&gt;0,L47/OBJETIVO_MES,"")</f>
-        <v>0.038314585123967</v>
+        <v>0.0525376919812374</v>
       </c>
       <c r="O47" s="39" t="n">
         <f aca="false">OBJETIVO_MES</f>
@@ -4477,35 +4477,35 @@
       </c>
       <c r="C59" s="41" t="n">
         <f aca="false">SUM(C47:C58)</f>
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="D59" s="42" t="n">
         <f aca="false">SUM(D47:D58)</f>
-        <v>618.37</v>
+        <v>651.18</v>
       </c>
       <c r="E59" s="43" t="n">
         <f aca="false">IF(C59&gt;0,D59/C59,"")</f>
-        <v>7.1903488372093</v>
+        <v>7.23533333333333</v>
       </c>
       <c r="F59" s="42" t="n">
         <f aca="false">SUM(F47:F58)</f>
-        <v>2909.14</v>
+        <v>3049.1</v>
       </c>
       <c r="G59" s="41" t="n">
         <f aca="false">SUM(G47:G58)</f>
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="H59" s="41" t="n">
         <f aca="false">SUM(H47:H58)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I59" s="44" t="n">
         <f aca="false">IF(G59+H59&gt;0,G59/(G59+H59),"")</f>
-        <v>0.826086956521739</v>
+        <v>0.864864864864865</v>
       </c>
       <c r="J59" s="42" t="n">
         <f aca="false">SUM(J47:J58)</f>
-        <v>383.14585123967</v>
+        <v>525.376919812374</v>
       </c>
       <c r="K59" s="42" t="n">
         <f aca="false">SUM(K47:K58)</f>
@@ -4513,7 +4513,7 @@
       </c>
       <c r="L59" s="42" t="n">
         <f aca="false">SUM(L47:L58)</f>
-        <v>383.14585123967</v>
+        <v>525.376919812374</v>
       </c>
       <c r="M59" s="45"/>
     </row>
@@ -4700,11 +4700,11 @@
       </c>
       <c r="B4" s="47" t="n">
         <f aca="false">SUM(B6:B370)</f>
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C4" s="47" t="n">
         <f aca="false">SUM(C6:C370)</f>
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D4" s="47" t="n">
         <f aca="false">SUM(D6:D370)</f>
@@ -4712,15 +4712,15 @@
       </c>
       <c r="E4" s="47" t="n">
         <f aca="false">SUM(E6:E370)</f>
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F4" s="47" t="n">
         <f aca="false">SUM(F6:F370)</f>
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G4" s="47" t="n">
         <f aca="false">SUM(G6:G370)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H4" s="47" t="n">
         <f aca="false">SUM(H6:H370)</f>
@@ -4732,123 +4732,123 @@
       </c>
       <c r="J4" s="47" t="n">
         <f aca="false">SUM(J6:J370)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" s="47" t="n">
         <f aca="false">SUM(K6:K370)</f>
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="L4" s="48" t="n">
         <f aca="false">SUM(L6:L370)</f>
-        <v>139.38</v>
+        <v>238.68</v>
       </c>
       <c r="M4" s="48" t="n">
         <f aca="false">SUM(M6:M370)</f>
-        <v>482.77</v>
+        <v>405.93</v>
       </c>
       <c r="N4" s="48" t="n">
         <f aca="false">SUM(N6:N370)</f>
-        <v>618.37</v>
+        <v>651.18</v>
       </c>
       <c r="P4" s="47" t="n">
         <f aca="false">SUM(P6:P370)</f>
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="Q4" s="47" t="n">
         <f aca="false">SUM(Q6:Q370)</f>
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="R4" s="48" t="n">
         <f aca="false">SUM(R6:R370)</f>
-        <v>2909.14</v>
+        <v>3049.1</v>
       </c>
       <c r="S4" s="48" t="n">
         <f aca="false">IF(P4&gt;0,R4/P4,"")</f>
-        <v>33.8272093023256</v>
+        <v>33.8788888888889</v>
       </c>
       <c r="T4" s="48" t="n">
         <f aca="false">IF(P4&gt;0,N4/P4,"")</f>
-        <v>7.1903488372093</v>
+        <v>7.23533333333333</v>
       </c>
       <c r="U4" s="49" t="n">
         <f aca="false">IF(N4&gt;0,R4/N4,"")</f>
-        <v>4.70452965053285</v>
+        <v>4.6824226788292</v>
       </c>
       <c r="V4" s="50" t="n">
         <f aca="false">IF(E4+F4+G4+H4+I4+J4&gt;0,(E4+F4+G4)/(E4+F4+G4+H4+I4+J4),"")</f>
-        <v>0.826086956521739</v>
+        <v>0.864864864864865</v>
       </c>
       <c r="W4" s="48" t="n">
         <f aca="false">SUM(W6:W370)</f>
-        <v>445.4167</v>
+        <v>757.8287</v>
       </c>
       <c r="X4" s="48" t="n">
         <f aca="false">SUM(X6:X370)</f>
-        <v>-388.38694214876</v>
+        <v>-192.099090909091</v>
       </c>
       <c r="Y4" s="48" t="n">
         <f aca="false">SUM(Y6:Y370)</f>
-        <v>383.14585123967</v>
+        <v>525.376919812374</v>
       </c>
       <c r="AA4" s="47" t="n">
         <f aca="false">SUM(AA6:AA370)</f>
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="AB4" s="47" t="n">
         <f aca="false">SUM(AB6:AB370)</f>
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="AC4" s="47" t="n">
         <f aca="false">SUM(AC6:AC370)</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AD4" s="51" t="n">
         <f aca="false">SUM(AD6:AD370)</f>
-        <v>48</v>
+        <v>53.5945945945946</v>
       </c>
       <c r="AE4" s="51" t="n">
         <f aca="false">SUM(AE6:AE370)</f>
-        <v>17.2</v>
+        <v>20.5135135135135</v>
       </c>
       <c r="AF4" s="51" t="n">
         <f aca="false">SUM(AF6:AF370)</f>
-        <v>4.2</v>
+        <v>3.72972972972973</v>
       </c>
       <c r="AG4" s="51" t="n">
         <f aca="false">SUM(AG6:AG370)</f>
-        <v>16.6</v>
+        <v>12.1621621621622</v>
       </c>
       <c r="AH4" s="48" t="n">
         <f aca="false">SUM(AH6:AH370)</f>
-        <v>2337.306</v>
+        <v>2614.08648648649</v>
       </c>
       <c r="AI4" s="48" t="n">
         <f aca="false">SUM(AI6:AI370)</f>
-        <v>228.7505</v>
+        <v>254.781851351351</v>
       </c>
       <c r="AJ4" s="48" t="n">
         <f aca="false">SUM(AJ6:AJ370)</f>
-        <v>525.596</v>
+        <v>589.754594594595</v>
       </c>
       <c r="AK4" s="48" t="n">
         <f aca="false">SUM(AK6:AK370)</f>
-        <v>133.796</v>
+        <v>98.027027027027</v>
       </c>
       <c r="AL4" s="48" t="n">
         <f aca="false">SUM(AL6:AL370)</f>
-        <v>365.947648760331</v>
+        <v>409.466093701139</v>
       </c>
       <c r="AM4" s="48" t="n">
         <f aca="false">SUM(AM6:AM370)</f>
-        <v>618.37</v>
+        <v>651.18</v>
       </c>
       <c r="AN4" s="47" t="n">
         <f aca="false">SUM(AN6:AN370)</f>
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="AO4" s="48" t="n">
         <f aca="false">SUM(AO6:AO370)</f>
-        <v>81.7</v>
+        <v>85.5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5049,7 +5049,7 @@
       </c>
       <c r="Y6" s="33" t="n">
         <f aca="false">AH6-AI6-AJ6-AK6-AL6-AM6-AO6</f>
-        <v>62.6280826446281</v>
+        <v>69.356477551932</v>
       </c>
       <c r="AA6" s="58" t="n">
         <f aca="false">MAX(0,B6-E6-H6)</f>
@@ -5065,11 +5065,11 @@
       </c>
       <c r="AD6" s="59" t="n">
         <f aca="false">E6+AA6*TASA_USADA</f>
-        <v>4.6</v>
+        <v>4.72972972972973</v>
       </c>
       <c r="AE6" s="59" t="n">
         <f aca="false">F6+AB6*TASA_USADA</f>
-        <v>3.6</v>
+        <v>3.72972972972973</v>
       </c>
       <c r="AF6" s="59" t="n">
         <f aca="false">G6+AC6*TASA_USADA</f>
@@ -5077,27 +5077,27 @@
       </c>
       <c r="AG6" s="59" t="n">
         <f aca="false">H6+I6+J6+(AA6+AB6+AC6)*(1-TASA_USADA)</f>
-        <v>0.8</v>
+        <v>0.54054054054054</v>
       </c>
       <c r="AH6" s="60" t="n">
         <f aca="false">AD6*P1_PVP+AE6*P2_PVP+AF6*P3_PVP</f>
-        <v>281.918</v>
+        <v>290.996486486486</v>
       </c>
       <c r="AI6" s="60" t="n">
         <f aca="false">AD6*P1_CPROD+AE6*P2_CPROD+AF6*P3_CPROD</f>
-        <v>28.41322</v>
+        <v>29.3503486486486</v>
       </c>
       <c r="AJ6" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L6),L6,E6*P1_LOG+F6*P2_LOG+G6*P3_LOG)+IF(ISNUMBER(M6),M6,AA6*P1_LOG+AB6*P2_LOG+AC6*P3_LOG)*TASA_USADA</f>
-        <v>64.212</v>
+        <v>66.3032432432432</v>
       </c>
       <c r="AK6" s="60" t="n">
         <f aca="false">AG6*COSTE_DEV</f>
-        <v>6.448</v>
+        <v>4.35675675675676</v>
       </c>
       <c r="AL6" s="60" t="n">
         <f aca="false">AD6*P1_IVAN+AE6*P2_IVAN+AF6*P3_IVAN-AG6*IVA_DEV</f>
-        <v>43.9966973553719</v>
+        <v>45.4096602859057</v>
       </c>
       <c r="AM6" s="60" t="n">
         <f aca="false">N6*(1+RECARGO_ADS)</f>
@@ -5188,7 +5188,7 @@
       </c>
       <c r="Y7" s="33" t="n">
         <f aca="false">AH7-AI7-AJ7-AK7-AL7-AM7-AO7</f>
-        <v>8.63823140495868</v>
+        <v>14.6518851909761</v>
       </c>
       <c r="AA7" s="58" t="n">
         <f aca="false">MAX(0,B7-E7-H7)</f>
@@ -5204,7 +5204,7 @@
       </c>
       <c r="AD7" s="59" t="n">
         <f aca="false">E7+AA7*TASA_USADA</f>
-        <v>5.2</v>
+        <v>5.45945945945946</v>
       </c>
       <c r="AE7" s="59" t="n">
         <f aca="false">F7+AB7*TASA_USADA</f>
@@ -5216,27 +5216,27 @@
       </c>
       <c r="AG7" s="59" t="n">
         <f aca="false">H7+I7+J7+(AA7+AB7+AC7)*(1-TASA_USADA)</f>
-        <v>1.8</v>
+        <v>1.54054054054054</v>
       </c>
       <c r="AH7" s="60" t="n">
         <f aca="false">AD7*P1_PVP+AE7*P2_PVP+AF7*P3_PVP</f>
-        <v>195.938</v>
+        <v>203.719189189189</v>
       </c>
       <c r="AI7" s="60" t="n">
         <f aca="false">AD7*P1_CPROD+AE7*P2_CPROD+AF7*P3_CPROD</f>
-        <v>17.33688</v>
+        <v>17.9616324324324</v>
       </c>
       <c r="AJ7" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L7),L7,E7*P1_LOG+F7*P2_LOG+G7*P3_LOG)+IF(ISNUMBER(M7),M7,AA7*P1_LOG+AB7*P2_LOG+AC7*P3_LOG)*TASA_USADA</f>
-        <v>46.678</v>
+        <v>48.67</v>
       </c>
       <c r="AK7" s="60" t="n">
         <f aca="false">AG7*COSTE_DEV</f>
-        <v>14.508</v>
+        <v>12.4167567567568</v>
       </c>
       <c r="AL7" s="60" t="n">
         <f aca="false">AD7*P1_IVAN+AE7*P2_IVAN+AF7*P3_IVAN-AG7*IVA_DEV</f>
-        <v>30.9968885950413</v>
+        <v>32.2389148090239</v>
       </c>
       <c r="AM7" s="60" t="n">
         <f aca="false">N7*(1+RECARGO_ADS)</f>
@@ -5275,7 +5275,7 @@
       <c r="I8" s="54"/>
       <c r="J8" s="54"/>
       <c r="K8" s="54" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L8" s="55" t="n">
         <v>22.65</v>
@@ -5325,7 +5325,7 @@
       </c>
       <c r="Y8" s="33" t="n">
         <f aca="false">AH8-AI8-AJ8-AK8-AL8-AM8-AO8</f>
-        <v>38.9722314049587</v>
+        <v>44.9424257315166</v>
       </c>
       <c r="AA8" s="58" t="n">
         <f aca="false">MAX(0,B8-E8-H8)</f>
@@ -5341,7 +5341,7 @@
       </c>
       <c r="AD8" s="59" t="n">
         <f aca="false">E8+AA8*TASA_USADA</f>
-        <v>5.2</v>
+        <v>5.45945945945946</v>
       </c>
       <c r="AE8" s="59" t="n">
         <f aca="false">F8+AB8*TASA_USADA</f>
@@ -5353,27 +5353,27 @@
       </c>
       <c r="AG8" s="59" t="n">
         <f aca="false">H8+I8+J8+(AA8+AB8+AC8)*(1-TASA_USADA)</f>
-        <v>0.8</v>
+        <v>0.54054054054054</v>
       </c>
       <c r="AH8" s="60" t="n">
         <f aca="false">AD8*P1_PVP+AE8*P2_PVP+AF8*P3_PVP</f>
-        <v>195.938</v>
+        <v>203.719189189189</v>
       </c>
       <c r="AI8" s="60" t="n">
         <f aca="false">AD8*P1_CPROD+AE8*P2_CPROD+AF8*P3_CPROD</f>
-        <v>17.33688</v>
+        <v>17.9616324324324</v>
       </c>
       <c r="AJ8" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L8),L8,E8*P1_LOG+F8*P2_LOG+G8*P3_LOG)+IF(ISNUMBER(M8),M8,AA8*P1_LOG+AB8*P2_LOG+AC8*P3_LOG)*TASA_USADA</f>
-        <v>47.754</v>
+        <v>49.7894594594595</v>
       </c>
       <c r="AK8" s="60" t="n">
         <f aca="false">AG8*COSTE_DEV</f>
-        <v>6.448</v>
+        <v>4.35675675675676</v>
       </c>
       <c r="AL8" s="60" t="n">
         <f aca="false">AD8*P1_IVAN+AE8*P2_IVAN+AF8*P3_IVAN-AG8*IVA_DEV</f>
-        <v>30.9968885950413</v>
+        <v>32.2389148090239</v>
       </c>
       <c r="AM8" s="60" t="n">
         <f aca="false">N8*(1+RECARGO_ADS)</f>
@@ -5402,7 +5402,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="54" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F9" s="54" t="n">
         <v>2</v>
@@ -5416,13 +5416,13 @@
       </c>
       <c r="J9" s="54"/>
       <c r="K9" s="54" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L9" s="55" t="n">
-        <v>42.15</v>
+        <v>50.21</v>
       </c>
       <c r="M9" s="55" t="n">
-        <v>54.7</v>
+        <v>46.64</v>
       </c>
       <c r="N9" s="55" t="n">
         <v>50.46</v>
@@ -5436,7 +5436,7 @@
       </c>
       <c r="Q9" s="31" t="n">
         <f aca="false">AA9+AB9+AC9</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="R9" s="32" t="n">
         <f aca="false">B9*P1_PVP+C9*P2_PVP+D9*P3_PVP</f>
@@ -5456,23 +5456,23 @@
       </c>
       <c r="V9" s="34" t="n">
         <f aca="false">IF(E9+F9+G9+H9+I9+J9&gt;0,(E9+F9+G9)/(E9+F9+G9+H9+I9+J9),"")</f>
-        <v>0.666666666666667</v>
+        <v>0.7</v>
       </c>
       <c r="W9" s="33" t="n">
         <f aca="false">E9*(P1_PVP-P1_CPROD)+F9*(P2_PVP-P2_CPROD)+G9*(P3_PVP-P3_CPROD)-IF(ISNUMBER(L9),L9,E9*P1_LOG+F9*P2_LOG+G9*P3_LOG)</f>
-        <v>153.711</v>
+        <v>173.2331</v>
       </c>
       <c r="X9" s="33" t="n">
         <f aca="false">W9-(E9*P1_IVAN+F9*P2_IVAN+G9*P3_IVAN)-(H9+I9+J9)*(COSTE_DEV-IVA_DEV)-AM9-AO9</f>
-        <v>29.8785950413223</v>
+        <v>44.6137190082644</v>
       </c>
       <c r="Y9" s="33" t="n">
         <f aca="false">AH9-AI9-AJ9-AK9-AL9-AM9-AO9</f>
-        <v>107.506859504132</v>
+        <v>121.456059861514</v>
       </c>
       <c r="AA9" s="58" t="n">
         <f aca="false">MAX(0,B9-E9-H9)</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AB9" s="58" t="n">
         <f aca="false">MAX(0,C9-F9-I9)</f>
@@ -5484,11 +5484,11 @@
       </c>
       <c r="AD9" s="59" t="n">
         <f aca="false">E9+AA9*TASA_USADA</f>
-        <v>7.8</v>
+        <v>8.32432432432433</v>
       </c>
       <c r="AE9" s="59" t="n">
         <f aca="false">F9+AB9*TASA_USADA</f>
-        <v>2.8</v>
+        <v>2.86486486486487</v>
       </c>
       <c r="AF9" s="59" t="n">
         <f aca="false">G9+AC9*TASA_USADA</f>
@@ -5496,27 +5496,27 @@
       </c>
       <c r="AG9" s="59" t="n">
         <f aca="false">H9+I9+J9+(AA9+AB9+AC9)*(1-TASA_USADA)</f>
-        <v>4.4</v>
+        <v>3.81081081081081</v>
       </c>
       <c r="AH9" s="60" t="n">
         <f aca="false">AD9*P1_PVP+AE9*P2_PVP+AF9*P3_PVP</f>
-        <v>395.884</v>
+        <v>414.202432432432</v>
       </c>
       <c r="AI9" s="60" t="n">
         <f aca="false">AD9*P1_CPROD+AE9*P2_CPROD+AF9*P3_CPROD</f>
-        <v>39.48956</v>
+        <v>41.0644567567568</v>
       </c>
       <c r="AJ9" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L9),L9,E9*P1_LOG+F9*P2_LOG+G9*P3_LOG)+IF(ISNUMBER(M9),M9,AA9*P1_LOG+AB9*P2_LOG+AC9*P3_LOG)*TASA_USADA</f>
-        <v>85.91</v>
+        <v>90.5472972972973</v>
       </c>
       <c r="AK9" s="60" t="n">
         <f aca="false">AG9*COSTE_DEV</f>
-        <v>35.464</v>
+        <v>30.7151351351351</v>
       </c>
       <c r="AL9" s="60" t="n">
         <f aca="false">AD9*P1_IVAN+AE9*P2_IVAN+AF9*P3_IVAN-AG9*IVA_DEV</f>
-        <v>61.8535804958678</v>
+        <v>64.7594833817288</v>
       </c>
       <c r="AM9" s="60" t="n">
         <f aca="false">N9*(1+RECARGO_ADS)</f>
@@ -5547,7 +5547,9 @@
       <c r="E10" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="F10" s="54"/>
+      <c r="F10" s="54" t="n">
+        <v>3</v>
+      </c>
       <c r="G10" s="54"/>
       <c r="H10" s="54"/>
       <c r="I10" s="54"/>
@@ -5556,10 +5558,10 @@
         <v>1</v>
       </c>
       <c r="L10" s="55" t="n">
+        <v>30.17</v>
+      </c>
+      <c r="M10" s="55" t="n">
         <v>7.2</v>
-      </c>
-      <c r="M10" s="55" t="n">
-        <v>30.17</v>
       </c>
       <c r="N10" s="55" t="n">
         <v>41.21</v>
@@ -5571,7 +5573,7 @@
       </c>
       <c r="Q10" s="31" t="n">
         <f aca="false">AA10+AB10+AC10</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="R10" s="32" t="n">
         <f aca="false">B10*P1_PVP+C10*P2_PVP+D10*P3_PVP</f>
@@ -5595,15 +5597,15 @@
       </c>
       <c r="W10" s="33" t="n">
         <f aca="false">E10*(P1_PVP-P1_CPROD)+F10*(P2_PVP-P2_CPROD)+G10*(P3_PVP-P3_CPROD)-IF(ISNUMBER(L10),L10,E10*P1_LOG+F10*P2_LOG+G10*P3_LOG)</f>
-        <v>20.3821</v>
+        <v>102.9347</v>
       </c>
       <c r="X10" s="33" t="n">
         <f aca="false">W10-(E10*P1_IVAN+F10*P2_IVAN+G10*P3_IVAN)-(H10+I10+J10)*(COSTE_DEV-IVA_DEV)-AM10-AO10</f>
-        <v>-30.3648760330579</v>
+        <v>33.8738842975206</v>
       </c>
       <c r="Y10" s="33" t="n">
         <f aca="false">AH10-AI10-AJ10-AK10-AL10-AM10-AO10</f>
-        <v>27.0542314049587</v>
+        <v>46.2723698905517</v>
       </c>
       <c r="AA10" s="58" t="n">
         <f aca="false">MAX(0,B10-E10-H10)</f>
@@ -5611,7 +5613,7 @@
       </c>
       <c r="AB10" s="58" t="n">
         <f aca="false">MAX(0,C10-F10-I10)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AC10" s="58" t="n">
         <f aca="false">MAX(0,D10-G10-J10)</f>
@@ -5619,11 +5621,11 @@
       </c>
       <c r="AD10" s="59" t="n">
         <f aca="false">E10+AA10*TASA_USADA</f>
-        <v>1.8</v>
+        <v>1.86486486486487</v>
       </c>
       <c r="AE10" s="59" t="n">
         <f aca="false">F10+AB10*TASA_USADA</f>
-        <v>2.4</v>
+        <v>3</v>
       </c>
       <c r="AF10" s="59" t="n">
         <f aca="false">G10+AC10*TASA_USADA</f>
@@ -5631,27 +5633,27 @@
       </c>
       <c r="AG10" s="59" t="n">
         <f aca="false">H10+I10+J10+(AA10+AB10+AC10)*(1-TASA_USADA)</f>
-        <v>0.8</v>
+        <v>0.135135135135135</v>
       </c>
       <c r="AH10" s="60" t="n">
         <f aca="false">AD10*P1_PVP+AE10*P2_PVP+AF10*P3_PVP</f>
-        <v>149.958</v>
+        <v>175.897297297297</v>
       </c>
       <c r="AI10" s="60" t="n">
         <f aca="false">AD10*P1_CPROD+AE10*P2_CPROD+AF10*P3_CPROD</f>
-        <v>15.89214</v>
+        <v>18.9378081081081</v>
       </c>
       <c r="AJ10" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L10),L10,E10*P1_LOG+F10*P2_LOG+G10*P3_LOG)+IF(ISNUMBER(M10),M10,AA10*P1_LOG+AB10*P2_LOG+AC10*P3_LOG)*TASA_USADA</f>
-        <v>31.336</v>
+        <v>36.397027027027</v>
       </c>
       <c r="AK10" s="60" t="n">
         <f aca="false">AG10*COSTE_DEV</f>
-        <v>6.448</v>
+        <v>1.08918918918919</v>
       </c>
       <c r="AL10" s="60" t="n">
         <f aca="false">AD10*P1_IVAN+AE10*P2_IVAN+AF10*P3_IVAN-AG10*IVA_DEV</f>
-        <v>23.2676285950413</v>
+        <v>27.2409030824213</v>
       </c>
       <c r="AM10" s="60" t="n">
         <f aca="false">N10*(1+RECARGO_ADS)</f>
@@ -5680,21 +5682,23 @@
         <v>1</v>
       </c>
       <c r="E11" s="54" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="54"/>
+      <c r="G11" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="54"/>
-      <c r="G11" s="54"/>
       <c r="H11" s="54"/>
       <c r="I11" s="54"/>
       <c r="J11" s="54"/>
       <c r="K11" s="54" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L11" s="55" t="n">
-        <v>6.85</v>
+        <v>22.11</v>
       </c>
       <c r="M11" s="55" t="n">
-        <v>60.02</v>
+        <v>44.76</v>
       </c>
       <c r="N11" s="55" t="n">
         <v>64.81</v>
@@ -5706,7 +5710,7 @@
       </c>
       <c r="Q11" s="31" t="n">
         <f aca="false">AA11+AB11+AC11</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="R11" s="32" t="n">
         <f aca="false">B11*P1_PVP+C11*P2_PVP+D11*P3_PVP</f>
@@ -5730,19 +5734,19 @@
       </c>
       <c r="W11" s="33" t="n">
         <f aca="false">E11*(P1_PVP-P1_CPROD)+F11*(P2_PVP-P2_CPROD)+G11*(P3_PVP-P3_CPROD)-IF(ISNUMBER(L11),L11,E11*P1_LOG+F11*P2_LOG+G11*P3_LOG)</f>
-        <v>20.7321</v>
+        <v>75.8205</v>
       </c>
       <c r="X11" s="33" t="n">
         <f aca="false">W11-(E11*P1_IVAN+F11*P2_IVAN+G11*P3_IVAN)-(H11+I11+J11)*(COSTE_DEV-IVA_DEV)-AM11-AO11</f>
-        <v>-57.4148760330579</v>
+        <v>-14.5357024793388</v>
       </c>
       <c r="Y11" s="33" t="n">
         <f aca="false">AH11-AI11-AJ11-AK11-AL11-AM11-AO11</f>
-        <v>47.6401983471074</v>
+        <v>69.3591467500559</v>
       </c>
       <c r="AA11" s="58" t="n">
         <f aca="false">MAX(0,B11-E11-H11)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AB11" s="58" t="n">
         <f aca="false">MAX(0,C11-F11-I11)</f>
@@ -5750,43 +5754,43 @@
       </c>
       <c r="AC11" s="58" t="n">
         <f aca="false">MAX(0,D11-G11-J11)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD11" s="59" t="n">
         <f aca="false">E11+AA11*TASA_USADA</f>
-        <v>5</v>
+        <v>5.45945945945946</v>
       </c>
       <c r="AE11" s="59" t="n">
         <f aca="false">F11+AB11*TASA_USADA</f>
-        <v>1.6</v>
+        <v>1.72972972972973</v>
       </c>
       <c r="AF11" s="59" t="n">
         <f aca="false">G11+AC11*TASA_USADA</f>
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="AG11" s="59" t="n">
         <f aca="false">H11+I11+J11+(AA11+AB11+AC11)*(1-TASA_USADA)</f>
-        <v>1.6</v>
+        <v>0.810810810810811</v>
       </c>
       <c r="AH11" s="60" t="n">
         <f aca="false">AD11*P1_PVP+AE11*P2_PVP+AF11*P3_PVP</f>
-        <v>253.926</v>
+        <v>282.891081081081</v>
       </c>
       <c r="AI11" s="60" t="n">
         <f aca="false">AD11*P1_CPROD+AE11*P2_CPROD+AF11*P3_CPROD</f>
-        <v>25.52374</v>
+        <v>28.6995648648649</v>
       </c>
       <c r="AJ11" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L11),L11,E11*P1_LOG+F11*P2_LOG+G11*P3_LOG)+IF(ISNUMBER(M11),M11,AA11*P1_LOG+AB11*P2_LOG+AC11*P3_LOG)*TASA_USADA</f>
-        <v>54.866</v>
+        <v>60.8213513513514</v>
       </c>
       <c r="AK11" s="60" t="n">
         <f aca="false">AG11*COSTE_DEV</f>
-        <v>12.896</v>
+        <v>6.53513513513513</v>
       </c>
       <c r="AL11" s="60" t="n">
         <f aca="false">AD11*P1_IVAN+AE11*P2_IVAN+AF11*P3_IVAN-AG11*IVA_DEV</f>
-        <v>39.6400616528926</v>
+        <v>44.1158829796739</v>
       </c>
       <c r="AM11" s="60" t="n">
         <f aca="false">N11*(1+RECARGO_ADS)</f>
@@ -5820,7 +5824,9 @@
       <c r="H12" s="54"/>
       <c r="I12" s="54"/>
       <c r="J12" s="54"/>
-      <c r="K12" s="54"/>
+      <c r="K12" s="54" t="n">
+        <v>4</v>
+      </c>
       <c r="L12" s="55" t="n">
         <v>0</v>
       </c>
@@ -5869,7 +5875,7 @@
       </c>
       <c r="Y12" s="33" t="n">
         <f aca="false">AH12-AI12-AJ12-AK12-AL12-AM12-AO12</f>
-        <v>-28.0618347107438</v>
+        <v>-18.6963077953987</v>
       </c>
       <c r="AA12" s="58" t="n">
         <f aca="false">MAX(0,B12-E12-H12)</f>
@@ -5885,11 +5891,11 @@
       </c>
       <c r="AD12" s="59" t="n">
         <f aca="false">E12+AA12*TASA_USADA</f>
-        <v>4</v>
+        <v>4.32432432432433</v>
       </c>
       <c r="AE12" s="59" t="n">
         <f aca="false">F12+AB12*TASA_USADA</f>
-        <v>0.8</v>
+        <v>0.864864864864865</v>
       </c>
       <c r="AF12" s="59" t="n">
         <f aca="false">G12+AC12*TASA_USADA</f>
@@ -5897,27 +5903,27 @@
       </c>
       <c r="AG12" s="59" t="n">
         <f aca="false">H12+I12+J12+(AA12+AB12+AC12)*(1-TASA_USADA)</f>
-        <v>1.2</v>
+        <v>0.810810810810811</v>
       </c>
       <c r="AH12" s="60" t="n">
         <f aca="false">AD12*P1_PVP+AE12*P2_PVP+AF12*P3_PVP</f>
-        <v>151.952</v>
+        <v>164.272432432432</v>
       </c>
       <c r="AI12" s="60" t="n">
         <f aca="false">AD12*P1_CPROD+AE12*P2_CPROD+AF12*P3_CPROD</f>
-        <v>13.48424</v>
+        <v>14.5775567567568</v>
       </c>
       <c r="AJ12" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L12),L12,E12*P1_LOG+F12*P2_LOG+G12*P3_LOG)+IF(ISNUMBER(M12),M12,AA12*P1_LOG+AB12*P2_LOG+AC12*P3_LOG)*TASA_USADA</f>
-        <v>37.616</v>
+        <v>40.665945945946</v>
       </c>
       <c r="AK12" s="60" t="n">
         <f aca="false">AG12*COSTE_DEV</f>
-        <v>9.672</v>
+        <v>6.53513513513513</v>
       </c>
       <c r="AL12" s="60" t="n">
         <f aca="false">AD12*P1_IVAN+AE12*P2_IVAN+AF12*P3_IVAN-AG12*IVA_DEV</f>
-        <v>24.0315947107438</v>
+        <v>25.9801023899933</v>
       </c>
       <c r="AM12" s="60" t="n">
         <f aca="false">N12*(1+RECARGO_ADS)</f>
@@ -5945,20 +5951,26 @@
       <c r="D13" s="54" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="54"/>
-      <c r="F13" s="54"/>
+      <c r="E13" s="54" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" s="54" t="n">
+        <v>2</v>
+      </c>
       <c r="G13" s="54"/>
       <c r="H13" s="54"/>
       <c r="I13" s="54"/>
-      <c r="J13" s="54"/>
+      <c r="J13" s="54" t="n">
+        <v>1</v>
+      </c>
       <c r="K13" s="54" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L13" s="55" t="n">
-        <v>0</v>
+        <v>38.42</v>
       </c>
       <c r="M13" s="55" t="n">
-        <v>103.76</v>
+        <v>58.14</v>
       </c>
       <c r="N13" s="55" t="n">
         <v>78.33</v>
@@ -5970,7 +5982,7 @@
       </c>
       <c r="Q13" s="31" t="n">
         <f aca="false">AA13+AB13+AC13</f>
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="R13" s="32" t="n">
         <f aca="false">B13*P1_PVP+C13*P2_PVP+D13*P3_PVP</f>
@@ -5988,69 +6000,69 @@
         <f aca="false">IF(N13&gt;0,R13/N13,"")</f>
         <v>6.25379803395889</v>
       </c>
-      <c r="V13" s="34" t="str">
+      <c r="V13" s="34" t="n">
         <f aca="false">IF(E13+F13+G13+H13+I13+J13&gt;0,(E13+F13+G13)/(E13+F13+G13+H13+I13+J13),"")</f>
-        <v/>
+        <v>0.833333333333333</v>
       </c>
       <c r="W13" s="33" t="n">
         <f aca="false">E13*(P1_PVP-P1_CPROD)+F13*(P2_PVP-P2_CPROD)+G13*(P3_PVP-P3_CPROD)-IF(ISNUMBER(L13),L13,E13*P1_LOG+F13*P2_LOG+G13*P3_LOG)</f>
-        <v>0</v>
+        <v>114.6747</v>
       </c>
       <c r="X13" s="33" t="n">
         <f aca="false">W13-(E13*P1_IVAN+F13*P2_IVAN+G13*P3_IVAN)-(H13+I13+J13)*(COSTE_DEV-IVA_DEV)-AM13-AO13</f>
-        <v>-91.63</v>
+        <v>-11.5854545454546</v>
       </c>
       <c r="Y13" s="33" t="n">
         <f aca="false">AH13-AI13-AJ13-AK13-AL13-AM13-AO13</f>
-        <v>93.2363801652893</v>
+        <v>103.415090462363</v>
       </c>
       <c r="AA13" s="58" t="n">
         <f aca="false">MAX(0,B13-E13-H13)</f>
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="AB13" s="58" t="n">
         <f aca="false">MAX(0,C13-F13-I13)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AC13" s="58" t="n">
         <f aca="false">MAX(0,D13-G13-J13)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AD13" s="59" t="n">
         <f aca="false">E13+AA13*TASA_USADA</f>
-        <v>7.2</v>
+        <v>8.18918918918919</v>
       </c>
       <c r="AE13" s="59" t="n">
         <f aca="false">F13+AB13*TASA_USADA</f>
-        <v>2.4</v>
+        <v>2.86486486486487</v>
       </c>
       <c r="AF13" s="59" t="n">
         <f aca="false">G13+AC13*TASA_USADA</f>
-        <v>1.6</v>
+        <v>0.864864864864865</v>
       </c>
       <c r="AG13" s="59" t="n">
         <f aca="false">H13+I13+J13+(AA13+AB13+AC13)*(1-TASA_USADA)</f>
-        <v>2.8</v>
+        <v>2.08108108108108</v>
       </c>
       <c r="AH13" s="60" t="n">
         <f aca="false">AD13*P1_PVP+AE13*P2_PVP+AF13*P3_PVP</f>
-        <v>391.888</v>
+        <v>403.394324324324</v>
       </c>
       <c r="AI13" s="60" t="n">
         <f aca="false">AD13*P1_CPROD+AE13*P2_CPROD+AF13*P3_CPROD</f>
-        <v>40.45272</v>
+        <v>39.7628891891892</v>
       </c>
       <c r="AJ13" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L13),L13,E13*P1_LOG+F13*P2_LOG+G13*P3_LOG)+IF(ISNUMBER(M13),M13,AA13*P1_LOG+AB13*P2_LOG+AC13*P3_LOG)*TASA_USADA</f>
-        <v>83.008</v>
+        <v>88.7032432432433</v>
       </c>
       <c r="AK13" s="60" t="n">
         <f aca="false">AG13*COSTE_DEV</f>
-        <v>22.568</v>
+        <v>16.7735135135135</v>
       </c>
       <c r="AL13" s="60" t="n">
         <f aca="false">AD13*P1_IVAN+AE13*P2_IVAN+AF13*P3_IVAN-AG13*IVA_DEV</f>
-        <v>60.9928998347107</v>
+        <v>63.1095879160152</v>
       </c>
       <c r="AM13" s="60" t="n">
         <f aca="false">N13*(1+RECARGO_ADS)</f>
@@ -6058,7 +6070,7 @@
       </c>
       <c r="AN13" s="58" t="n">
         <f aca="false">IF(ISNUMBER(L13),E13+F13+G13+AA13+AB13+AC13,0)</f>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AO13" s="60" t="n">
         <f aca="false">P13*COMISION</f>
@@ -6070,7 +6082,7 @@
         <v>46308</v>
       </c>
       <c r="B14" s="54" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C14" s="54" t="n">
         <v>1</v>
@@ -6078,26 +6090,30 @@
       <c r="D14" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="54"/>
+      <c r="E14" s="54" t="n">
+        <v>1</v>
+      </c>
       <c r="F14" s="54"/>
       <c r="G14" s="54"/>
       <c r="H14" s="54"/>
       <c r="I14" s="54"/>
       <c r="J14" s="54"/>
-      <c r="K14" s="54"/>
+      <c r="K14" s="54" t="n">
+        <v>3</v>
+      </c>
       <c r="L14" s="55" t="n">
-        <v>0</v>
+        <v>7.39</v>
       </c>
       <c r="M14" s="55" t="n">
-        <v>60.53</v>
+        <v>61.2</v>
       </c>
       <c r="N14" s="55" t="n">
-        <v>68.04</v>
+        <v>68.05</v>
       </c>
       <c r="O14" s="56"/>
       <c r="P14" s="31" t="n">
         <f aca="false">B14+C14+D14</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q14" s="31" t="n">
         <f aca="false">AA14+AB14+AC14</f>
@@ -6105,35 +6121,35 @@
       </c>
       <c r="R14" s="32" t="n">
         <f aca="false">B14*P1_PVP+C14*P2_PVP+D14*P3_PVP</f>
-        <v>269.92</v>
+        <v>299.91</v>
       </c>
       <c r="S14" s="32" t="n">
         <f aca="false">IF(P14&gt;0,R14/P14,"")</f>
-        <v>33.74</v>
+        <v>33.3233333333333</v>
       </c>
       <c r="T14" s="32" t="n">
         <f aca="false">IF(P14&gt;0,N14/P14,"")</f>
-        <v>8.505</v>
+        <v>7.56111111111111</v>
       </c>
       <c r="U14" s="57" t="n">
         <f aca="false">IF(N14&gt;0,R14/N14,"")</f>
-        <v>3.96707818930041</v>
-      </c>
-      <c r="V14" s="34" t="str">
+        <v>4.40720058780309</v>
+      </c>
+      <c r="V14" s="34" t="n">
         <f aca="false">IF(E14+F14+G14+H14+I14+J14&gt;0,(E14+F14+G14)/(E14+F14+G14+H14+I14+J14),"")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="W14" s="33" t="n">
         <f aca="false">E14*(P1_PVP-P1_CPROD)+F14*(P2_PVP-P2_CPROD)+G14*(P3_PVP-P3_CPROD)-IF(ISNUMBER(L14),L14,E14*P1_LOG+F14*P2_LOG+G14*P3_LOG)</f>
-        <v>0</v>
+        <v>20.1921</v>
       </c>
       <c r="X14" s="33" t="n">
         <f aca="false">W14-(E14*P1_IVAN+F14*P2_IVAN+G14*P3_IVAN)-(H14+I14+J14)*(COSTE_DEV-IVA_DEV)-AM14-AO14</f>
-        <v>-75.64</v>
+        <v>-61.1948760330579</v>
       </c>
       <c r="Y14" s="33" t="n">
         <f aca="false">AH14-AI14-AJ14-AK14-AL14-AM14-AO14</f>
-        <v>23.9875041322314</v>
+        <v>51.1591824882734</v>
       </c>
       <c r="AA14" s="58" t="n">
         <f aca="false">MAX(0,B14-E14-H14)</f>
@@ -6149,51 +6165,51 @@
       </c>
       <c r="AD14" s="59" t="n">
         <f aca="false">E14+AA14*TASA_USADA</f>
-        <v>4.8</v>
+        <v>6.18918918918919</v>
       </c>
       <c r="AE14" s="59" t="n">
         <f aca="false">F14+AB14*TASA_USADA</f>
-        <v>0.8</v>
+        <v>0.864864864864865</v>
       </c>
       <c r="AF14" s="59" t="n">
         <f aca="false">G14+AC14*TASA_USADA</f>
-        <v>0.8</v>
+        <v>0.864864864864865</v>
       </c>
       <c r="AG14" s="59" t="n">
         <f aca="false">H14+I14+J14+(AA14+AB14+AC14)*(1-TASA_USADA)</f>
-        <v>1.6</v>
+        <v>1.08108108108108</v>
       </c>
       <c r="AH14" s="60" t="n">
         <f aca="false">AD14*P1_PVP+AE14*P2_PVP+AF14*P3_PVP</f>
-        <v>215.936</v>
+        <v>263.434324324324</v>
       </c>
       <c r="AI14" s="60" t="n">
         <f aca="false">AD14*P1_CPROD+AE14*P2_CPROD+AF14*P3_CPROD</f>
-        <v>21.18952</v>
+        <v>25.3154891891892</v>
       </c>
       <c r="AJ14" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L14),L14,E14*P1_LOG+F14*P2_LOG+G14*P3_LOG)+IF(ISNUMBER(M14),M14,AA14*P1_LOG+AB14*P2_LOG+AC14*P3_LOG)*TASA_USADA</f>
-        <v>48.424</v>
+        <v>60.3197297297297</v>
       </c>
       <c r="AK14" s="60" t="n">
         <f aca="false">AG14*COSTE_DEV</f>
-        <v>12.896</v>
+        <v>8.71351351351351</v>
       </c>
       <c r="AL14" s="60" t="n">
         <f aca="false">AD14*P1_IVAN+AE14*P2_IVAN+AF14*P3_IVAN-AG14*IVA_DEV</f>
-        <v>33.7989758677686</v>
+        <v>41.3264094036185</v>
       </c>
       <c r="AM14" s="60" t="n">
         <f aca="false">N14*(1+RECARGO_ADS)</f>
-        <v>68.04</v>
+        <v>68.05</v>
       </c>
       <c r="AN14" s="58" t="n">
         <f aca="false">IF(ISNUMBER(L14),E14+F14+G14+AA14+AB14+AC14,0)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AO14" s="60" t="n">
         <f aca="false">P14*COMISION</f>
-        <v>7.6</v>
+        <v>8.55</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6201,15 +6217,17 @@
         <v>46309</v>
       </c>
       <c r="B15" s="54" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" s="54" t="n">
         <v>3</v>
       </c>
-      <c r="C15" s="54" t="n">
+      <c r="D15" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="D15" s="54" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="54"/>
       <c r="F15" s="54"/>
       <c r="G15" s="54"/>
       <c r="H15" s="54"/>
@@ -6217,54 +6235,54 @@
       <c r="J15" s="54"/>
       <c r="K15" s="54"/>
       <c r="L15" s="55" t="n">
-        <v>0</v>
+        <v>7.2</v>
       </c>
       <c r="M15" s="55" t="n">
-        <v>32.24</v>
+        <v>46.64</v>
       </c>
       <c r="N15" s="55" t="n">
-        <v>40.38</v>
+        <v>73.18</v>
       </c>
       <c r="O15" s="56"/>
       <c r="P15" s="31" t="n">
         <f aca="false">B15+C15+D15</f>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="Q15" s="31" t="n">
         <f aca="false">AA15+AB15+AC15</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R15" s="32" t="n">
         <f aca="false">B15*P1_PVP+C15*P2_PVP+D15*P3_PVP</f>
-        <v>129.96</v>
+        <v>239.93</v>
       </c>
       <c r="S15" s="32" t="n">
         <f aca="false">IF(P15&gt;0,R15/P15,"")</f>
-        <v>32.49</v>
+        <v>34.2757142857143</v>
       </c>
       <c r="T15" s="32" t="n">
         <f aca="false">IF(P15&gt;0,N15/P15,"")</f>
-        <v>10.095</v>
+        <v>10.4542857142857</v>
       </c>
       <c r="U15" s="57" t="n">
         <f aca="false">IF(N15&gt;0,R15/N15,"")</f>
-        <v>3.2184249628529</v>
-      </c>
-      <c r="V15" s="34" t="str">
+        <v>3.27862804044821</v>
+      </c>
+      <c r="V15" s="34" t="n">
         <f aca="false">IF(E15+F15+G15+H15+I15+J15&gt;0,(E15+F15+G15)/(E15+F15+G15+H15+I15+J15),"")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="W15" s="33" t="n">
         <f aca="false">E15*(P1_PVP-P1_CPROD)+F15*(P2_PVP-P2_CPROD)+G15*(P3_PVP-P3_CPROD)-IF(ISNUMBER(L15),L15,E15*P1_LOG+F15*P2_LOG+G15*P3_LOG)</f>
-        <v>0</v>
+        <v>20.3821</v>
       </c>
       <c r="X15" s="33" t="n">
         <f aca="false">W15-(E15*P1_IVAN+F15*P2_IVAN+G15*P3_IVAN)-(H15+I15+J15)*(COSTE_DEV-IVA_DEV)-AM15-AO15</f>
-        <v>-44.18</v>
+        <v>-64.2348760330579</v>
       </c>
       <c r="Y15" s="33" t="n">
         <f aca="false">AH15-AI15-AJ15-AK15-AL15-AM15-AO15</f>
-        <v>1.54396694214877</v>
+        <v>23.4605896805897</v>
       </c>
       <c r="AA15" s="58" t="n">
         <f aca="false">MAX(0,B15-E15-H15)</f>
@@ -6272,7 +6290,7 @@
       </c>
       <c r="AB15" s="58" t="n">
         <f aca="false">MAX(0,C15-F15-I15)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AC15" s="58" t="n">
         <f aca="false">MAX(0,D15-G15-J15)</f>
@@ -6280,11 +6298,11 @@
       </c>
       <c r="AD15" s="59" t="n">
         <f aca="false">E15+AA15*TASA_USADA</f>
-        <v>2.4</v>
+        <v>3.59459459459459</v>
       </c>
       <c r="AE15" s="59" t="n">
         <f aca="false">F15+AB15*TASA_USADA</f>
-        <v>0.8</v>
+        <v>2.59459459459459</v>
       </c>
       <c r="AF15" s="59" t="n">
         <f aca="false">G15+AC15*TASA_USADA</f>
@@ -6292,39 +6310,39 @@
       </c>
       <c r="AG15" s="59" t="n">
         <f aca="false">H15+I15+J15+(AA15+AB15+AC15)*(1-TASA_USADA)</f>
-        <v>0.8</v>
+        <v>0.810810810810811</v>
       </c>
       <c r="AH15" s="60" t="n">
         <f aca="false">AD15*P1_PVP+AE15*P2_PVP+AF15*P3_PVP</f>
-        <v>103.968</v>
+        <v>211.55972972973</v>
       </c>
       <c r="AI15" s="60" t="n">
         <f aca="false">AD15*P1_CPROD+AE15*P2_CPROD+AF15*P3_CPROD</f>
-        <v>9.6316</v>
+        <v>21.150472972973</v>
       </c>
       <c r="AJ15" s="60" t="n">
         <f aca="false">IF(ISNUMBER(L15),L15,E15*P1_LOG+F15*P2_LOG+G15*P3_LOG)+IF(ISNUMBER(M15),M15,AA15*P1_LOG+AB15*P2_LOG+AC15*P3_LOG)*TASA_USADA</f>
-        <v>25.792</v>
+        <v>47.5372972972973</v>
       </c>
       <c r="AK15" s="60" t="n">
         <f aca="false">AG15*COSTE_DEV</f>
-        <v>6.448</v>
+        <v>6.53513513513513</v>
       </c>
       <c r="AL15" s="60" t="n">
         <f aca="false">AD15*P1_IVAN+AE15*P2_IVAN+AF15*P3_IVAN-AG15*IVA_DEV</f>
-        <v>16.3724330578512</v>
+        <v>33.0462346437346</v>
       </c>
       <c r="AM15" s="60" t="n">
         <f aca="false">N15*(1+RECARGO_ADS)</f>
-        <v>40.38</v>
+        <v>73.18</v>
       </c>
       <c r="AN15" s="58" t="n">
         <f aca="false">IF(ISNUMBER(L15),E15+F15+G15+AA15+AB15+AC15,0)</f>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="AO15" s="60" t="n">
         <f aca="false">P15*COMISION</f>
-        <v>3.8</v>
+        <v>6.65</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51246,7 +51264,7 @@
       </c>
       <c r="C37" s="31" t="n">
         <f aca="false">(SUM(Diario!$E$6:$E$370)+SUM(Diario!$F$6:$F$370)+SUM(Diario!$G$6:$G$370))+(SUM(Diario!$H$6:$H$370)+SUM(Diario!$I$6:$I$370)+SUM(Diario!$J$6:$J$370))</f>
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="F37" s="67" t="s">
         <v>183</v>
@@ -51258,7 +51276,7 @@
       </c>
       <c r="C38" s="34" t="n">
         <f aca="false">IF(C37&gt;0,(SUM(Diario!$E$6:$E$370)+SUM(Diario!$F$6:$F$370)+SUM(Diario!$G$6:$G$370))/C37,"")</f>
-        <v>0.826086956521739</v>
+        <v>0.864864864864865</v>
       </c>
       <c r="F38" s="67" t="s">
         <v>185</v>
@@ -51270,7 +51288,7 @@
       </c>
       <c r="C39" s="34" t="n">
         <f aca="false">IF(AND(C37&gt;=C25,C38&lt;&gt;""),C38,C24)</f>
-        <v>0.8</v>
+        <v>0.864864864864865</v>
       </c>
       <c r="F39" s="67" t="s">
         <v>187</v>
@@ -51282,11 +51300,11 @@
       </c>
       <c r="C40" s="34" t="n">
         <f aca="false">IF(SUM(Diario!$P$6:$P$370)&gt;0,SUM(Diario!$C$6:$C$370)/SUM(Diario!$P$6:$P$370),"")</f>
-        <v>0.267441860465116</v>
+        <v>0.277777777777778</v>
       </c>
       <c r="D40" s="34" t="n">
         <f aca="false">IF(SUM(Diario!$P$6:$P$370)&gt;0,SUM(Diario!$D$6:$D$370)/SUM(Diario!$P$6:$P$370),"")</f>
-        <v>0.0581395348837209</v>
+        <v>0.0555555555555556</v>
       </c>
       <c r="F40" s="67" t="s">
         <v>189</v>
@@ -51298,11 +51316,11 @@
       </c>
       <c r="C41" s="34" t="n">
         <f aca="false">IF(C40="",C26,C40)</f>
-        <v>0.267441860465116</v>
+        <v>0.277777777777778</v>
       </c>
       <c r="D41" s="34" t="n">
         <f aca="false">IF(D40="",D26,D40)</f>
-        <v>0.0581395348837209</v>
+        <v>0.0555555555555556</v>
       </c>
       <c r="F41" s="67"/>
     </row>
@@ -51312,7 +51330,7 @@
       </c>
       <c r="C42" s="32" t="n">
         <f aca="false">IF(SUM(Diario!$AN$6:$AN$370)&gt;0,(SUM(Diario!$L$6:$L$370)+SUM(Diario!$M$6:$M$370))/SUM(Diario!$AN$6:$AN$370),"")</f>
-        <v>7.58719512195122</v>
+        <v>7.58364705882353</v>
       </c>
       <c r="F42" s="67" t="s">
         <v>192</v>
@@ -51324,7 +51342,7 @@
       </c>
       <c r="C43" s="32" t="n">
         <f aca="false">(1-C41-D41)*C5+C41*D5+D41*E5</f>
-        <v>33.8272093023256</v>
+        <v>33.8788888888889</v>
       </c>
       <c r="F43" s="67"/>
     </row>
@@ -51334,7 +51352,7 @@
       </c>
       <c r="C44" s="32" t="n">
         <f aca="false">(1-C41-D41)*(C5-C9-IF(C42="",C8,C42)-C14)+C41*(D5-D9-IF(C42="",D8,C42)-D14)+D41*(E5-E9-IF(C42="",E8,C42)-E14)</f>
-        <v>17.615571551122</v>
+        <v>17.651545778642</v>
       </c>
       <c r="F44" s="67" t="s">
         <v>195</v>
@@ -51346,7 +51364,7 @@
       </c>
       <c r="C45" s="32" t="n">
         <f aca="false">C39*C44-(1-C39)*C36-COMISION</f>
-        <v>11.5304572408976</v>
+        <v>13.227012565312</v>
       </c>
       <c r="F45" s="67" t="s">
         <v>197</v>
@@ -51358,7 +51376,7 @@
       </c>
       <c r="C46" s="33" t="n">
         <f aca="false">C45/(1+RECARGO_ADS)</f>
-        <v>11.5304572408976</v>
+        <v>13.227012565312</v>
       </c>
       <c r="F46" s="67" t="s">
         <v>199</v>
@@ -51370,7 +51388,7 @@
       </c>
       <c r="C47" s="72" t="n">
         <f aca="false">IF(C46&gt;0,C43/C46,"")</f>
-        <v>2.93372661600471</v>
+        <v>2.5613409469147</v>
       </c>
       <c r="F47" s="67" t="s">
         <v>201</v>

</xml_diff>

<commit_message>
Beneficio sin restar IVA; el CPA máximo para decidir sigue con IVA
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFjE4yx23BY3D6kaMQowKe
</commit_message>
<xml_diff>
--- a/contabilidad/CeraLux_Contabilidad.xlsx
+++ b/contabilidad/CeraLux_Contabilidad.xlsx
@@ -186,7 +186,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="250">
   <si>
     <t xml:space="preserve">CeraLux · Dashboard de rentabilidad</t>
   </si>
@@ -650,16 +650,13 @@
     <t xml:space="preserve">¿Descontar el IVA del beneficio?</t>
   </si>
   <si>
-    <t xml:space="preserve">SÍ</t>
+    <t xml:space="preserve">NO</t>
   </si>
   <si>
     <t xml:space="preserve">SÍ si facturas como autónomo o SL (Hacienda se queda ~4,8 € por Pack 1 entregado). NO solo para ver el bruto.</t>
   </si>
   <si>
     <t xml:space="preserve">¿El envío lleva IVA deducible?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NO</t>
   </si>
   <si>
     <t xml:space="preserve">NO: el export dice 'Coste de envío (SIN IVA)' y el coste total no le suma IVA, así que no hay IVA que deducir.</t>
@@ -797,7 +794,7 @@
     <t xml:space="preserve">CPA break-even (máximo que puedes pagar por pedido)</t>
   </si>
   <si>
-    <t xml:space="preserve">Por encima de este CPA pierdes dinero.</t>
+    <t xml:space="preserve">Por encima de este CPA pierdes dinero. Siempre con IVA, aunque el beneficio se vea sin restarlo (por prudencia).</t>
   </si>
   <si>
     <t xml:space="preserve">ROAS break-even</t>
@@ -1907,43 +1904,43 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>22.9958729338843</c:v>
+                  <c:v>58.41544375</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-26.1452763429752</c:v>
+                  <c:v>-2.68787500000001</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.64922914207006</c:v>
+                  <c:v>29.5482860119048</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>58.4114591942149</c:v>
+                  <c:v>109.394384375</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>35.7265909090909</c:v>
+                  <c:v>60.772115625</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>14.9950180785124</c:v>
+                  <c:v>47.572321875</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-71.3545851575824</c:v>
+                  <c:v>-56.655200124008</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>36.7725025826446</c:v>
+                  <c:v>85.81071875</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>-9.28123708677689</c:v>
+                  <c:v>19.1361625</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>27.503331242621</c:v>
+                  <c:v>64.8592464285714</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-6.21946803669812</c:v>
+                  <c:v>14.1641483630953</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>101.339236521055</c:v>
+                  <c:v>167.180376190476</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>32.8470878000787</c:v>
+                  <c:v>60.0451762380952</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1951,8 +1948,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="6407622"/>
-        <c:axId val="768210"/>
+        <c:axId val="97772333"/>
+        <c:axId val="23101351"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2121,11 +2118,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="6407622"/>
-        <c:axId val="768210"/>
+        <c:axId val="97772333"/>
+        <c:axId val="23101351"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="6407622"/>
+        <c:axId val="97772333"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2157,7 +2154,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="768210"/>
+        <c:crossAx val="23101351"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2165,7 +2162,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="768210"/>
+        <c:axId val="23101351"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2207,7 +2204,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6407622"/>
+        <c:crossAx val="97772333"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2406,7 +2403,7 @@
                 <c:formatCode>#,##0" €";[RED]\-#,##0" €";\-</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>223.239761780139</c:v>
+                  <c:v>657.555304983135</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -2447,8 +2444,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="80473490"/>
-        <c:axId val="22150094"/>
+        <c:axId val="23807062"/>
+        <c:axId val="52012147"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2545,11 +2542,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="80473490"/>
-        <c:axId val="22150094"/>
+        <c:axId val="23807062"/>
+        <c:axId val="52012147"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="80473490"/>
+        <c:axId val="23807062"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2581,7 +2578,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="22150094"/>
+        <c:crossAx val="52012147"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2589,7 +2586,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="22150094"/>
+        <c:axId val="52012147"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2631,7 +2628,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80473490"/>
+        <c:crossAx val="23807062"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3025,7 +3022,7 @@
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="10" t="n">
         <f aca="false">F25</f>
-        <v>223.239761780139</v>
+        <v>657.555304983135</v>
       </c>
       <c r="C7" s="10"/>
       <c r="D7" s="10" t="n">
@@ -3035,7 +3032,7 @@
       <c r="E7" s="10"/>
       <c r="F7" s="10" t="n">
         <f aca="false">SUMIFS(Diario!$X$6:$X$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)+F24</f>
-        <v>-273.960661157025</v>
+        <v>-51.3419000000001</v>
       </c>
       <c r="G7" s="10"/>
       <c r="H7" s="11" t="n">
@@ -3234,7 +3231,7 @@
       <c r="K17" s="15"/>
       <c r="L17" s="20" t="n">
         <f aca="false">F25/I3</f>
-        <v>13.1317506929493</v>
+        <v>38.6797238225374</v>
       </c>
       <c r="M17" s="20"/>
     </row>
@@ -3260,7 +3257,7 @@
       <c r="K18" s="15"/>
       <c r="L18" s="18" t="n">
         <f aca="false">L17*30</f>
-        <v>393.95252078848</v>
+        <v>1160.39171467612</v>
       </c>
       <c r="M18" s="18"/>
     </row>
@@ -3286,7 +3283,7 @@
       <c r="K19" s="21"/>
       <c r="L19" s="22" t="n">
         <f aca="false">IF(L16&gt;0,L18/L16,"")</f>
-        <v>0.039395252078848</v>
+        <v>0.116039171467612</v>
       </c>
       <c r="M19" s="22"/>
     </row>
@@ -3312,7 +3309,7 @@
       <c r="K20" s="15"/>
       <c r="L20" s="20" t="n">
         <f aca="false">BEN_PEDIDO</f>
-        <v>9.45028972502196</v>
+        <v>13.2265344237077</v>
       </c>
       <c r="M20" s="20"/>
     </row>
@@ -3324,11 +3321,11 @@
       <c r="D21" s="15"/>
       <c r="E21" s="19" t="n">
         <f aca="false">IF($F$16&gt;0,F21/$F$16,"")</f>
-        <v>-0.155613915096803</v>
+        <v>-0</v>
       </c>
       <c r="F21" s="17" t="n">
         <f aca="false">-SUMIFS(Diario!$AL$6:$AL$370,Diario!$A$6:$A$370,"&gt;="&amp;$C$3,Diario!$A$6:$A$370,"&lt;="&amp;$F$3)</f>
-        <v>-434.315543202996</v>
+        <v>-0</v>
       </c>
       <c r="H21" s="15" t="s">
         <v>39</v>
@@ -3364,7 +3361,7 @@
       <c r="K22" s="15"/>
       <c r="L22" s="20" t="n">
         <f aca="false">IF(ISNUMBER(L21),L20-L21*(1+RECARGO_ADS),"")</f>
-        <v>1.91168102936978</v>
+        <v>5.68792572805555</v>
       </c>
       <c r="M22" s="20"/>
     </row>
@@ -3376,11 +3373,11 @@
       <c r="D23" s="23"/>
       <c r="E23" s="24" t="n">
         <f aca="false">IF($F$16&gt;0,F23/$F$16,"")</f>
-        <v>0.0799861158080824</v>
+        <v>0.235600030904885</v>
       </c>
       <c r="F23" s="25" t="n">
         <f aca="false">SUM(F16:F22)</f>
-        <v>223.239761780139</v>
+        <v>657.555304983135</v>
       </c>
       <c r="H23" s="21" t="s">
         <v>43</v>
@@ -3390,7 +3387,7 @@
       <c r="K23" s="21"/>
       <c r="L23" s="26" t="n">
         <f aca="false">IF(NOT(ISNUMBER(L22)),"",IF(L22&lt;=0,"Baja el CPA",ROUNDUP((L16-F24/I3*30)/30/L22,0)))</f>
-        <v>175</v>
+        <v>59</v>
       </c>
       <c r="M23" s="26"/>
     </row>
@@ -3416,7 +3413,7 @@
       <c r="K24" s="15"/>
       <c r="L24" s="18" t="n">
         <f aca="false">IF(ISNUMBER(L23),L23*L21,"")</f>
-        <v>1319.25652173913</v>
+        <v>444.777913043478</v>
       </c>
       <c r="M24" s="18"/>
     </row>
@@ -3428,11 +3425,11 @@
       <c r="D25" s="23"/>
       <c r="E25" s="24" t="n">
         <f aca="false">IF($F$16&gt;0,F25/$F$16,"")</f>
-        <v>0.0799861158080824</v>
+        <v>0.235600030904885</v>
       </c>
       <c r="F25" s="25" t="n">
         <f aca="false">F23+F24</f>
-        <v>223.239761780139</v>
+        <v>657.555304983135</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3443,7 +3440,7 @@
       <c r="D26" s="27"/>
       <c r="F26" s="28" t="n">
         <f aca="false">IF(F16&gt;0,F25/F16,"")</f>
-        <v>0.0799861158080824</v>
+        <v>0.235600030904885</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3521,7 +3518,7 @@
       </c>
       <c r="F30" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B30)</f>
-        <v>22.9958729338843</v>
+        <v>58.41544375</v>
       </c>
       <c r="G30" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B30)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B30)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B30)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B30)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B30)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B30))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B30)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B30)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B30))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B30)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B30)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B30)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B30)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B30)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B30)),"")</f>
@@ -3547,7 +3544,7 @@
       </c>
       <c r="F31" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B31)</f>
-        <v>-26.1452763429752</v>
+        <v>-2.68787500000001</v>
       </c>
       <c r="G31" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B31)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B31)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B31)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B31)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B31)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B31))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B31)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B31)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B31))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B31)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B31)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B31)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B31)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B31)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B31)),"")</f>
@@ -3573,7 +3570,7 @@
       </c>
       <c r="F32" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B32)</f>
-        <v>5.64922914207006</v>
+        <v>29.5482860119048</v>
       </c>
       <c r="G32" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B32))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B32))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B32)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B32)),"")</f>
@@ -3599,7 +3596,7 @@
       </c>
       <c r="F33" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B33)</f>
-        <v>58.4114591942149</v>
+        <v>109.394384375</v>
       </c>
       <c r="G33" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B33))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B33))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B33)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B33)),"")</f>
@@ -3625,7 +3622,7 @@
       </c>
       <c r="F34" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B34)</f>
-        <v>35.7265909090909</v>
+        <v>60.772115625</v>
       </c>
       <c r="G34" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B34))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B34))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B34)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B34)),"")</f>
@@ -3651,7 +3648,7 @@
       </c>
       <c r="F35" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B35)</f>
-        <v>14.9950180785124</v>
+        <v>47.572321875</v>
       </c>
       <c r="G35" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B35))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B35))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B35)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B35)),"")</f>
@@ -3677,7 +3674,7 @@
       </c>
       <c r="F36" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B36)</f>
-        <v>-71.3545851575824</v>
+        <v>-56.655200124008</v>
       </c>
       <c r="G36" s="34" t="str">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B36))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B36))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B36)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B36)),"")</f>
@@ -3703,7 +3700,7 @@
       </c>
       <c r="F37" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B37)</f>
-        <v>36.7725025826446</v>
+        <v>85.81071875</v>
       </c>
       <c r="G37" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B37))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B37))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B37)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B37)),"")</f>
@@ -3729,7 +3726,7 @@
       </c>
       <c r="F38" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B38)</f>
-        <v>-9.28123708677689</v>
+        <v>19.1361625</v>
       </c>
       <c r="G38" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B38))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B38))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B38)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B38)),"")</f>
@@ -3755,7 +3752,7 @@
       </c>
       <c r="F39" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B39)</f>
-        <v>27.503331242621</v>
+        <v>64.8592464285714</v>
       </c>
       <c r="G39" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B39))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B39))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B39)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B39)),"")</f>
@@ -3781,7 +3778,7 @@
       </c>
       <c r="F40" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B40)</f>
-        <v>-6.21946803669812</v>
+        <v>14.1641483630953</v>
       </c>
       <c r="G40" s="34" t="n">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B40))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B40))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B40)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B40)),"")</f>
@@ -3807,7 +3804,7 @@
       </c>
       <c r="F41" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B41)</f>
-        <v>101.339236521055</v>
+        <v>167.180376190476</v>
       </c>
       <c r="G41" s="34" t="str">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B41))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B41))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B41)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B41)),"")</f>
@@ -3833,7 +3830,7 @@
       </c>
       <c r="F42" s="33" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,$B42)</f>
-        <v>32.8470878000787</v>
+        <v>60.0451762380952</v>
       </c>
       <c r="G42" s="34" t="str">
         <f aca="false">IF((SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B42))&gt;0,(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B42))/(SUMIFS(Diario!$E$6:$E$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$F$6:$F$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$G$6:$G$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$H$6:$H$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$I$6:$I$370,Diario!$A$6:$A$370,$B42)+SUMIFS(Diario!$J$6:$J$370,Diario!$A$6:$A$370,$B42)),"")</f>
@@ -3932,7 +3929,7 @@
       </c>
       <c r="J47" s="37" t="n">
         <f aca="false">SUMIFS(Diario!$Y$6:$Y$370,Diario!$A$6:$A$370,"&gt;="&amp;$B47,Diario!$A$6:$A$370,"&lt;="&amp;EOMONTH($B47,0))</f>
-        <v>223.239761780139</v>
+        <v>657.555304983135</v>
       </c>
       <c r="K47" s="37" t="n">
         <f aca="false">-SUMIFS(Gastos!$D$5:$D$304,Gastos!$A$5:$A$304,"&gt;="&amp;$B47,Gastos!$A$5:$A$304,"&lt;="&amp;EOMONTH($B47,0))</f>
@@ -3940,11 +3937,11 @@
       </c>
       <c r="L47" s="38" t="n">
         <f aca="false">J47+K47</f>
-        <v>223.239761780139</v>
+        <v>657.555304983135</v>
       </c>
       <c r="M47" s="34" t="n">
         <f aca="false">IF(OBJETIVO_MES&gt;0,L47/OBJETIVO_MES,"")</f>
-        <v>0.0223239761780139</v>
+        <v>0.0657555304983135</v>
       </c>
       <c r="O47" s="39" t="n">
         <f aca="false">OBJETIVO_MES</f>
@@ -4579,7 +4576,7 @@
       </c>
       <c r="J59" s="42" t="n">
         <f aca="false">SUM(J47:J58)</f>
-        <v>223.239761780139</v>
+        <v>657.555304983135</v>
       </c>
       <c r="K59" s="42" t="n">
         <f aca="false">SUM(K47:K58)</f>
@@ -4587,7 +4584,7 @@
       </c>
       <c r="L59" s="42" t="n">
         <f aca="false">SUM(L47:L58)</f>
-        <v>223.239761780139</v>
+        <v>657.555304983135</v>
       </c>
       <c r="M59" s="45"/>
     </row>
@@ -4858,11 +4855,11 @@
       </c>
       <c r="X4" s="48" t="n">
         <f aca="false">SUM(X6:X370)</f>
-        <v>-273.960661157025</v>
+        <v>-51.3419000000001</v>
       </c>
       <c r="Y4" s="48" t="n">
         <f aca="false">SUM(Y6:Y370)</f>
-        <v>223.239761780139</v>
+        <v>657.555304983135</v>
       </c>
       <c r="AA4" s="47" t="n">
         <f aca="false">SUM(AA6:AA370)</f>
@@ -4910,7 +4907,7 @@
       </c>
       <c r="AL4" s="48" t="n">
         <f aca="false">SUM(AL6:AL370)</f>
-        <v>434.315543202996</v>
+        <v>0</v>
       </c>
       <c r="AM4" s="48" t="n">
         <f aca="false">SUM(AM6:AM370)</f>
@@ -5129,11 +5126,11 @@
       </c>
       <c r="X6" s="33" t="n">
         <f aca="false">W6-(E6*P1_IVAN+F6*P2_IVAN+G6*IF($A6&lt;P3_DESDE,P3A_IVAN,P3_IVAN))-(H6+I6+J6)*(COSTE_DEV-IVA_DEV)-AM6-AO6</f>
-        <v>11.8845454545454</v>
+        <v>38.4547</v>
       </c>
       <c r="Y6" s="33" t="n">
         <f aca="false">AH6-AI6-AJ6-AK6-AL6-AM6-AO6</f>
-        <v>22.9958729338843</v>
+        <v>58.41544375</v>
       </c>
       <c r="AA6" s="58" t="n">
         <f aca="false">MAX(0,B6-E6-H6)</f>
@@ -5181,7 +5178,7 @@
       </c>
       <c r="AL6" s="60" t="n">
         <f aca="false">AD6*P1_IVAN+AE6*P2_IVAN+AF6*IF($A6&lt;P3_DESDE,P3A_IVAN,P3_IVAN)-AG6*IVA_DEV</f>
-        <v>35.4195708161157</v>
+        <v>0</v>
       </c>
       <c r="AM6" s="60" t="n">
         <f aca="false">N6*(1+RECARGO_ADS)</f>
@@ -5276,11 +5273,11 @@
       </c>
       <c r="X7" s="33" t="n">
         <f aca="false">W7-(E7*P1_IVAN+F7*P2_IVAN+G7*IF($A7&lt;P3_DESDE,P3A_IVAN,P3_IVAN))-(H7+I7+J7)*(COSTE_DEV-IVA_DEV)-AM7-AO7</f>
-        <v>-32.7801652892562</v>
+        <v>-17.1016</v>
       </c>
       <c r="Y7" s="33" t="n">
         <f aca="false">AH7-AI7-AJ7-AK7-AL7-AM7-AO7</f>
-        <v>-26.1452763429752</v>
+        <v>-2.68787500000001</v>
       </c>
       <c r="AA7" s="58" t="n">
         <f aca="false">MAX(0,B7-E7-H7)</f>
@@ -5328,7 +5325,7 @@
       </c>
       <c r="AL7" s="60" t="n">
         <f aca="false">AD7*P1_IVAN+AE7*P2_IVAN+AF7*IF($A7&lt;P3_DESDE,P3A_IVAN,P3_IVAN)-AG7*IVA_DEV</f>
-        <v>23.4574013429752</v>
+        <v>0</v>
       </c>
       <c r="AM7" s="60" t="n">
         <f aca="false">N7*(1+RECARGO_ADS)</f>
@@ -5423,11 +5420,11 @@
       </c>
       <c r="X8" s="33" t="n">
         <f aca="false">W8-(E8*P1_IVAN+F8*P2_IVAN+G8*IF($A8&lt;P3_DESDE,P3A_IVAN,P3_IVAN))-(H8+I8+J8)*(COSTE_DEV-IVA_DEV)-AM8-AO8</f>
-        <v>-9.97016528925619</v>
+        <v>5.7084</v>
       </c>
       <c r="Y8" s="33" t="n">
         <f aca="false">AH8-AI8-AJ8-AK8-AL8-AM8-AO8</f>
-        <v>5.64922914207006</v>
+        <v>29.5482860119048</v>
       </c>
       <c r="AA8" s="58" t="n">
         <f aca="false">MAX(0,B8-E8-H8)</f>
@@ -5475,7 +5472,7 @@
       </c>
       <c r="AL8" s="60" t="n">
         <f aca="false">AD8*P1_IVAN+AE8*P2_IVAN+AF8*IF($A8&lt;P3_DESDE,P3A_IVAN,P3_IVAN)-AG8*IVA_DEV</f>
-        <v>23.8990568698347</v>
+        <v>0</v>
       </c>
       <c r="AM8" s="60" t="n">
         <f aca="false">N8*(1+RECARGO_ADS)</f>
@@ -5574,11 +5571,11 @@
       </c>
       <c r="X9" s="33" t="n">
         <f aca="false">W9-(E9*P1_IVAN+F9*P2_IVAN+G9*IF($A9&lt;P3_DESDE,P3A_IVAN,P3_IVAN))-(H9+I9+J9)*(COSTE_DEV-IVA_DEV)-AM9-AO9</f>
-        <v>46.1437190082644</v>
+        <v>84.9231</v>
       </c>
       <c r="Y9" s="33" t="n">
         <f aca="false">AH9-AI9-AJ9-AK9-AL9-AM9-AO9</f>
-        <v>58.4114591942149</v>
+        <v>109.394384375</v>
       </c>
       <c r="AA9" s="58" t="n">
         <f aca="false">MAX(0,B9-E9-H9)</f>
@@ -5626,7 +5623,7 @@
       </c>
       <c r="AL9" s="60" t="n">
         <f aca="false">AD9*P1_IVAN+AE9*P2_IVAN+AF9*IF($A9&lt;P3_DESDE,P3A_IVAN,P3_IVAN)-AG9*IVA_DEV</f>
-        <v>50.9829251807851</v>
+        <v>0</v>
       </c>
       <c r="AM9" s="60" t="n">
         <f aca="false">N9*(1+RECARGO_ADS)</f>
@@ -5719,11 +5716,11 @@
       </c>
       <c r="X10" s="33" t="n">
         <f aca="false">W10-(E10*P1_IVAN+F10*P2_IVAN+G10*IF($A10&lt;P3_DESDE,P3A_IVAN,P3_IVAN))-(H10+I10+J10)*(COSTE_DEV-IVA_DEV)-AM10-AO10</f>
-        <v>33.8738842975206</v>
+        <v>56.9747</v>
       </c>
       <c r="Y10" s="33" t="n">
         <f aca="false">AH10-AI10-AJ10-AK10-AL10-AM10-AO10</f>
-        <v>35.7265909090909</v>
+        <v>60.772115625</v>
       </c>
       <c r="AA10" s="58" t="n">
         <f aca="false">MAX(0,B10-E10-H10)</f>
@@ -5771,7 +5768,7 @@
       </c>
       <c r="AL10" s="60" t="n">
         <f aca="false">AD10*P1_IVAN+AE10*P2_IVAN+AF10*IF($A10&lt;P3_DESDE,P3A_IVAN,P3_IVAN)-AG10*IVA_DEV</f>
-        <v>25.0455247159091</v>
+        <v>0</v>
       </c>
       <c r="AM10" s="60" t="n">
         <f aca="false">N10*(1+RECARGO_ADS)</f>
@@ -5864,11 +5861,11 @@
       </c>
       <c r="X11" s="33" t="n">
         <f aca="false">W11-(E11*P1_IVAN+F11*P2_IVAN+G11*IF($A11&lt;P3_DESDE,P3A_IVAN,P3_IVAN))-(H11+I11+J11)*(COSTE_DEV-IVA_DEV)-AM11-AO11</f>
-        <v>1.40942148760329</v>
+        <v>23.1926</v>
       </c>
       <c r="Y11" s="33" t="n">
         <f aca="false">AH11-AI11-AJ11-AK11-AL11-AM11-AO11</f>
-        <v>14.9950180785124</v>
+        <v>47.572321875</v>
       </c>
       <c r="AA11" s="58" t="n">
         <f aca="false">MAX(0,B11-E11-H11)</f>
@@ -5916,7 +5913,7 @@
       </c>
       <c r="AL11" s="60" t="n">
         <f aca="false">AD11*P1_IVAN+AE11*P2_IVAN+AF11*IF($A11&lt;P3_DESDE,P3A_IVAN,P3_IVAN)-AG11*IVA_DEV</f>
-        <v>32.5773037964876</v>
+        <v>0</v>
       </c>
       <c r="AM11" s="60" t="n">
         <f aca="false">N11*(1+RECARGO_ADS)</f>
@@ -6009,7 +6006,7 @@
       </c>
       <c r="Y12" s="33" t="n">
         <f aca="false">AH12-AI12-AJ12-AK12-AL12-AM12-AO12</f>
-        <v>-71.3545851575824</v>
+        <v>-56.655200124008</v>
       </c>
       <c r="AA12" s="58" t="n">
         <f aca="false">MAX(0,B12-E12-H12)</f>
@@ -6057,7 +6054,7 @@
       </c>
       <c r="AL12" s="60" t="n">
         <f aca="false">AD12*P1_IVAN+AE12*P2_IVAN+AF12*IF($A12&lt;P3_DESDE,P3A_IVAN,P3_IVAN)-AG12*IVA_DEV</f>
-        <v>14.6993850335744</v>
+        <v>0</v>
       </c>
       <c r="AM12" s="60" t="n">
         <f aca="false">N12*(1+RECARGO_ADS)</f>
@@ -6156,11 +6153,11 @@
       </c>
       <c r="X13" s="33" t="n">
         <f aca="false">W13-(E13*P1_IVAN+F13*P2_IVAN+G13*IF($A13&lt;P3_DESDE,P3A_IVAN,P3_IVAN))-(H13+I13+J13)*(COSTE_DEV-IVA_DEV)-AM13-AO13</f>
-        <v>25.4637190082645</v>
+        <v>64.2431</v>
       </c>
       <c r="Y13" s="33" t="n">
         <f aca="false">AH13-AI13-AJ13-AK13-AL13-AM13-AO13</f>
-        <v>36.7725025826446</v>
+        <v>85.81071875</v>
       </c>
       <c r="AA13" s="58" t="n">
         <f aca="false">MAX(0,B13-E13-H13)</f>
@@ -6208,7 +6205,7 @@
       </c>
       <c r="AL13" s="60" t="n">
         <f aca="false">AD13*P1_IVAN+AE13*P2_IVAN+AF13*IF($A13&lt;P3_DESDE,P3A_IVAN,P3_IVAN)-AG13*IVA_DEV</f>
-        <v>49.0382161673554</v>
+        <v>0</v>
       </c>
       <c r="AM13" s="60" t="n">
         <f aca="false">N13*(1+RECARGO_ADS)</f>
@@ -6301,11 +6298,11 @@
       </c>
       <c r="X14" s="33" t="n">
         <f aca="false">W14-(E14*P1_IVAN+F14*P2_IVAN+G14*IF($A14&lt;P3_DESDE,P3A_IVAN,P3_IVAN))-(H14+I14+J14)*(COSTE_DEV-IVA_DEV)-AM14-AO14</f>
-        <v>-24.2401652892562</v>
+        <v>-8.5616</v>
       </c>
       <c r="Y14" s="33" t="n">
         <f aca="false">AH14-AI14-AJ14-AK14-AL14-AM14-AO14</f>
-        <v>-9.28123708677689</v>
+        <v>19.1361625</v>
       </c>
       <c r="AA14" s="58" t="n">
         <f aca="false">MAX(0,B14-E14-H14)</f>
@@ -6353,7 +6350,7 @@
       </c>
       <c r="AL14" s="60" t="n">
         <f aca="false">AD14*P1_IVAN+AE14*P2_IVAN+AF14*IF($A14&lt;P3_DESDE,P3A_IVAN,P3_IVAN)-AG14*IVA_DEV</f>
-        <v>28.4173995867769</v>
+        <v>0</v>
       </c>
       <c r="AM14" s="60" t="n">
         <f aca="false">N14*(1+RECARGO_ADS)</f>
@@ -6446,11 +6443,11 @@
       </c>
       <c r="X15" s="33" t="n">
         <f aca="false">W15-(E15*P1_IVAN+F15*P2_IVAN+G15*IF($A15&lt;P3_DESDE,P3A_IVAN,P3_IVAN))-(H15+I15+J15)*(COSTE_DEV-IVA_DEV)-AM15-AO15</f>
-        <v>-14.9650413223141</v>
+        <v>5.5005</v>
       </c>
       <c r="Y15" s="33" t="n">
         <f aca="false">AH15-AI15-AJ15-AK15-AL15-AM15-AO15</f>
-        <v>27.503331242621</v>
+        <v>64.8592464285714</v>
       </c>
       <c r="AA15" s="58" t="n">
         <f aca="false">MAX(0,B15-E15-H15)</f>
@@ -6498,7 +6495,7 @@
       </c>
       <c r="AL15" s="60" t="n">
         <f aca="false">AD15*P1_IVAN+AE15*P2_IVAN+AF15*IF($A15&lt;P3_DESDE,P3A_IVAN,P3_IVAN)-AG15*IVA_DEV</f>
-        <v>37.3559151859504</v>
+        <v>0</v>
       </c>
       <c r="AM15" s="60" t="n">
         <f aca="false">N15*(1+RECARGO_ADS)</f>
@@ -6589,11 +6586,11 @@
       </c>
       <c r="X16" s="33" t="n">
         <f aca="false">W16-(E16*P1_IVAN+F16*P2_IVAN+G16*IF($A16&lt;P3_DESDE,P3A_IVAN,P3_IVAN))-(H16+I16+J16)*(COSTE_DEV-IVA_DEV)-AM16-AO16</f>
-        <v>-43.6804132231405</v>
+        <v>-37.5758</v>
       </c>
       <c r="Y16" s="33" t="n">
         <f aca="false">AH16-AI16-AJ16-AK16-AL16-AM16-AO16</f>
-        <v>-6.21946803669812</v>
+        <v>14.1641483630953</v>
       </c>
       <c r="AA16" s="58" t="n">
         <f aca="false">MAX(0,B16-E16-H16)</f>
@@ -6641,7 +6638,7 @@
       </c>
       <c r="AL16" s="60" t="n">
         <f aca="false">AD16*P1_IVAN+AE16*P2_IVAN+AF16*IF($A16&lt;P3_DESDE,P3A_IVAN,P3_IVAN)-AG16*IVA_DEV</f>
-        <v>20.3836163997934</v>
+        <v>0</v>
       </c>
       <c r="AM16" s="60" t="n">
         <f aca="false">N16*(1+RECARGO_ADS)</f>
@@ -6732,7 +6729,7 @@
       </c>
       <c r="Y17" s="33" t="n">
         <f aca="false">AH17-AI17-AJ17-AK17-AL17-AM17-AO17</f>
-        <v>101.339236521055</v>
+        <v>167.180376190476</v>
       </c>
       <c r="AA17" s="58" t="n">
         <f aca="false">MAX(0,B17-E17-H17)</f>
@@ -6780,7 +6777,7 @@
       </c>
       <c r="AL17" s="60" t="n">
         <f aca="false">AD17*P1_IVAN+AE17*P2_IVAN+AF17*IF($A17&lt;P3_DESDE,P3A_IVAN,P3_IVAN)-AG17*IVA_DEV</f>
-        <v>65.8411396694215</v>
+        <v>0</v>
       </c>
       <c r="AM17" s="60" t="n">
         <f aca="false">N17*(1+RECARGO_ADS)</f>
@@ -6871,7 +6868,7 @@
       </c>
       <c r="Y18" s="33" t="n">
         <f aca="false">AH18-AI18-AJ18-AK18-AL18-AM18-AO18</f>
-        <v>32.8470878000787</v>
+        <v>60.0451762380952</v>
       </c>
       <c r="AA18" s="58" t="n">
         <f aca="false">MAX(0,B18-E18-H18)</f>
@@ -6919,7 +6916,7 @@
       </c>
       <c r="AL18" s="60" t="n">
         <f aca="false">AD18*P1_IVAN+AE18*P2_IVAN+AF18*IF($A18&lt;P3_DESDE,P3A_IVAN,P3_IVAN)-AG18*IVA_DEV</f>
-        <v>27.1980884380165</v>
+        <v>0</v>
       </c>
       <c r="AM18" s="60" t="n">
         <f aca="false">N18*(1+RECARGO_ADS)</f>
@@ -54093,22 +54090,22 @@
       </c>
       <c r="C14" s="32" t="n">
         <f aca="false">IF(APLICA_IVA=1,C12-C13,0)</f>
-        <v>4.78697603305785</v>
+        <v>0</v>
       </c>
       <c r="D14" s="32" t="n">
         <f aca="false">IF(APLICA_IVA=1,D12-D13,0)</f>
-        <v>6.1046132231405</v>
+        <v>0</v>
       </c>
       <c r="E14" s="32" t="n">
         <f aca="false">IF(APLICA_IVA=1,E12-E13,0)</f>
-        <v>8.27786660330579</v>
+        <v>0</v>
       </c>
       <c r="F14" s="68" t="s">
         <v>142</v>
       </c>
       <c r="G14" s="32" t="n">
         <f aca="false">IF(APLICA_IVA=1,G12-G13,0)</f>
-        <v>7.42225041322314</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -54117,22 +54114,22 @@
       </c>
       <c r="C15" s="33" t="n">
         <f aca="false">C11-C14</f>
-        <v>15.2451239669421</v>
+        <v>20.0321</v>
       </c>
       <c r="D15" s="33" t="n">
         <f aca="false">D11-D14</f>
-        <v>21.5195867768595</v>
+        <v>27.6242</v>
       </c>
       <c r="E15" s="33" t="n">
         <f aca="false">E11-E14</f>
-        <v>31.8684123966942</v>
+        <v>40.146279</v>
       </c>
       <c r="F15" s="68" t="s">
         <v>144</v>
       </c>
       <c r="G15" s="33" t="n">
         <f aca="false">G11-G14</f>
-        <v>27.7940495867769</v>
+        <v>35.2163</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -54194,59 +54191,59 @@
         <v>156</v>
       </c>
       <c r="C21" s="71" t="s">
+        <v>154</v>
+      </c>
+      <c r="F21" s="66" t="s">
         <v>157</v>
-      </c>
-      <c r="F21" s="66" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="64" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C22" s="65" t="n">
         <v>7.55</v>
       </c>
       <c r="F22" s="66" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="64" t="s">
+        <v>160</v>
+      </c>
+      <c r="C23" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="66" t="s">
         <v>161</v>
-      </c>
-      <c r="C23" s="70" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="66" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="64" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C24" s="70" t="n">
         <v>0.8</v>
       </c>
       <c r="F24" s="66" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="64" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C25" s="67" t="n">
         <v>30</v>
       </c>
       <c r="F25" s="66" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="64" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C26" s="70" t="n">
         <v>0.3</v>
@@ -54255,7 +54252,7 @@
         <v>0.05</v>
       </c>
       <c r="F26" s="66" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -54266,56 +54263,56 @@
         <v>10000</v>
       </c>
       <c r="F27" s="66" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="64" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C28" s="4" t="n">
         <v>46300</v>
       </c>
       <c r="F28" s="66" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="64" t="s">
+        <v>171</v>
+      </c>
+      <c r="C29" s="71" t="s">
         <v>172</v>
       </c>
-      <c r="C29" s="71" t="s">
+      <c r="F29" s="66" t="s">
         <v>173</v>
-      </c>
-      <c r="F29" s="66" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="64" t="s">
+        <v>174</v>
+      </c>
+      <c r="C30" s="71" t="s">
         <v>175</v>
       </c>
-      <c r="C30" s="71" t="s">
+      <c r="F30" s="66" t="s">
         <v>176</v>
-      </c>
-      <c r="F30" s="66" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="64" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C31" s="65" t="n">
         <v>0.95</v>
       </c>
       <c r="F31" s="66" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="63" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C32" s="29" t="s">
         <v>147</v>
@@ -54323,22 +54320,22 @@
       <c r="D32" s="29"/>
       <c r="E32" s="29"/>
       <c r="F32" s="29" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="64" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C33" s="31" t="n">
         <f aca="false">IF(C20="SÍ",1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F33" s="68"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="64" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C34" s="31" t="n">
         <f aca="false">IF(C21="SÍ",1,0)</f>
@@ -54348,7 +54345,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="64" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C35" s="32" t="n">
         <f aca="false">IF(AND(APLICA_IVA=1,LOG_IVA=1),C22*IVA_VENTAS/(1+IVA_VENTAS),0)</f>
@@ -54358,7 +54355,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="64" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C36" s="32" t="n">
         <f aca="false">C22-C35</f>
@@ -54368,43 +54365,43 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="64" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C37" s="31" t="n">
         <f aca="false">(SUM(Diario!$E$6:$E$370)+SUM(Diario!$F$6:$F$370)+SUM(Diario!$G$6:$G$370))+(SUM(Diario!$H$6:$H$370)+SUM(Diario!$I$6:$I$370)+SUM(Diario!$J$6:$J$370))</f>
         <v>48</v>
       </c>
       <c r="F37" s="68" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="64" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C38" s="34" t="n">
         <f aca="false">IF(C37&gt;0,(SUM(Diario!$E$6:$E$370)+SUM(Diario!$F$6:$F$370)+SUM(Diario!$G$6:$G$370))/C37,"")</f>
         <v>0.854166666666667</v>
       </c>
       <c r="F38" s="68" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="64" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C39" s="34" t="n">
         <f aca="false">IF(AND(C37-C52&gt;=C25,C55&lt;&gt;""),C55,C24)</f>
         <v>0.904761904761905</v>
       </c>
       <c r="F39" s="68" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="64" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C40" s="34" t="n">
         <f aca="false">IF(SUM(Diario!$P$6:$P$370)&gt;0,SUM(Diario!$C$6:$C$370)/SUM(Diario!$P$6:$P$370),"")</f>
@@ -54415,12 +54412,12 @@
         <v>0.0521739130434783</v>
       </c>
       <c r="F40" s="68" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="64" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C41" s="34" t="n">
         <f aca="false">IF(C40="",C26,C40)</f>
@@ -54434,19 +54431,19 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="64" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C42" s="32" t="n">
         <f aca="false">IF(SUM(Diario!$AN$6:$AN$370)&gt;0,(SUM(Diario!$L$6:$L$370)+SUM(Diario!$M$6:$M$370))/SUM(Diario!$AN$6:$AN$370),"")</f>
         <v>7.59564814814815</v>
       </c>
       <c r="F42" s="68" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="64" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C43" s="32" t="n">
         <f aca="false">(1-C41-D41)*C5+C41*D5+D41*E5</f>
@@ -54456,55 +54453,55 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="64" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C44" s="32" t="n">
         <f aca="false">(1-C41-D41)*(C5-C9-IF(C42="",C8,C42)-C14)+C41*(D5-D9-IF(C42="",D8,C42)-D14)+D41*(E5-E9-IF(C42="",E8,C42)-E14)</f>
-        <v>18.1946391245791</v>
+        <v>23.6105994518518</v>
       </c>
       <c r="F44" s="68" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="64" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C45" s="32" t="n">
         <f aca="false">TASA_BE*C44-(1-TASA_BE)*C36-COMISION</f>
-        <v>9.45028972502196</v>
+        <v>13.2265344237077</v>
       </c>
       <c r="F45" s="68" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="69" t="s">
+        <v>201</v>
+      </c>
+      <c r="C46" s="33" t="n">
+        <f aca="false">(C45-IF(APLICA_IVA=1,0,TASA_BE*((1-C41-D41)*(C12-C13)+C41*(D12-D13)+D41*(E12-E13))))/(1+RECARGO_ADS)</f>
+        <v>9.45028972502196</v>
+      </c>
+      <c r="F46" s="68" t="s">
         <v>202</v>
-      </c>
-      <c r="C46" s="33" t="n">
-        <f aca="false">C45/(1+RECARGO_ADS)</f>
-        <v>9.45028972502196</v>
-      </c>
-      <c r="F46" s="68" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="69" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C47" s="73" t="n">
         <f aca="false">IF(C46&gt;0,C43/C46,"")</f>
         <v>3.69793125459434</v>
       </c>
       <c r="F47" s="68" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="63" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C49" s="29" t="s">
         <v>147</v>
@@ -54517,40 +54514,40 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="64" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C50" s="70" t="n">
         <v>0.35</v>
       </c>
       <c r="F50" s="66" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="64" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C51" s="67" t="n">
         <v>10</v>
       </c>
       <c r="F51" s="66" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="64" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C52" s="67" t="n">
         <v>6</v>
       </c>
       <c r="F52" s="66" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="64" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C53" s="67" t="n">
         <v>3</v>
@@ -54559,31 +54556,31 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="64" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C54" s="34" t="n">
         <f aca="false">(C53+C50*C51)/(C52+C51)</f>
         <v>0.40625</v>
       </c>
       <c r="F54" s="68" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="64" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C55" s="34" t="n">
         <f aca="false">IF(C37-C52&gt;0,((SUM(Diario!$E$6:$E$370)+SUM(Diario!$F$6:$F$370)+SUM(Diario!$G$6:$G$370))-C53)/(C37-C52),"")</f>
         <v>0.904761904761905</v>
       </c>
       <c r="F55" s="68" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C56" s="31" t="n">
         <f aca="false">SUM(Diario!$Q$6:$Q$370)</f>
@@ -54593,7 +54590,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="64" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C57" s="31" t="n">
         <f aca="false">SUM(Diario!$AP$6:$AP$370)</f>
@@ -54603,14 +54600,14 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="69" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C58" s="74" t="n">
         <f aca="false">IF(C37+C56&gt;0,((SUM(Diario!$E$6:$E$370)+SUM(Diario!$F$6:$F$370)+SUM(Diario!$G$6:$G$370))+(C56-C57)*C39+C57*C54)/(C37+C56),C39)</f>
         <v>0.697243788819876</v>
       </c>
       <c r="F58" s="68" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
   </sheetData>
@@ -54644,147 +54641,147 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="75" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="76" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="76" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="76" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="76" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="75" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="76" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="76" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="76" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="75" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="76" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="76" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="76" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="75" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="76" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="76" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="76" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="75" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="76" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="76" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="76" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="75" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="76" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="76" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="76" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="76" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="75" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="76" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
   </sheetData>

</xml_diff>